<commit_message>
docs: ticket migrations and translations
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E222"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3374,9 +3374,808 @@
         <v>Tout donner</v>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>Low</v>
+      </c>
+      <c r="B176" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C176" t="str">
+        <v>Baixa</v>
+      </c>
+      <c r="D176" t="str">
+        <v>Baja</v>
+      </c>
+      <c r="E176" t="str">
+        <v>Faible</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>High</v>
+      </c>
+      <c r="B177" t="str">
+        <v>High</v>
+      </c>
+      <c r="C177" t="str">
+        <v>Alta</v>
+      </c>
+      <c r="D177" t="str">
+        <v>Alta</v>
+      </c>
+      <c r="E177" t="str">
+        <v>Élevée</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>Urgent</v>
+      </c>
+      <c r="B178" t="str">
+        <v>Urgent</v>
+      </c>
+      <c r="C178" t="str">
+        <v>Urgente</v>
+      </c>
+      <c r="D178" t="str">
+        <v>Urgente</v>
+      </c>
+      <c r="E178" t="str">
+        <v>Urgente</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>Open</v>
+      </c>
+      <c r="B179" t="str">
+        <v>Open</v>
+      </c>
+      <c r="C179" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="D179" t="str">
+        <v>Abierto</v>
+      </c>
+      <c r="E179" t="str">
+        <v>Ouvert</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>Closed</v>
+      </c>
+      <c r="B180" t="str">
+        <v>Closed</v>
+      </c>
+      <c r="C180" t="str">
+        <v>Fechado</v>
+      </c>
+      <c r="D180" t="str">
+        <v>Cerrado</v>
+      </c>
+      <c r="E180" t="str">
+        <v>Fermé</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>Tickets</v>
+      </c>
+      <c r="B181" t="str">
+        <v>Tickets</v>
+      </c>
+      <c r="C181" t="str">
+        <v>Tickets</v>
+      </c>
+      <c r="D181" t="str">
+        <v>Tickets</v>
+      </c>
+      <c r="E181" t="str">
+        <v>Tickets</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>Done</v>
+      </c>
+      <c r="B182" t="str">
+        <v>Done</v>
+      </c>
+      <c r="C182" t="str">
+        <v>Concluído</v>
+      </c>
+      <c r="D182" t="str">
+        <v>Hecho</v>
+      </c>
+      <c r="E182" t="str">
+        <v>Terminé</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>Could not complete</v>
+      </c>
+      <c r="B183" t="str">
+        <v>Could not complete</v>
+      </c>
+      <c r="C183" t="str">
+        <v>Não foi possível concluir</v>
+      </c>
+      <c r="D183" t="str">
+        <v>No se pudo completar</v>
+      </c>
+      <c r="E183" t="str">
+        <v>Impossible de terminer</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>Attention</v>
+      </c>
+      <c r="B184" t="str">
+        <v>Attention</v>
+      </c>
+      <c r="C184" t="str">
+        <v>Atenção</v>
+      </c>
+      <c r="D184" t="str">
+        <v>Atención</v>
+      </c>
+      <c r="E184" t="str">
+        <v>Attention</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>Failed to load the tickets</v>
+      </c>
+      <c r="B185" t="str">
+        <v>Failed to load the tickets</v>
+      </c>
+      <c r="C185" t="str">
+        <v>Não foi possível carregar os tickets</v>
+      </c>
+      <c r="D185" t="str">
+        <v>No se pudieron cargar los tickets</v>
+      </c>
+      <c r="E185" t="str">
+        <v>Impossible de charger les tickets</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>Search by name, e-mail or subject...</v>
+      </c>
+      <c r="B186" t="str">
+        <v>Search by name, e-mail or subject...</v>
+      </c>
+      <c r="C186" t="str">
+        <v>Pesquisar por nome, e-mail ou assunto...</v>
+      </c>
+      <c r="D186" t="str">
+        <v>Buscar por nombre, correo o asunto...</v>
+      </c>
+      <c r="E186" t="str">
+        <v>Rechercher par nom, e-mail ou sujet...</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="B187" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="C187" t="str">
+        <v>Prioridade</v>
+      </c>
+      <c r="D187" t="str">
+        <v>Prioridad</v>
+      </c>
+      <c r="E187" t="str">
+        <v>Priorité</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>Assignee</v>
+      </c>
+      <c r="B188" t="str">
+        <v>Assignee</v>
+      </c>
+      <c r="C188" t="str">
+        <v>Responsável</v>
+      </c>
+      <c r="D188" t="str">
+        <v>Responsable</v>
+      </c>
+      <c r="E188" t="str">
+        <v>Responsable</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>No assignee</v>
+      </c>
+      <c r="B189" t="str">
+        <v>No assignee</v>
+      </c>
+      <c r="C189" t="str">
+        <v>Sem responsável</v>
+      </c>
+      <c r="D189" t="str">
+        <v>Sin responsable</v>
+      </c>
+      <c r="E189" t="str">
+        <v>Sans responsable</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>{{total}} tickets</v>
+      </c>
+      <c r="B190" t="str">
+        <v>{{total}} tickets</v>
+      </c>
+      <c r="C190" t="str">
+        <v>{{total}} tickets</v>
+      </c>
+      <c r="D190" t="str">
+        <v>{{total}} tickets</v>
+      </c>
+      <c r="E190" t="str">
+        <v>{{total}} tickets</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>My tickets</v>
+      </c>
+      <c r="B191" t="str">
+        <v>My tickets</v>
+      </c>
+      <c r="C191" t="str">
+        <v>Os meus tickets</v>
+      </c>
+      <c r="D191" t="str">
+        <v>Mis tickets</v>
+      </c>
+      <c r="E191" t="str">
+        <v>Mes tickets</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>Total</v>
+      </c>
+      <c r="B192" t="str">
+        <v>Total</v>
+      </c>
+      <c r="C192" t="str">
+        <v>Total</v>
+      </c>
+      <c r="D192" t="str">
+        <v>Total</v>
+      </c>
+      <c r="E192" t="str">
+        <v>Total</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>{{count}} unread</v>
+      </c>
+      <c r="B193" t="str">
+        <v>{{count}} unread</v>
+      </c>
+      <c r="C193" t="str">
+        <v>{{count}} por ler</v>
+      </c>
+      <c r="D193" t="str">
+        <v>{{count}} sin leer</v>
+      </c>
+      <c r="E193" t="str">
+        <v>{{count}} non lus</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>The last message was from the user and nobody on the team has replied yet.</v>
+      </c>
+      <c r="B194" t="str">
+        <v>The last message was from the user and nobody on the team has replied yet.</v>
+      </c>
+      <c r="C194" t="str">
+        <v>A última mensagem foi do utilizador e ainda ninguém da equipa respondeu.</v>
+      </c>
+      <c r="D194" t="str">
+        <v>El último mensaje fue del usuario y nadie del equipo ha respondido todavía.</v>
+      </c>
+      <c r="E194" t="str">
+        <v>Le dernier message était de l'utilisateur et personne dans l'équipe n'a encore répondu.</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>No reply for {{days}} days</v>
+      </c>
+      <c r="B195" t="str">
+        <v>No reply for {{days}} days</v>
+      </c>
+      <c r="C195" t="str">
+        <v>Sem resposta há {{days}} dias</v>
+      </c>
+      <c r="D195" t="str">
+        <v>Sin respuesta desde hace {{days}} días</v>
+      </c>
+      <c r="E195" t="str">
+        <v>Sans réponse depuis {{days}} jours</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>View ticket</v>
+      </c>
+      <c r="B196" t="str">
+        <v>View ticket</v>
+      </c>
+      <c r="C196" t="str">
+        <v>Ver ticket</v>
+      </c>
+      <c r="D196" t="str">
+        <v>Ver ticket</v>
+      </c>
+      <c r="E196" t="str">
+        <v>Voir le ticket</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>Failed to load your tickets</v>
+      </c>
+      <c r="B197" t="str">
+        <v>Failed to load your tickets</v>
+      </c>
+      <c r="C197" t="str">
+        <v>Não foi possível carregar os seus tickets</v>
+      </c>
+      <c r="D197" t="str">
+        <v>No se pudieron cargar tus tickets</v>
+      </c>
+      <c r="E197" t="str">
+        <v>Impossible de charger vos tickets</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>Ticket</v>
+      </c>
+      <c r="B198" t="str">
+        <v>Ticket</v>
+      </c>
+      <c r="C198" t="str">
+        <v>Ticket</v>
+      </c>
+      <c r="D198" t="str">
+        <v>Ticket</v>
+      </c>
+      <c r="E198" t="str">
+        <v>Ticket</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>New ticket</v>
+      </c>
+      <c r="B199" t="str">
+        <v>New ticket</v>
+      </c>
+      <c r="C199" t="str">
+        <v>Novo ticket</v>
+      </c>
+      <c r="D199" t="str">
+        <v>Nuevo ticket</v>
+      </c>
+      <c r="E199" t="str">
+        <v>Nouveau ticket</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>You don't have any tickets yet</v>
+      </c>
+      <c r="B200" t="str">
+        <v>You don't have any tickets yet</v>
+      </c>
+      <c r="C200" t="str">
+        <v>Ainda não tem nenhum ticket</v>
+      </c>
+      <c r="D200" t="str">
+        <v>Todavía no tienes ningún ticket</v>
+      </c>
+      <c r="E200" t="str">
+        <v>Vous n'avez pas encore de ticket</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>Could not open the attachment.</v>
+      </c>
+      <c r="B201" t="str">
+        <v>Could not open the attachment.</v>
+      </c>
+      <c r="C201" t="str">
+        <v>Não foi possível abrir o anexo.</v>
+      </c>
+      <c r="D201" t="str">
+        <v>No se pudo abrir el archivo adjunto.</v>
+      </c>
+      <c r="E201" t="str">
+        <v>Impossible d'ouvrir la pièce jointe.</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>Could not send the reply.</v>
+      </c>
+      <c r="B202" t="str">
+        <v>Could not send the reply.</v>
+      </c>
+      <c r="C202" t="str">
+        <v>Não foi possível enviar a resposta.</v>
+      </c>
+      <c r="D202" t="str">
+        <v>No se pudo enviar la respuesta.</v>
+      </c>
+      <c r="E202" t="str">
+        <v>Impossible d'envoyer la réponse.</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>Could not load this ticket. Please try again.</v>
+      </c>
+      <c r="B203" t="str">
+        <v>Could not load this ticket. Please try again.</v>
+      </c>
+      <c r="C203" t="str">
+        <v>Não foi possível carregar este ticket. Tente novamente.</v>
+      </c>
+      <c r="D203" t="str">
+        <v>No se pudo cargar este ticket. Inténtalo de nuevo.</v>
+      </c>
+      <c r="E203" t="str">
+        <v>Impossible de charger ce ticket. Veuillez réessayer.</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>Ticket not found</v>
+      </c>
+      <c r="B204" t="str">
+        <v>Ticket not found</v>
+      </c>
+      <c r="C204" t="str">
+        <v>Ticket não encontrado</v>
+      </c>
+      <c r="D204" t="str">
+        <v>Ticket no encontrado</v>
+      </c>
+      <c r="E204" t="str">
+        <v>Ticket introuvable</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>Could not update the priority.</v>
+      </c>
+      <c r="B205" t="str">
+        <v>Could not update the priority.</v>
+      </c>
+      <c r="C205" t="str">
+        <v>Não foi possível atualizar a prioridade.</v>
+      </c>
+      <c r="D205" t="str">
+        <v>No se pudo actualizar la prioridad.</v>
+      </c>
+      <c r="E205" t="str">
+        <v>Impossible de mettre à jour la priorité.</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>Could not update the assignee.</v>
+      </c>
+      <c r="B206" t="str">
+        <v>Could not update the assignee.</v>
+      </c>
+      <c r="C206" t="str">
+        <v>Não foi possível atualizar o responsável.</v>
+      </c>
+      <c r="D206" t="str">
+        <v>No se pudo actualizar el responsable.</v>
+      </c>
+      <c r="E206" t="str">
+        <v>Impossible de mettre à jour le responsable.</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>Close this ticket?</v>
+      </c>
+      <c r="B207" t="str">
+        <v>Close this ticket?</v>
+      </c>
+      <c r="C207" t="str">
+        <v>Fechar este ticket?</v>
+      </c>
+      <c r="D207" t="str">
+        <v>¿Cerrar este ticket?</v>
+      </c>
+      <c r="E207" t="str">
+        <v>Fermer ce ticket ?</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>Yes, close</v>
+      </c>
+      <c r="B208" t="str">
+        <v>Yes, close</v>
+      </c>
+      <c r="C208" t="str">
+        <v>Sim, fechar</v>
+      </c>
+      <c r="D208" t="str">
+        <v>Sí, cerrar</v>
+      </c>
+      <c r="E208" t="str">
+        <v>Oui, fermer</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>Could not update the status.</v>
+      </c>
+      <c r="B209" t="str">
+        <v>Could not update the status.</v>
+      </c>
+      <c r="C209" t="str">
+        <v>Não foi possível atualizar o estado.</v>
+      </c>
+      <c r="D209" t="str">
+        <v>No se pudo actualizar el estado.</v>
+      </c>
+      <c r="E209" t="str">
+        <v>Impossible de mettre à jour l'état.</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>Close ticket</v>
+      </c>
+      <c r="B210" t="str">
+        <v>Close ticket</v>
+      </c>
+      <c r="C210" t="str">
+        <v>Fechar ticket</v>
+      </c>
+      <c r="D210" t="str">
+        <v>Cerrar ticket</v>
+      </c>
+      <c r="E210" t="str">
+        <v>Fermer le ticket</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>Reopen ticket</v>
+      </c>
+      <c r="B211" t="str">
+        <v>Reopen ticket</v>
+      </c>
+      <c r="C211" t="str">
+        <v>Reabrir ticket</v>
+      </c>
+      <c r="D211" t="str">
+        <v>Reabrir ticket</v>
+      </c>
+      <c r="E211" t="str">
+        <v>Rouvrir le ticket</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>Write a reply...</v>
+      </c>
+      <c r="B212" t="str">
+        <v>Write a reply...</v>
+      </c>
+      <c r="C212" t="str">
+        <v>Escreva uma resposta...</v>
+      </c>
+      <c r="D212" t="str">
+        <v>Escribe una respuesta...</v>
+      </c>
+      <c r="E212" t="str">
+        <v>Écrivez une réponse...</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>"{{name}}" is too large. The maximum size is 2MB.</v>
+      </c>
+      <c r="B213" t="str">
+        <v>"{{name}}" is too large. The maximum size is 2MB.</v>
+      </c>
+      <c r="C213" t="str">
+        <v>"{{name}}" é demasiado grande. O tamanho máximo permitido é 2MB.</v>
+      </c>
+      <c r="D213" t="str">
+        <v>"{{name}}" es demasiado grande. El tamaño máximo permitido es 2 MB.</v>
+      </c>
+      <c r="E213" t="str">
+        <v>"{{name}}" est trop volumineux. La taille maximale autorisée est de 2 Mo.</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>Accepted formats: PDF, PNG, JPG, GIF and WEBP (max. 2MB per file)</v>
+      </c>
+      <c r="B214" t="str">
+        <v>Accepted formats: PDF, PNG, JPG, GIF and WEBP (max. 2MB per file)</v>
+      </c>
+      <c r="C214" t="str">
+        <v>Formatos aceites: PDF, PNG, JPG, GIF e WEBP (máx. 2MB por ficheiro)</v>
+      </c>
+      <c r="D214" t="str">
+        <v>Formatos admitidos: PDF, PNG, JPG, GIF y WEBP (máx. 2 MB por archivo)</v>
+      </c>
+      <c r="E214" t="str">
+        <v>Formats acceptés : PDF, PNG, JPG, GIF et WEBP (max. 2 Mo par fichier)</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>Attach</v>
+      </c>
+      <c r="B215" t="str">
+        <v>Attach</v>
+      </c>
+      <c r="C215" t="str">
+        <v>Anexar</v>
+      </c>
+      <c r="D215" t="str">
+        <v>Adjuntar</v>
+      </c>
+      <c r="E215" t="str">
+        <v>Joindre</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>Ticket created successfully.</v>
+      </c>
+      <c r="B216" t="str">
+        <v>Ticket created successfully.</v>
+      </c>
+      <c r="C216" t="str">
+        <v>Ticket criado com sucesso.</v>
+      </c>
+      <c r="D216" t="str">
+        <v>Ticket creado correctamente.</v>
+      </c>
+      <c r="E216" t="str">
+        <v>Ticket créé avec succès.</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>Could not create the ticket.</v>
+      </c>
+      <c r="B217" t="str">
+        <v>Could not create the ticket.</v>
+      </c>
+      <c r="C217" t="str">
+        <v>Não foi possível criar o ticket.</v>
+      </c>
+      <c r="D217" t="str">
+        <v>No se pudo crear el ticket.</v>
+      </c>
+      <c r="E217" t="str">
+        <v>Impossible de créer le ticket.</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>Describe your question...</v>
+      </c>
+      <c r="B218" t="str">
+        <v>Describe your question...</v>
+      </c>
+      <c r="C218" t="str">
+        <v>Descreva a sua questão...</v>
+      </c>
+      <c r="D218" t="str">
+        <v>Describe tu consulta...</v>
+      </c>
+      <c r="E218" t="str">
+        <v>Décrivez votre question...</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>Attach files</v>
+      </c>
+      <c r="B219" t="str">
+        <v>Attach files</v>
+      </c>
+      <c r="C219" t="str">
+        <v>Anexar ficheiros</v>
+      </c>
+      <c r="D219" t="str">
+        <v>Adjuntar archivos</v>
+      </c>
+      <c r="E219" t="str">
+        <v>Joindre des fichiers</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>New ticket activity</v>
+      </c>
+      <c r="B220" t="str">
+        <v>New ticket activity</v>
+      </c>
+      <c r="C220" t="str">
+        <v>Novidades nos tickets</v>
+      </c>
+      <c r="D220" t="str">
+        <v>Novedades en los tickets</v>
+      </c>
+      <c r="E220" t="str">
+        <v>Nouveautés dans les tickets</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>There is a new ticket or reply, go check it out!</v>
+      </c>
+      <c r="B221" t="str">
+        <v>There is a new ticket or reply, go check it out!</v>
+      </c>
+      <c r="C221" t="str">
+        <v>Há um novo ticket ou uma nova resposta, vá ver!</v>
+      </c>
+      <c r="D221" t="str">
+        <v>Hay un nuevo ticket o una nueva respuesta, ¡ve a verlo!</v>
+      </c>
+      <c r="E221" t="str">
+        <v>Il y a un nouveau ticket ou une nouvelle réponse, allez voir !</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>Your session has expired. Please log in again.</v>
+      </c>
+      <c r="B222" t="str">
+        <v>Your session has expired. Please log in again.</v>
+      </c>
+      <c r="C222" t="str">
+        <v>A sua sessão expirou. Inicie sessão novamente.</v>
+      </c>
+      <c r="D222" t="str">
+        <v>Tu sesión ha caducado. Inicia sesión de nuevo.</v>
+      </c>
+      <c r="E222" t="str">
+        <v>Votre session a expiré. Veuillez vous reconnecter.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E175"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E222"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(webapp): shared UI polish, FAQ drag and drop and course list updates
- confirmation modals, refresh/export tooltips, uniform button hover, Bial spinner and loaders
- courses: start/end date columns, single Update action, product in General; inline filters
- FAQs sortable by drag and drop; dashboard activity progress per course
- logout modal redesign; layout/profile menu; list layout uniformity
- translations (Excel)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E222"/>
+  <dimension ref="A1:E384"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4173,9 +4173,2763 @@
         <v>Votre session a expiré. Veuillez vous reconnecter.</v>
       </c>
     </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>Could not load this user</v>
+      </c>
+      <c r="B223" t="str">
+        <v>Could not load this user</v>
+      </c>
+      <c r="C223" t="str">
+        <v>Não foi possível carregar este utilizador</v>
+      </c>
+      <c r="D223" t="str">
+        <v>No se pudo cargar este usuario</v>
+      </c>
+      <c r="E223" t="str">
+        <v>Impossible de charger cet utilisateur</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>Registered on</v>
+      </c>
+      <c r="B224" t="str">
+        <v>Registered on</v>
+      </c>
+      <c r="C224" t="str">
+        <v>Registado a</v>
+      </c>
+      <c r="D224" t="str">
+        <v>Registrado el</v>
+      </c>
+      <c r="E224" t="str">
+        <v>Inscrit le</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>Progress and tests of this student in each course</v>
+      </c>
+      <c r="B225" t="str">
+        <v>Progress and tests of this student in each course</v>
+      </c>
+      <c r="C225" t="str">
+        <v>Progresso e testes deste aluno em cada curso</v>
+      </c>
+      <c r="D225" t="str">
+        <v>Progreso y tests de este alumno en cada curso</v>
+      </c>
+      <c r="E225" t="str">
+        <v>Progression et tests de cet apprenant dans chaque cours</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>Personal data and password of this student</v>
+      </c>
+      <c r="B226" t="str">
+        <v>Personal data and password of this student</v>
+      </c>
+      <c r="C226" t="str">
+        <v>Dados pessoais e palavra-passe deste aluno</v>
+      </c>
+      <c r="D226" t="str">
+        <v>Datos personales y contraseña de este alumno</v>
+      </c>
+      <c r="E226" t="str">
+        <v>Données personnelles et mot de passe de cet apprenant</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>You do not have permission to edit this account</v>
+      </c>
+      <c r="B227" t="str">
+        <v>You do not have permission to edit this account</v>
+      </c>
+      <c r="C227" t="str">
+        <v>Não tem permissão para editar esta conta</v>
+      </c>
+      <c r="D227" t="str">
+        <v>No tienes permiso para editar esta cuenta</v>
+      </c>
+      <c r="E227" t="str">
+        <v>Vous n'avez pas la permission de modifier ce compte</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>Personal data</v>
+      </c>
+      <c r="B228" t="str">
+        <v>Personal data</v>
+      </c>
+      <c r="C228" t="str">
+        <v>Dados pessoais</v>
+      </c>
+      <c r="D228" t="str">
+        <v>Datos personales</v>
+      </c>
+      <c r="E228" t="str">
+        <v>Données personnelles</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>Leave empty to keep the current password</v>
+      </c>
+      <c r="B229" t="str">
+        <v>Leave empty to keep the current password</v>
+      </c>
+      <c r="C229" t="str">
+        <v>Deixe em branco para manter a palavra-passe atual</v>
+      </c>
+      <c r="D229" t="str">
+        <v>Déjalo en blanco para mantener la contraseña actual</v>
+      </c>
+      <c r="E229" t="str">
+        <v>Laissez vide pour conserver le mot de passe actuel</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>New password</v>
+      </c>
+      <c r="B230" t="str">
+        <v>New password</v>
+      </c>
+      <c r="C230" t="str">
+        <v>Nova palavra-passe</v>
+      </c>
+      <c r="D230" t="str">
+        <v>Nueva contraseña</v>
+      </c>
+      <c r="E230" t="str">
+        <v>Nouveau mot de passe</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>Overview</v>
+      </c>
+      <c r="B231" t="str">
+        <v>Overview</v>
+      </c>
+      <c r="C231" t="str">
+        <v>Resumo</v>
+      </c>
+      <c r="D231" t="str">
+        <v>Resumen</v>
+      </c>
+      <c r="E231" t="str">
+        <v>Résumé</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>Available</v>
+      </c>
+      <c r="B232" t="str">
+        <v>Available</v>
+      </c>
+      <c r="C232" t="str">
+        <v>Disponível</v>
+      </c>
+      <c r="D232" t="str">
+        <v>Disponible</v>
+      </c>
+      <c r="E232" t="str">
+        <v>Disponible</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>Not available</v>
+      </c>
+      <c r="B233" t="str">
+        <v>Not available</v>
+      </c>
+      <c r="C233" t="str">
+        <v>Indisponível</v>
+      </c>
+      <c r="D233" t="str">
+        <v>No disponible</v>
+      </c>
+      <c r="E233" t="str">
+        <v>Indisponible</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>This course has no tests</v>
+      </c>
+      <c r="B234" t="str">
+        <v>This course has no tests</v>
+      </c>
+      <c r="C234" t="str">
+        <v>Este curso não tem testes</v>
+      </c>
+      <c r="D234" t="str">
+        <v>Este curso no tiene tests</v>
+      </c>
+      <c r="E234" t="str">
+        <v>Ce cours n'a pas de tests</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>Progress reset successfully</v>
+      </c>
+      <c r="B235" t="str">
+        <v>Progress reset successfully</v>
+      </c>
+      <c r="C235" t="str">
+        <v>Progresso reposto com sucesso</v>
+      </c>
+      <c r="D235" t="str">
+        <v>Progreso restablecido correctamente</v>
+      </c>
+      <c r="E235" t="str">
+        <v>Progression réinitialisée avec succès</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>Could not reset the progress</v>
+      </c>
+      <c r="B236" t="str">
+        <v>Could not reset the progress</v>
+      </c>
+      <c r="C236" t="str">
+        <v>Não foi possível repor o progresso</v>
+      </c>
+      <c r="D236" t="str">
+        <v>No se pudo restablecer el progreso</v>
+      </c>
+      <c r="E236" t="str">
+        <v>Impossible de réinitialiser la progression</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>No modules</v>
+      </c>
+      <c r="B237" t="str">
+        <v>No modules</v>
+      </c>
+      <c r="C237" t="str">
+        <v>Sem módulos</v>
+      </c>
+      <c r="D237" t="str">
+        <v>Sin módulos</v>
+      </c>
+      <c r="E237" t="str">
+        <v>Aucun module</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>{{done}} of {{total}} items completed</v>
+      </c>
+      <c r="B238" t="str">
+        <v>{{done}} of {{total}} items completed</v>
+      </c>
+      <c r="C238" t="str">
+        <v>{{done}} de {{total}} itens concluídos</v>
+      </c>
+      <c r="D238" t="str">
+        <v>{{done}} de {{total}} elementos completados</v>
+      </c>
+      <c r="E238" t="str">
+        <v>{{done}} sur {{total}} éléments terminés</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>Reset progress</v>
+      </c>
+      <c r="B239" t="str">
+        <v>Reset progress</v>
+      </c>
+      <c r="C239" t="str">
+        <v>Repor progresso</v>
+      </c>
+      <c r="D239" t="str">
+        <v>Restablecer progreso</v>
+      </c>
+      <c r="E239" t="str">
+        <v>Réinitialiser la progression</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>This item and the following ones will be marked as not done. Continue?</v>
+      </c>
+      <c r="B240" t="str">
+        <v>This item and the following ones will be marked as not done. Continue?</v>
+      </c>
+      <c r="C240" t="str">
+        <v>Este item e os seguintes ficam por concluir. Continuar?</v>
+      </c>
+      <c r="D240" t="str">
+        <v>Este elemento y los siguientes quedarán sin completar. ¿Continuar?</v>
+      </c>
+      <c r="E240" t="str">
+        <v>Cet élément et les suivants seront marqués comme non terminés. Continuer ?</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>Reset progress from here</v>
+      </c>
+      <c r="B241" t="str">
+        <v>Reset progress from here</v>
+      </c>
+      <c r="C241" t="str">
+        <v>Repor progresso a partir daqui</v>
+      </c>
+      <c r="D241" t="str">
+        <v>Restablecer progreso desde aquí</v>
+      </c>
+      <c r="E241" t="str">
+        <v>Réinitialiser la progression à partir d'ici</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>Try deleted successfully</v>
+      </c>
+      <c r="B242" t="str">
+        <v>Try deleted successfully</v>
+      </c>
+      <c r="C242" t="str">
+        <v>Tentativa eliminada com sucesso</v>
+      </c>
+      <c r="D242" t="str">
+        <v>Intento eliminado correctamente</v>
+      </c>
+      <c r="E242" t="str">
+        <v>Tentative supprimée avec succès</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>Could not delete the try</v>
+      </c>
+      <c r="B243" t="str">
+        <v>Could not delete the try</v>
+      </c>
+      <c r="C243" t="str">
+        <v>Não foi possível eliminar a tentativa</v>
+      </c>
+      <c r="D243" t="str">
+        <v>No se pudo eliminar el intento</v>
+      </c>
+      <c r="E243" t="str">
+        <v>Impossible de supprimer la tentative</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>Are you sure you want to delete this try?</v>
+      </c>
+      <c r="B244" t="str">
+        <v>Are you sure you want to delete this try?</v>
+      </c>
+      <c r="C244" t="str">
+        <v>Tem a certeza de que quer eliminar esta tentativa?</v>
+      </c>
+      <c r="D244" t="str">
+        <v>¿Seguro que quieres eliminar este intento?</v>
+      </c>
+      <c r="E244" t="str">
+        <v>Voulez-vous vraiment supprimer cette tentative ?</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>Progress completed successfully</v>
+      </c>
+      <c r="B245" t="str">
+        <v>Progress completed successfully</v>
+      </c>
+      <c r="C245" t="str">
+        <v>Progresso completado com sucesso</v>
+      </c>
+      <c r="D245" t="str">
+        <v>Progreso completado correctamente</v>
+      </c>
+      <c r="E245" t="str">
+        <v>Progression complétée avec succès</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>Could not complete the progress</v>
+      </c>
+      <c r="B246" t="str">
+        <v>Could not complete the progress</v>
+      </c>
+      <c r="C246" t="str">
+        <v>Não foi possível completar o progresso</v>
+      </c>
+      <c r="D246" t="str">
+        <v>No se pudo completar el progreso</v>
+      </c>
+      <c r="E246" t="str">
+        <v>Impossible de compléter la progression</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>Complete the course</v>
+      </c>
+      <c r="B247" t="str">
+        <v>Complete the course</v>
+      </c>
+      <c r="C247" t="str">
+        <v>Completar o curso</v>
+      </c>
+      <c r="D247" t="str">
+        <v>Completar el curso</v>
+      </c>
+      <c r="E247" t="str">
+        <v>Terminer le cours</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>All the items of this course will be marked as completed for this student. Continue?</v>
+      </c>
+      <c r="B248" t="str">
+        <v>All the items of this course will be marked as completed for this student. Continue?</v>
+      </c>
+      <c r="C248" t="str">
+        <v>Todos os itens deste curso ficam concluídos para este aluno. Continuar?</v>
+      </c>
+      <c r="D248" t="str">
+        <v>Todos los elementos de este curso se marcarán como completados para este alumno. ¿Continuar?</v>
+      </c>
+      <c r="E248" t="str">
+        <v>Tous les éléments de ce cours seront marqués comme terminés pour cet apprenant. Continuer ?</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>Complete the module</v>
+      </c>
+      <c r="B249" t="str">
+        <v>Complete the module</v>
+      </c>
+      <c r="C249" t="str">
+        <v>Completar o módulo</v>
+      </c>
+      <c r="D249" t="str">
+        <v>Completar el módulo</v>
+      </c>
+      <c r="E249" t="str">
+        <v>Terminer le module</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>All the items of this module will be marked as completed. Continue?</v>
+      </c>
+      <c r="B250" t="str">
+        <v>All the items of this module will be marked as completed. Continue?</v>
+      </c>
+      <c r="C250" t="str">
+        <v>Todos os itens deste módulo ficam concluídos. Continuar?</v>
+      </c>
+      <c r="D250" t="str">
+        <v>Todos los elementos de este módulo se marcarán como completados. ¿Continuar?</v>
+      </c>
+      <c r="E250" t="str">
+        <v>Tous les éléments de ce module seront marqués comme terminés. Continuer ?</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>Mark as completed</v>
+      </c>
+      <c r="B251" t="str">
+        <v>Mark as completed</v>
+      </c>
+      <c r="C251" t="str">
+        <v>Marcar como concluído</v>
+      </c>
+      <c r="D251" t="str">
+        <v>Marcar como completado</v>
+      </c>
+      <c r="E251" t="str">
+        <v>Marquer comme terminé</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>This item will be marked as completed for this student. Continue?</v>
+      </c>
+      <c r="B252" t="str">
+        <v>This item will be marked as completed for this student. Continue?</v>
+      </c>
+      <c r="C252" t="str">
+        <v>Este item fica concluído para este aluno. Continuar?</v>
+      </c>
+      <c r="D252" t="str">
+        <v>Este elemento se marcará como completado para este alumno. ¿Continuar?</v>
+      </c>
+      <c r="E252" t="str">
+        <v>Cet élément sera marqué comme terminé pour cet apprenant. Continuer ?</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>Confirm</v>
+      </c>
+      <c r="B253" t="str">
+        <v>Confirm</v>
+      </c>
+      <c r="C253" t="str">
+        <v>Confirmar</v>
+      </c>
+      <c r="D253" t="str">
+        <v>Confirmar</v>
+      </c>
+      <c r="E253" t="str">
+        <v>Confirmer</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>There are no answers recorded for this try</v>
+      </c>
+      <c r="B254" t="str">
+        <v>There are no answers recorded for this try</v>
+      </c>
+      <c r="C254" t="str">
+        <v>Não há respostas registadas nesta tentativa</v>
+      </c>
+      <c r="D254" t="str">
+        <v>No hay respuestas registradas en este intento</v>
+      </c>
+      <c r="E254" t="str">
+        <v>Aucune réponse enregistrée pour cette tentative</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>Student's answer</v>
+      </c>
+      <c r="B255" t="str">
+        <v>Student's answer</v>
+      </c>
+      <c r="C255" t="str">
+        <v>Resposta do aluno</v>
+      </c>
+      <c r="D255" t="str">
+        <v>Respuesta del alumno</v>
+      </c>
+      <c r="E255" t="str">
+        <v>Réponse de l'apprenant</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>View details</v>
+      </c>
+      <c r="B256" t="str">
+        <v>View details</v>
+      </c>
+      <c r="C256" t="str">
+        <v>Ver detalhes</v>
+      </c>
+      <c r="D256" t="str">
+        <v>Ver detalles</v>
+      </c>
+      <c r="E256" t="str">
+        <v>Voir les détails</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>Complete</v>
+      </c>
+      <c r="B257" t="str">
+        <v>Complete</v>
+      </c>
+      <c r="C257" t="str">
+        <v>Completar</v>
+      </c>
+      <c r="D257" t="str">
+        <v>Completar</v>
+      </c>
+      <c r="E257" t="str">
+        <v>Terminer</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>IEC</v>
+      </c>
+      <c r="B258" t="str">
+        <v>IEC</v>
+      </c>
+      <c r="C258" t="str">
+        <v>IEC</v>
+      </c>
+      <c r="D258" t="str">
+        <v>IEC</v>
+      </c>
+      <c r="E258" t="str">
+        <v>IEC</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>Delete module</v>
+      </c>
+      <c r="B259" t="str">
+        <v>Delete module</v>
+      </c>
+      <c r="C259" t="str">
+        <v>Eliminar módulo</v>
+      </c>
+      <c r="D259" t="str">
+        <v>Eliminar módulo</v>
+      </c>
+      <c r="E259" t="str">
+        <v>Supprimer le module</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>Your progress and tests in each course</v>
+      </c>
+      <c r="B260" t="str">
+        <v>Your progress and tests in each course</v>
+      </c>
+      <c r="C260" t="str">
+        <v>O seu progresso e testes em cada curso</v>
+      </c>
+      <c r="D260" t="str">
+        <v>Tu progreso y tests en cada curso</v>
+      </c>
+      <c r="E260" t="str">
+        <v>Votre progression et vos tests dans chaque cours</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>Your personal data and password</v>
+      </c>
+      <c r="B261" t="str">
+        <v>Your personal data and password</v>
+      </c>
+      <c r="C261" t="str">
+        <v>Os seus dados pessoais e palavra-passe</v>
+      </c>
+      <c r="D261" t="str">
+        <v>Tus datos personales y contraseña</v>
+      </c>
+      <c r="E261" t="str">
+        <v>Vos données personnelles et mot de passe</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>Could not load the fields to match. Please try again.</v>
+      </c>
+      <c r="B262" t="str">
+        <v>Could not load the fields to match. Please try again.</v>
+      </c>
+      <c r="C262" t="str">
+        <v>Não foi possível carregar os campos a associar. Tente novamente.</v>
+      </c>
+      <c r="D262" t="str">
+        <v>No se pudieron cargar los campos a asociar. Inténtalo de nuevo.</v>
+      </c>
+      <c r="E262" t="str">
+        <v>Impossible de charger les champs à associer. Veuillez réessayer.</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>The file has no data rows. Check that the 1st row has the column names and that there is at least one row below it.</v>
+      </c>
+      <c r="B263" t="str">
+        <v>The file has no data rows. Check that the 1st row has the column names and that there is at least one row below it.</v>
+      </c>
+      <c r="C263" t="str">
+        <v>O ficheiro não tem linhas de dados. Confirme que a 1.ª linha tem os nomes das colunas e que há pelo menos uma linha por baixo.</v>
+      </c>
+      <c r="D263" t="str">
+        <v>El archivo no tiene filas de datos. Comprueba que la 1.ª fila tiene los nombres de las columnas y que hay al menos una fila debajo.</v>
+      </c>
+      <c r="E263" t="str">
+        <v>Le fichier ne contient aucune ligne de données. Vérifiez que la 1re ligne contient les noms des colonnes et qu'il y a au moins une ligne en dessous.</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>Could not load the fields to match.</v>
+      </c>
+      <c r="B264" t="str">
+        <v>Could not load the fields to match.</v>
+      </c>
+      <c r="C264" t="str">
+        <v>Não foi possível carregar os campos a associar.</v>
+      </c>
+      <c r="D264" t="str">
+        <v>No se pudieron cargar los campos a asociar.</v>
+      </c>
+      <c r="E264" t="str">
+        <v>Impossible de charger les champs à associer.</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>Try again</v>
+      </c>
+      <c r="B265" t="str">
+        <v>Try again</v>
+      </c>
+      <c r="C265" t="str">
+        <v>Tentar novamente</v>
+      </c>
+      <c r="D265" t="str">
+        <v>Intentar de nuevo</v>
+      </c>
+      <c r="E265" t="str">
+        <v>Réessayer</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>Upload an XLSX file with the data to import.</v>
+      </c>
+      <c r="B266" t="str">
+        <v>Upload an XLSX file with the data to import.</v>
+      </c>
+      <c r="C266" t="str">
+        <v>Carregue um ficheiro XLSX com os dados a importar.</v>
+      </c>
+      <c r="D266" t="str">
+        <v>Sube un archivo XLSX con los datos a importar.</v>
+      </c>
+      <c r="E266" t="str">
+        <v>Téléversez un fichier XLSX avec les données à importer.</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>Download template</v>
+      </c>
+      <c r="B267" t="str">
+        <v>Download template</v>
+      </c>
+      <c r="C267" t="str">
+        <v>Descarregar modelo</v>
+      </c>
+      <c r="D267" t="str">
+        <v>Descargar plantilla</v>
+      </c>
+      <c r="E267" t="str">
+        <v>Télécharger le modèle</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>Click or drag the file to this area to upload it</v>
+      </c>
+      <c r="B268" t="str">
+        <v>Click or drag the file to this area to upload it</v>
+      </c>
+      <c r="C268" t="str">
+        <v>Clique ou arraste o ficheiro para esta área para o carregar</v>
+      </c>
+      <c r="D268" t="str">
+        <v>Haz clic o arrastra el archivo a esta área para subirlo</v>
+      </c>
+      <c r="E268" t="str">
+        <v>Cliquez ou faites glisser le fichier dans cette zone pour le téléverser</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>Only</v>
+      </c>
+      <c r="B269" t="str">
+        <v>Only</v>
+      </c>
+      <c r="C269" t="str">
+        <v>Só</v>
+      </c>
+      <c r="D269" t="str">
+        <v>Solo</v>
+      </c>
+      <c r="E269" t="str">
+        <v>Uniquement</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>files — the 1st row must have the column names</v>
+      </c>
+      <c r="B270" t="str">
+        <v>files — the 1st row must have the column names</v>
+      </c>
+      <c r="C270" t="str">
+        <v>— a 1.ª linha tem de ter os nomes das colunas</v>
+      </c>
+      <c r="D270" t="str">
+        <v>— la 1.ª fila debe tener los nombres de las columnas</v>
+      </c>
+      <c r="E270" t="str">
+        <v>— la 1re ligne doit contenir les noms des colonnes</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>Expected columns</v>
+      </c>
+      <c r="B271" t="str">
+        <v>Expected columns</v>
+      </c>
+      <c r="C271" t="str">
+        <v>Colunas esperadas</v>
+      </c>
+      <c r="D271" t="str">
+        <v>Columnas esperadas</v>
+      </c>
+      <c r="E271" t="str">
+        <v>Colonnes attendues</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>Required: e-mail and a name (first and last name, or the full name). The other columns are optional.</v>
+      </c>
+      <c r="B272" t="str">
+        <v>Required: e-mail and a name (first and last name, or the full name). The other columns are optional.</v>
+      </c>
+      <c r="C272" t="str">
+        <v>Obrigatórios: e-mail e um nome (nome e apelido, ou o nome completo). As restantes colunas são opcionais.</v>
+      </c>
+      <c r="D272" t="str">
+        <v>Obligatorios: correo y un nombre (nombre y apellido, o el nombre completo). Las demás columnas son opcionales.</v>
+      </c>
+      <c r="E272" t="str">
+        <v>Obligatoires : e-mail et un nom (prénom et nom, ou le nom complet). Les autres colonnes sont facultatives.</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>Ignored</v>
+      </c>
+      <c r="B273" t="str">
+        <v>Ignored</v>
+      </c>
+      <c r="C273" t="str">
+        <v>Ignorada</v>
+      </c>
+      <c r="D273" t="str">
+        <v>Ignorada</v>
+      </c>
+      <c r="E273" t="str">
+        <v>Ignorée</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>Confirm which field each column of your file corresponds to</v>
+      </c>
+      <c r="B274" t="str">
+        <v>Confirm which field each column of your file corresponds to</v>
+      </c>
+      <c r="C274" t="str">
+        <v>Confirme a que campo corresponde cada coluna do seu ficheiro</v>
+      </c>
+      <c r="D274" t="str">
+        <v>Confirma a qué campo corresponde cada columna de tu archivo</v>
+      </c>
+      <c r="E274" t="str">
+        <v>Confirmez à quel champ correspond chaque colonne de votre fichier</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>{{count}} rows</v>
+      </c>
+      <c r="B275" t="str">
+        <v>{{count}} rows</v>
+      </c>
+      <c r="C275" t="str">
+        <v>{{count}} linhas</v>
+      </c>
+      <c r="D275" t="str">
+        <v>{{count}} filas</v>
+      </c>
+      <c r="E275" t="str">
+        <v>{{count}} lignes</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>{{count}} columns</v>
+      </c>
+      <c r="B276" t="str">
+        <v>{{count}} columns</v>
+      </c>
+      <c r="C276" t="str">
+        <v>{{count}} colunas</v>
+      </c>
+      <c r="D276" t="str">
+        <v>{{count}} columnas</v>
+      </c>
+      <c r="E276" t="str">
+        <v>{{count}} colonnes</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>Remove file?</v>
+      </c>
+      <c r="B277" t="str">
+        <v>Remove file?</v>
+      </c>
+      <c r="C277" t="str">
+        <v>Remover ficheiro?</v>
+      </c>
+      <c r="D277" t="str">
+        <v>¿Quitar el archivo?</v>
+      </c>
+      <c r="E277" t="str">
+        <v>Supprimer le fichier ?</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>Goes back to the upload step to choose another file.</v>
+      </c>
+      <c r="B278" t="str">
+        <v>Goes back to the upload step to choose another file.</v>
+      </c>
+      <c r="C278" t="str">
+        <v>Volta ao passo de carregar para escolher outro ficheiro.</v>
+      </c>
+      <c r="D278" t="str">
+        <v>Vuelve al paso de subida para elegir otro archivo.</v>
+      </c>
+      <c r="E278" t="str">
+        <v>Retourne à l'étape de téléversement pour choisir un autre fichier.</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>Preview (first {{shown}} of {{total}} rows)</v>
+      </c>
+      <c r="B279" t="str">
+        <v>Preview (first {{shown}} of {{total}} rows)</v>
+      </c>
+      <c r="C279" t="str">
+        <v>Pré-visualização (primeiras {{shown}} de {{total}} linhas)</v>
+      </c>
+      <c r="D279" t="str">
+        <v>Vista previa (primeras {{shown}} de {{total}} filas)</v>
+      </c>
+      <c r="E279" t="str">
+        <v>Aperçu (premières {{shown}} sur {{total}} lignes)</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>{{mapped}}/{{total}} columns matched</v>
+      </c>
+      <c r="B280" t="str">
+        <v>{{mapped}}/{{total}} columns matched</v>
+      </c>
+      <c r="C280" t="str">
+        <v>{{mapped}}/{{total}} colunas associadas</v>
+      </c>
+      <c r="D280" t="str">
+        <v>{{mapped}}/{{total}} columnas asociadas</v>
+      </c>
+      <c r="E280" t="str">
+        <v>{{mapped}}/{{total}} colonnes associées</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>File column</v>
+      </c>
+      <c r="B281" t="str">
+        <v>File column</v>
+      </c>
+      <c r="C281" t="str">
+        <v>Coluna do ficheiro</v>
+      </c>
+      <c r="D281" t="str">
+        <v>Columna del archivo</v>
+      </c>
+      <c r="E281" t="str">
+        <v>Colonne du fichier</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B282" t="str">
+        <v>Field</v>
+      </c>
+      <c r="C282" t="str">
+        <v>Campo</v>
+      </c>
+      <c r="D282" t="str">
+        <v>Campo</v>
+      </c>
+      <c r="E282" t="str">
+        <v>Champ</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>Ignore this column</v>
+      </c>
+      <c r="B283" t="str">
+        <v>Ignore this column</v>
+      </c>
+      <c r="C283" t="str">
+        <v>Ignorar esta coluna</v>
+      </c>
+      <c r="D283" t="str">
+        <v>Ignorar esta columna</v>
+      </c>
+      <c r="E283" t="str">
+        <v>Ignorer cette colonne</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>Match the required fields to continue</v>
+      </c>
+      <c r="B284" t="str">
+        <v>Match the required fields to continue</v>
+      </c>
+      <c r="C284" t="str">
+        <v>Associe os campos obrigatórios para continuar</v>
+      </c>
+      <c r="D284" t="str">
+        <v>Asocia los campos obligatorios para continuar</v>
+      </c>
+      <c r="E284" t="str">
+        <v>Associez les champs obligatoires pour continuer</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>The e-mail and the name (first and last name, or the full name) are required.</v>
+      </c>
+      <c r="B285" t="str">
+        <v>The e-mail and the name (first and last name, or the full name) are required.</v>
+      </c>
+      <c r="C285" t="str">
+        <v>O e-mail e o nome (nome e apelido, ou o nome completo) são obrigatórios.</v>
+      </c>
+      <c r="D285" t="str">
+        <v>El correo y el nombre (nombre y apellido, o el nombre completo) son obligatorios.</v>
+      </c>
+      <c r="E285" t="str">
+        <v>L'e-mail et le nom (prénom et nom, ou le nom complet) sont obligatoires.</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>Import finished: {{inserted}} new, {{skipped}} skipped.</v>
+      </c>
+      <c r="B286" t="str">
+        <v>Import finished: {{inserted}} new, {{skipped}} skipped.</v>
+      </c>
+      <c r="C286" t="str">
+        <v>Importação concluída: {{inserted}} novo(s), {{skipped}} ignorado(s).</v>
+      </c>
+      <c r="D286" t="str">
+        <v>Importación terminada: {{inserted}} nuevo(s), {{skipped}} omitido(s).</v>
+      </c>
+      <c r="E286" t="str">
+        <v>Importation terminée : {{inserted}} nouveau(x), {{skipped}} ignoré(s).</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>Could not import the data. Please try again.</v>
+      </c>
+      <c r="B287" t="str">
+        <v>Could not import the data. Please try again.</v>
+      </c>
+      <c r="C287" t="str">
+        <v>Não foi possível importar os dados. Tente novamente.</v>
+      </c>
+      <c r="D287" t="str">
+        <v>No se pudieron importar los datos. Inténtalo de nuevo.</v>
+      </c>
+      <c r="E287" t="str">
+        <v>Impossible d'importer les données. Veuillez réessayer.</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>Reason</v>
+      </c>
+      <c r="B288" t="str">
+        <v>Reason</v>
+      </c>
+      <c r="C288" t="str">
+        <v>Motivo</v>
+      </c>
+      <c r="D288" t="str">
+        <v>Motivo</v>
+      </c>
+      <c r="E288" t="str">
+        <v>Motif</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>Importing the data, please wait...</v>
+      </c>
+      <c r="B289" t="str">
+        <v>Importing the data, please wait...</v>
+      </c>
+      <c r="C289" t="str">
+        <v>A importar os dados, aguarde...</v>
+      </c>
+      <c r="D289" t="str">
+        <v>Importando los datos, espera...</v>
+      </c>
+      <c r="E289" t="str">
+        <v>Importation des données, veuillez patienter...</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>Import finished</v>
+      </c>
+      <c r="B290" t="str">
+        <v>Import finished</v>
+      </c>
+      <c r="C290" t="str">
+        <v>Importação concluída</v>
+      </c>
+      <c r="D290" t="str">
+        <v>Importación terminada</v>
+      </c>
+      <c r="E290" t="str">
+        <v>Importation terminée</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>The data was processed</v>
+      </c>
+      <c r="B291" t="str">
+        <v>The data was processed</v>
+      </c>
+      <c r="C291" t="str">
+        <v>Os dados foram processados</v>
+      </c>
+      <c r="D291" t="str">
+        <v>Los datos se han procesado</v>
+      </c>
+      <c r="E291" t="str">
+        <v>Les données ont été traitées</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>Imported</v>
+      </c>
+      <c r="B292" t="str">
+        <v>Imported</v>
+      </c>
+      <c r="C292" t="str">
+        <v>Importados</v>
+      </c>
+      <c r="D292" t="str">
+        <v>Importados</v>
+      </c>
+      <c r="E292" t="str">
+        <v>Importés</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>Skipped</v>
+      </c>
+      <c r="B293" t="str">
+        <v>Skipped</v>
+      </c>
+      <c r="C293" t="str">
+        <v>Ignorados</v>
+      </c>
+      <c r="D293" t="str">
+        <v>Omitidos</v>
+      </c>
+      <c r="E293" t="str">
+        <v>Ignorés</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>E-mails sent</v>
+      </c>
+      <c r="B294" t="str">
+        <v>E-mails sent</v>
+      </c>
+      <c r="C294" t="str">
+        <v>E-mails enviados</v>
+      </c>
+      <c r="D294" t="str">
+        <v>Correos enviados</v>
+      </c>
+      <c r="E294" t="str">
+        <v>E-mails envoyés</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>{{count}} e-mails could not be sent. Those users can use "Forgot password" to set their password.</v>
+      </c>
+      <c r="B295" t="str">
+        <v>{{count}} e-mails could not be sent. Those users can use "Forgot password" to set their password.</v>
+      </c>
+      <c r="C295" t="str">
+        <v>Não foi possível enviar {{count}} e-mail(s). Esses utilizadores podem usar "Esqueci-me da palavra-passe" para definir a sua.</v>
+      </c>
+      <c r="D295" t="str">
+        <v>No se pudieron enviar {{count}} correo(s). Esos usuarios pueden usar "Olvidé mi contraseña" para definir la suya.</v>
+      </c>
+      <c r="E295" t="str">
+        <v>Impossible d'envoyer {{count}} e-mail(s). Ces utilisateurs peuvent utiliser « Mot de passe oublié » pour définir le leur.</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>Skipped rows</v>
+      </c>
+      <c r="B296" t="str">
+        <v>Skipped rows</v>
+      </c>
+      <c r="C296" t="str">
+        <v>Linhas ignoradas</v>
+      </c>
+      <c r="D296" t="str">
+        <v>Filas omitidas</v>
+      </c>
+      <c r="E296" t="str">
+        <v>Lignes ignorées</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>Download skipped rows</v>
+      </c>
+      <c r="B297" t="str">
+        <v>Download skipped rows</v>
+      </c>
+      <c r="C297" t="str">
+        <v>Descarregar linhas ignoradas</v>
+      </c>
+      <c r="D297" t="str">
+        <v>Descargar filas omitidas</v>
+      </c>
+      <c r="E297" t="str">
+        <v>Télécharger les lignes ignorées</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>Row(s) to import</v>
+      </c>
+      <c r="B298" t="str">
+        <v>Row(s) to import</v>
+      </c>
+      <c r="C298" t="str">
+        <v>Linha(s) a importar</v>
+      </c>
+      <c r="D298" t="str">
+        <v>Fila(s) a importar</v>
+      </c>
+      <c r="E298" t="str">
+        <v>Ligne(s) à importer</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>Send an access e-mail to the new users</v>
+      </c>
+      <c r="B299" t="str">
+        <v>Send an access e-mail to the new users</v>
+      </c>
+      <c r="C299" t="str">
+        <v>Enviar um e-mail de acesso aos novos utilizadores</v>
+      </c>
+      <c r="D299" t="str">
+        <v>Enviar un correo de acceso a los nuevos usuarios</v>
+      </c>
+      <c r="E299" t="str">
+        <v>Envoyer un e-mail d'accès aux nouveaux utilisateurs</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>They receive a code to choose their password. New users are approved and active.</v>
+      </c>
+      <c r="B300" t="str">
+        <v>They receive a code to choose their password. New users are approved and active.</v>
+      </c>
+      <c r="C300" t="str">
+        <v>Recebem um código para escolher a sua palavra-passe. Os novos utilizadores ficam aprovados e ativos.</v>
+      </c>
+      <c r="D300" t="str">
+        <v>Reciben un código para elegir su contraseña. Los nuevos usuarios quedan aprobados y activos.</v>
+      </c>
+      <c r="E300" t="str">
+        <v>Ils reçoivent un code pour choisir leur mot de passe. Les nouveaux utilisateurs sont approuvés et actifs.</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>File "{{name}}" exported successfully.</v>
+      </c>
+      <c r="B301" t="str">
+        <v>File "{{name}}" exported successfully.</v>
+      </c>
+      <c r="C301" t="str">
+        <v>Ficheiro "{{name}}" exportado com sucesso.</v>
+      </c>
+      <c r="D301" t="str">
+        <v>Archivo "{{name}}" exportado correctamente.</v>
+      </c>
+      <c r="E301" t="str">
+        <v>Fichier « {{name}} » exporté avec succès.</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>Could not generate the export file. Please try again.</v>
+      </c>
+      <c r="B302" t="str">
+        <v>Could not generate the export file. Please try again.</v>
+      </c>
+      <c r="C302" t="str">
+        <v>Não foi possível gerar o ficheiro de exportação. Tente novamente.</v>
+      </c>
+      <c r="D302" t="str">
+        <v>No se pudo generar el archivo de exportación. Inténtalo de nuevo.</v>
+      </c>
+      <c r="E302" t="str">
+        <v>Impossible de générer le fichier d'exportation. Veuillez réessayer.</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>{{count}} records</v>
+      </c>
+      <c r="B303" t="str">
+        <v>{{count}} records</v>
+      </c>
+      <c r="C303" t="str">
+        <v>{{count}} registos</v>
+      </c>
+      <c r="D303" t="str">
+        <v>{{count}} registros</v>
+      </c>
+      <c r="E303" t="str">
+        <v>{{count}} enregistrements</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>Format</v>
+      </c>
+      <c r="B304" t="str">
+        <v>Format</v>
+      </c>
+      <c r="C304" t="str">
+        <v>Formato</v>
+      </c>
+      <c r="D304" t="str">
+        <v>Formato</v>
+      </c>
+      <c r="E304" t="str">
+        <v>Format</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>Columns</v>
+      </c>
+      <c r="B305" t="str">
+        <v>Columns</v>
+      </c>
+      <c r="C305" t="str">
+        <v>Colunas</v>
+      </c>
+      <c r="D305" t="str">
+        <v>Columnas</v>
+      </c>
+      <c r="E305" t="str">
+        <v>Colonnes</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>None</v>
+      </c>
+      <c r="B306" t="str">
+        <v>None</v>
+      </c>
+      <c r="C306" t="str">
+        <v>Nenhuma</v>
+      </c>
+      <c r="D306" t="str">
+        <v>Ninguna</v>
+      </c>
+      <c r="E306" t="str">
+        <v>Aucune</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>{{total}} users</v>
+      </c>
+      <c r="B307" t="str">
+        <v>{{total}} users</v>
+      </c>
+      <c r="C307" t="str">
+        <v>{{total}} utilizadores</v>
+      </c>
+      <c r="D307" t="str">
+        <v>{{total}} usuarios</v>
+      </c>
+      <c r="E307" t="str">
+        <v>{{total}} utilisateurs</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>{{total}} documents</v>
+      </c>
+      <c r="B308" t="str">
+        <v>{{total}} documents</v>
+      </c>
+      <c r="C308" t="str">
+        <v>{{total}} documentos</v>
+      </c>
+      <c r="D308" t="str">
+        <v>{{total}} documentos</v>
+      </c>
+      <c r="E308" t="str">
+        <v>{{total}} documents</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>{{total}} downloads</v>
+      </c>
+      <c r="B309" t="str">
+        <v>{{total}} downloads</v>
+      </c>
+      <c r="C309" t="str">
+        <v>{{total}} downloads</v>
+      </c>
+      <c r="D309" t="str">
+        <v>{{total}} descargas</v>
+      </c>
+      <c r="E309" t="str">
+        <v>{{total}} téléchargements</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>{{total}} FAQs</v>
+      </c>
+      <c r="B310" t="str">
+        <v>{{total}} FAQs</v>
+      </c>
+      <c r="C310" t="str">
+        <v>{{total}} FAQs</v>
+      </c>
+      <c r="D310" t="str">
+        <v>{{total}} FAQs</v>
+      </c>
+      <c r="E310" t="str">
+        <v>{{total}} FAQ</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>{{total}} products</v>
+      </c>
+      <c r="B311" t="str">
+        <v>{{total}} products</v>
+      </c>
+      <c r="C311" t="str">
+        <v>{{total}} produtos</v>
+      </c>
+      <c r="D311" t="str">
+        <v>{{total}} productos</v>
+      </c>
+      <c r="E311" t="str">
+        <v>{{total}} produits</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>{{total}} translations</v>
+      </c>
+      <c r="B312" t="str">
+        <v>{{total}} translations</v>
+      </c>
+      <c r="C312" t="str">
+        <v>{{total}} traduções</v>
+      </c>
+      <c r="D312" t="str">
+        <v>{{total}} traducciones</v>
+      </c>
+      <c r="E312" t="str">
+        <v>{{total}} traductions</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>{{total}} submissions</v>
+      </c>
+      <c r="B313" t="str">
+        <v>{{total}} submissions</v>
+      </c>
+      <c r="C313" t="str">
+        <v>{{total}} respostas</v>
+      </c>
+      <c r="D313" t="str">
+        <v>{{total}} respuestas</v>
+      </c>
+      <c r="E313" t="str">
+        <v>{{total}} réponses</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>{{total}} notifications</v>
+      </c>
+      <c r="B314" t="str">
+        <v>{{total}} notifications</v>
+      </c>
+      <c r="C314" t="str">
+        <v>{{total}} notificações</v>
+      </c>
+      <c r="D314" t="str">
+        <v>{{total}} notificaciones</v>
+      </c>
+      <c r="E314" t="str">
+        <v>{{total}} notifications</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>{{total}} templates</v>
+      </c>
+      <c r="B315" t="str">
+        <v>{{total}} templates</v>
+      </c>
+      <c r="C315" t="str">
+        <v>{{total}} templates</v>
+      </c>
+      <c r="D315" t="str">
+        <v>{{total}} plantillas</v>
+      </c>
+      <c r="E315" t="str">
+        <v>{{total}} modèles</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>This file already exists</v>
+      </c>
+      <c r="B316" t="str">
+        <v>This file already exists</v>
+      </c>
+      <c r="C316" t="str">
+        <v>Este ficheiro já existe</v>
+      </c>
+      <c r="D316" t="str">
+        <v>Este archivo ya existe</v>
+      </c>
+      <c r="E316" t="str">
+        <v>Ce fichier existe déjà</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>Replace</v>
+      </c>
+      <c r="B317" t="str">
+        <v>Replace</v>
+      </c>
+      <c r="C317" t="str">
+        <v>Substituir</v>
+      </c>
+      <c r="D317" t="str">
+        <v>Reemplazar</v>
+      </c>
+      <c r="E317" t="str">
+        <v>Remplacer</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>Uploading will replace the current file. The link and QR code will not change.</v>
+      </c>
+      <c r="B318" t="str">
+        <v>Uploading will replace the current file. The link and QR code will not change.</v>
+      </c>
+      <c r="C318" t="str">
+        <v>Ao carregar, o ficheiro atual é substituído. O link e o QR code não mudam.</v>
+      </c>
+      <c r="D318" t="str">
+        <v>Al subirlo se reemplazará el archivo actual. El enlace y el código QR no cambiarán.</v>
+      </c>
+      <c r="E318" t="str">
+        <v>Le téléversement remplacera le fichier actuel. Le lien et le code QR ne changeront pas.</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>Current file</v>
+      </c>
+      <c r="B319" t="str">
+        <v>Current file</v>
+      </c>
+      <c r="C319" t="str">
+        <v>Ficheiro atual</v>
+      </c>
+      <c r="D319" t="str">
+        <v>Archivo actual</v>
+      </c>
+      <c r="E319" t="str">
+        <v>Fichier actuel</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>New file</v>
+      </c>
+      <c r="B320" t="str">
+        <v>New file</v>
+      </c>
+      <c r="C320" t="str">
+        <v>Novo ficheiro</v>
+      </c>
+      <c r="D320" t="str">
+        <v>Nuevo archivo</v>
+      </c>
+      <c r="E320" t="str">
+        <v>Nouveau fichier</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>Failed to load IECs</v>
+      </c>
+      <c r="B321" t="str">
+        <v>Failed to load IECs</v>
+      </c>
+      <c r="C321" t="str">
+        <v>Não foi possível carregar os IECs</v>
+      </c>
+      <c r="D321" t="str">
+        <v>No se pudieron cargar los IEC</v>
+      </c>
+      <c r="E321" t="str">
+        <v>Impossible de charger les IEC</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>replaced</v>
+      </c>
+      <c r="B322" t="str">
+        <v>replaced</v>
+      </c>
+      <c r="C322" t="str">
+        <v>substituído(s)</v>
+      </c>
+      <c r="D322" t="str">
+        <v>reemplazado(s)</v>
+      </c>
+      <c r="E322" t="str">
+        <v>remplacé(s)</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>skipped</v>
+      </c>
+      <c r="B323" t="str">
+        <v>skipped</v>
+      </c>
+      <c r="C323" t="str">
+        <v>ignorado(s)</v>
+      </c>
+      <c r="D323" t="str">
+        <v>omitido(s)</v>
+      </c>
+      <c r="E323" t="str">
+        <v>ignoré(s)</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>Upload cancelled</v>
+      </c>
+      <c r="B324" t="str">
+        <v>Upload cancelled</v>
+      </c>
+      <c r="C324" t="str">
+        <v>Carregamento cancelado</v>
+      </c>
+      <c r="D324" t="str">
+        <v>Subida cancelada</v>
+      </c>
+      <c r="E324" t="str">
+        <v>Téléversement annulé</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>files uploaded successfully</v>
+      </c>
+      <c r="B325" t="str">
+        <v>files uploaded successfully</v>
+      </c>
+      <c r="C325" t="str">
+        <v>ficheiros carregados com sucesso</v>
+      </c>
+      <c r="D325" t="str">
+        <v>archivos subidos correctamente</v>
+      </c>
+      <c r="E325" t="str">
+        <v>fichiers téléversés avec succès</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>Some files could not be uploaded</v>
+      </c>
+      <c r="B326" t="str">
+        <v>Some files could not be uploaded</v>
+      </c>
+      <c r="C326" t="str">
+        <v>Alguns ficheiros não foram carregados</v>
+      </c>
+      <c r="D326" t="str">
+        <v>Algunos archivos no se pudieron subir</v>
+      </c>
+      <c r="E326" t="str">
+        <v>Certains fichiers n'ont pas pu être téléversés</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>Only PDF, MP4, PNG and JPG files are allowed</v>
+      </c>
+      <c r="B327" t="str">
+        <v>Only PDF, MP4, PNG and JPG files are allowed</v>
+      </c>
+      <c r="C327" t="str">
+        <v>Só são permitidos ficheiros PDF, MP4, PNG e JPG</v>
+      </c>
+      <c r="D327" t="str">
+        <v>Solo se permiten archivos PDF, MP4, PNG y JPG</v>
+      </c>
+      <c r="E327" t="str">
+        <v>Seuls les fichiers PDF, MP4, PNG et JPG sont autorisés</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>Link copied</v>
+      </c>
+      <c r="B328" t="str">
+        <v>Link copied</v>
+      </c>
+      <c r="C328" t="str">
+        <v>Link copiado</v>
+      </c>
+      <c r="D328" t="str">
+        <v>Enlace copiado</v>
+      </c>
+      <c r="E328" t="str">
+        <v>Lien copié</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>Download QR code</v>
+      </c>
+      <c r="B329" t="str">
+        <v>Download QR code</v>
+      </c>
+      <c r="C329" t="str">
+        <v>Descarregar QR code</v>
+      </c>
+      <c r="D329" t="str">
+        <v>Descargar código QR</v>
+      </c>
+      <c r="E329" t="str">
+        <v>Télécharger le code QR</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>Click or drag PDF, MP4, PNG or JPG files to this area to upload</v>
+      </c>
+      <c r="B330" t="str">
+        <v>Click or drag PDF, MP4, PNG or JPG files to this area to upload</v>
+      </c>
+      <c r="C330" t="str">
+        <v>Clique ou arraste ficheiros PDF, MP4, PNG ou JPG para esta área para os carregar</v>
+      </c>
+      <c r="D330" t="str">
+        <v>Haz clic o arrastra archivos PDF, MP4, PNG o JPG a esta área para subirlos</v>
+      </c>
+      <c r="E330" t="str">
+        <v>Cliquez ou faites glisser des fichiers PDF, MP4, PNG ou JPG dans cette zone pour les téléverser</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>Uploading a file with an existing name replaces it. The QR code of each IEC never changes.</v>
+      </c>
+      <c r="B331" t="str">
+        <v>Uploading a file with an existing name replaces it. The QR code of each IEC never changes.</v>
+      </c>
+      <c r="C331" t="str">
+        <v>Carregar um ficheiro com um nome já existente substitui-o. O QR code de cada IEC nunca muda.</v>
+      </c>
+      <c r="D331" t="str">
+        <v>Subir un archivo con un nombre existente lo reemplaza. El código QR de cada IEC nunca cambia.</v>
+      </c>
+      <c r="E331" t="str">
+        <v>Téléverser un fichier avec un nom existant le remplace. Le code QR de chaque IEC ne change jamais.</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>File missing</v>
+      </c>
+      <c r="B332" t="str">
+        <v>File missing</v>
+      </c>
+      <c r="C332" t="str">
+        <v>Ficheiro em falta</v>
+      </c>
+      <c r="D332" t="str">
+        <v>Archivo ausente</v>
+      </c>
+      <c r="E332" t="str">
+        <v>Fichier manquant</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>Missing name</v>
+      </c>
+      <c r="B333" t="str">
+        <v>Missing name</v>
+      </c>
+      <c r="C333" t="str">
+        <v>Falta o nome</v>
+      </c>
+      <c r="D333" t="str">
+        <v>Falta el nombre</v>
+      </c>
+      <c r="E333" t="str">
+        <v>Nom manquant</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>Invalid e-mail</v>
+      </c>
+      <c r="B334" t="str">
+        <v>Invalid e-mail</v>
+      </c>
+      <c r="C334" t="str">
+        <v>E-mail inválido</v>
+      </c>
+      <c r="D334" t="str">
+        <v>Correo no válido</v>
+      </c>
+      <c r="E334" t="str">
+        <v>E-mail invalide</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>E-mail already registered</v>
+      </c>
+      <c r="B335" t="str">
+        <v>E-mail already registered</v>
+      </c>
+      <c r="C335" t="str">
+        <v>E-mail já registado</v>
+      </c>
+      <c r="D335" t="str">
+        <v>Correo ya registrado</v>
+      </c>
+      <c r="E335" t="str">
+        <v>E-mail déjà enregistré</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>Unknown language</v>
+      </c>
+      <c r="B336" t="str">
+        <v>Unknown language</v>
+      </c>
+      <c r="C336" t="str">
+        <v>Idioma desconhecido</v>
+      </c>
+      <c r="D336" t="str">
+        <v>Idioma desconocido</v>
+      </c>
+      <c r="E336" t="str">
+        <v>Langue inconnue</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>Country not available for the language</v>
+      </c>
+      <c r="B337" t="str">
+        <v>Country not available for the language</v>
+      </c>
+      <c r="C337" t="str">
+        <v>País não disponível para o idioma</v>
+      </c>
+      <c r="D337" t="str">
+        <v>País no disponible para el idioma</v>
+      </c>
+      <c r="E337" t="str">
+        <v>Pays non disponible pour la langue</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="str">
+        <v>Invalid gender</v>
+      </c>
+      <c r="B338" t="str">
+        <v>Invalid gender</v>
+      </c>
+      <c r="C338" t="str">
+        <v>Género inválido</v>
+      </c>
+      <c r="D338" t="str">
+        <v>Género no válido</v>
+      </c>
+      <c r="E338" t="str">
+        <v>Genre invalide</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="str">
+        <v>Invalid academic background</v>
+      </c>
+      <c r="B339" t="str">
+        <v>Invalid academic background</v>
+      </c>
+      <c r="C339" t="str">
+        <v>Formação académica inválida</v>
+      </c>
+      <c r="D339" t="str">
+        <v>Formación académica no válida</v>
+      </c>
+      <c r="E339" t="str">
+        <v>Formation académique invalide</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="str">
+        <v>Invalid date</v>
+      </c>
+      <c r="B340" t="str">
+        <v>Invalid date</v>
+      </c>
+      <c r="C340" t="str">
+        <v>Data inválida</v>
+      </c>
+      <c r="D340" t="str">
+        <v>Fecha no válida</v>
+      </c>
+      <c r="E340" t="str">
+        <v>Date invalide</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="str">
+        <v>Full name</v>
+      </c>
+      <c r="B341" t="str">
+        <v>Full name</v>
+      </c>
+      <c r="C341" t="str">
+        <v>Nome completo</v>
+      </c>
+      <c r="D341" t="str">
+        <v>Nombre completo</v>
+      </c>
+      <c r="E341" t="str">
+        <v>Nom complet</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="str">
+        <v>Slug</v>
+      </c>
+      <c r="B342" t="str">
+        <v>Slug</v>
+      </c>
+      <c r="C342" t="str">
+        <v>Slug</v>
+      </c>
+      <c r="D342" t="str">
+        <v>Slug</v>
+      </c>
+      <c r="E342" t="str">
+        <v>Slug</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>Default</v>
+      </c>
+      <c r="B343" t="str">
+        <v>Default</v>
+      </c>
+      <c r="C343" t="str">
+        <v>Por omissão</v>
+      </c>
+      <c r="D343" t="str">
+        <v>Por defecto</v>
+      </c>
+      <c r="E343" t="str">
+        <v>Par défaut</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>XLSX file</v>
+      </c>
+      <c r="B344" t="str">
+        <v>XLSX file</v>
+      </c>
+      <c r="C344" t="str">
+        <v>Ficheiro XLSX</v>
+      </c>
+      <c r="D344" t="str">
+        <v>Archivo XLSX</v>
+      </c>
+      <c r="E344" t="str">
+        <v>Fichier XLSX</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>Text separated by ; for Excel or other apps</v>
+      </c>
+      <c r="B345" t="str">
+        <v>Text separated by ; for Excel or other apps</v>
+      </c>
+      <c r="C345" t="str">
+        <v>Texto separado por ; para Excel ou outras aplicações</v>
+      </c>
+      <c r="D345" t="str">
+        <v>Texto separado por ; para Excel u otras aplicaciones</v>
+      </c>
+      <c r="E345" t="str">
+        <v>Texte séparé par ; pour Excel ou d'autres applications</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>Order saved</v>
+      </c>
+      <c r="B346" t="str">
+        <v>Order saved</v>
+      </c>
+      <c r="C346" t="str">
+        <v>Ordem guardada</v>
+      </c>
+      <c r="D346" t="str">
+        <v>Orden guardado</v>
+      </c>
+      <c r="E346" t="str">
+        <v>Ordre enregistré</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>Could not save the order</v>
+      </c>
+      <c r="B347" t="str">
+        <v>Could not save the order</v>
+      </c>
+      <c r="C347" t="str">
+        <v>Não foi possível guardar a ordem</v>
+      </c>
+      <c r="D347" t="str">
+        <v>No se pudo guardar el orden</v>
+      </c>
+      <c r="E347" t="str">
+        <v>Impossible d'enregistrer l'ordre</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>My profile</v>
+      </c>
+      <c r="B348" t="str">
+        <v>My profile</v>
+      </c>
+      <c r="C348" t="str">
+        <v>O meu perfil</v>
+      </c>
+      <c r="D348" t="str">
+        <v>Mi perfil</v>
+      </c>
+      <c r="E348" t="str">
+        <v>Mon profil</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>Personal data of this student</v>
+      </c>
+      <c r="B349" t="str">
+        <v>Personal data of this student</v>
+      </c>
+      <c r="C349" t="str">
+        <v>Dados pessoais deste aluno</v>
+      </c>
+      <c r="D349" t="str">
+        <v>Datos personales de este alumno</v>
+      </c>
+      <c r="E349" t="str">
+        <v>Données personnelles de cet apprenant</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>You will need to sign in again to access your account.</v>
+      </c>
+      <c r="B350" t="str">
+        <v>You will need to sign in again to access your account.</v>
+      </c>
+      <c r="C350" t="str">
+        <v>Terá de iniciar sessão novamente para aceder à sua conta.</v>
+      </c>
+      <c r="D350" t="str">
+        <v>Tendrás que iniciar sesión de nuevo para acceder a tu cuenta.</v>
+      </c>
+      <c r="E350" t="str">
+        <v>Vous devrez vous reconnecter pour accéder à votre compte.</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>Stay signed in</v>
+      </c>
+      <c r="B351" t="str">
+        <v>Stay signed in</v>
+      </c>
+      <c r="C351" t="str">
+        <v>Manter sessão iniciada</v>
+      </c>
+      <c r="D351" t="str">
+        <v>Mantener la sesión iniciada</v>
+      </c>
+      <c r="E351" t="str">
+        <v>Rester connecté</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>Unsaved changes on the page you are on will be lost.</v>
+      </c>
+      <c r="B352" t="str">
+        <v>Unsaved changes on the page you are on will be lost.</v>
+      </c>
+      <c r="C352" t="str">
+        <v>As alterações por guardar na página em que está serão perdidas.</v>
+      </c>
+      <c r="D352" t="str">
+        <v>Los cambios sin guardar en la página actual se perderán.</v>
+      </c>
+      <c r="E352" t="str">
+        <v>Les modifications non enregistrées sur la page actuelle seront perdues.</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>Your progress in the courses is saved.</v>
+      </c>
+      <c r="B353" t="str">
+        <v>Your progress in the courses is saved.</v>
+      </c>
+      <c r="C353" t="str">
+        <v>O seu progresso nos cursos fica guardado.</v>
+      </c>
+      <c r="D353" t="str">
+        <v>Tu progreso en los cursos queda guardado.</v>
+      </c>
+      <c r="E353" t="str">
+        <v>Votre progression dans les cours est enregistrée.</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>For your security, log out if you are using a shared computer.</v>
+      </c>
+      <c r="B354" t="str">
+        <v>For your security, log out if you are using a shared computer.</v>
+      </c>
+      <c r="C354" t="str">
+        <v>Por segurança, termine sessão se estiver a usar um computador partilhado.</v>
+      </c>
+      <c r="D354" t="str">
+        <v>Por seguridad, cierra la sesión si usas un ordenador compartido.</v>
+      </c>
+      <c r="E354" t="str">
+        <v>Par sécurité, déconnectez-vous si vous utilisez un ordinateur partagé.</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>Last activity</v>
+      </c>
+      <c r="B355" t="str">
+        <v>Last activity</v>
+      </c>
+      <c r="C355" t="str">
+        <v>Última atividade</v>
+      </c>
+      <c r="D355" t="str">
+        <v>Última actividad</v>
+      </c>
+      <c r="E355" t="str">
+        <v>Dernière activité</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>Days in the course</v>
+      </c>
+      <c r="B356" t="str">
+        <v>Days in the course</v>
+      </c>
+      <c r="C356" t="str">
+        <v>Dias no curso</v>
+      </c>
+      <c r="D356" t="str">
+        <v>Días en el curso</v>
+      </c>
+      <c r="E356" t="str">
+        <v>Jours dans le cours</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="str">
+        <v>Progress (%)</v>
+      </c>
+      <c r="B357" t="str">
+        <v>Progress (%)</v>
+      </c>
+      <c r="C357" t="str">
+        <v>Progresso (%)</v>
+      </c>
+      <c r="D357" t="str">
+        <v>Progreso (%)</v>
+      </c>
+      <c r="E357" t="str">
+        <v>Progression (%)</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>Total test tries</v>
+      </c>
+      <c r="B358" t="str">
+        <v>Total test tries</v>
+      </c>
+      <c r="C358" t="str">
+        <v>Total de tentativas de testes</v>
+      </c>
+      <c r="D358" t="str">
+        <v>Total de intentos de tests</v>
+      </c>
+      <c r="E358" t="str">
+        <v>Total des tentatives de tests</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v>Passed tries</v>
+      </c>
+      <c r="B359" t="str">
+        <v>Passed tries</v>
+      </c>
+      <c r="C359" t="str">
+        <v>Tentativas aprovadas</v>
+      </c>
+      <c r="D359" t="str">
+        <v>Intentos aprobados</v>
+      </c>
+      <c r="E359" t="str">
+        <v>Tentatives réussies</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v>Failed tries</v>
+      </c>
+      <c r="B360" t="str">
+        <v>Failed tries</v>
+      </c>
+      <c r="C360" t="str">
+        <v>Tentativas reprovadas</v>
+      </c>
+      <c r="D360" t="str">
+        <v>Intentos suspendidos</v>
+      </c>
+      <c r="E360" t="str">
+        <v>Tentatives échouées</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v>Test status</v>
+      </c>
+      <c r="B361" t="str">
+        <v>Test status</v>
+      </c>
+      <c r="C361" t="str">
+        <v>Estado do teste</v>
+      </c>
+      <c r="D361" t="str">
+        <v>Estado del test</v>
+      </c>
+      <c r="E361" t="str">
+        <v>État du test</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v>Best score (%)</v>
+      </c>
+      <c r="B362" t="str">
+        <v>Best score (%)</v>
+      </c>
+      <c r="C362" t="str">
+        <v>Melhor resultado (%)</v>
+      </c>
+      <c r="D362" t="str">
+        <v>Mejor resultado (%)</v>
+      </c>
+      <c r="E362" t="str">
+        <v>Meilleur résultat (%)</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v>Last score (%)</v>
+      </c>
+      <c r="B363" t="str">
+        <v>Last score (%)</v>
+      </c>
+      <c r="C363" t="str">
+        <v>Último resultado (%)</v>
+      </c>
+      <c r="D363" t="str">
+        <v>Último resultado (%)</v>
+      </c>
+      <c r="E363" t="str">
+        <v>Dernier résultat (%)</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v>Correct answers (last try)</v>
+      </c>
+      <c r="B364" t="str">
+        <v>Correct answers (last try)</v>
+      </c>
+      <c r="C364" t="str">
+        <v>Respostas certas (última tentativa)</v>
+      </c>
+      <c r="D364" t="str">
+        <v>Respuestas correctas (último intento)</v>
+      </c>
+      <c r="E364" t="str">
+        <v>Bonnes réponses (dernière tentative)</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v>Time (last try)</v>
+      </c>
+      <c r="B365" t="str">
+        <v>Time (last try)</v>
+      </c>
+      <c r="C365" t="str">
+        <v>Tempo (última tentativa)</v>
+      </c>
+      <c r="D365" t="str">
+        <v>Tiempo (último intento)</v>
+      </c>
+      <c r="E365" t="str">
+        <v>Temps (dernière tentative)</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>Date of last try</v>
+      </c>
+      <c r="B366" t="str">
+        <v>Date of last try</v>
+      </c>
+      <c r="C366" t="str">
+        <v>Data da última tentativa</v>
+      </c>
+      <c r="D366" t="str">
+        <v>Fecha del último intento</v>
+      </c>
+      <c r="E366" t="str">
+        <v>Date de la dernière tentative</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>Date passed</v>
+      </c>
+      <c r="B367" t="str">
+        <v>Date passed</v>
+      </c>
+      <c r="C367" t="str">
+        <v>Data de aprovação</v>
+      </c>
+      <c r="D367" t="str">
+        <v>Fecha de aprobación</v>
+      </c>
+      <c r="E367" t="str">
+        <v>Date de réussite</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>Export the list to Excel or CSV</v>
+      </c>
+      <c r="B368" t="str">
+        <v>Export the list to Excel or CSV</v>
+      </c>
+      <c r="C368" t="str">
+        <v>Exportar a lista para Excel ou CSV</v>
+      </c>
+      <c r="D368" t="str">
+        <v>Exportar la lista a Excel o CSV</v>
+      </c>
+      <c r="E368" t="str">
+        <v>Exporter la liste vers Excel ou CSV</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>Filter the list by more fields</v>
+      </c>
+      <c r="B369" t="str">
+        <v>Filter the list by more fields</v>
+      </c>
+      <c r="C369" t="str">
+        <v>Filtrar a lista por mais campos</v>
+      </c>
+      <c r="D369" t="str">
+        <v>Filtrar la lista por más campos</v>
+      </c>
+      <c r="E369" t="str">
+        <v>Filtrer la liste par d'autres champs</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>Show only the tickets assigned to me</v>
+      </c>
+      <c r="B370" t="str">
+        <v>Show only the tickets assigned to me</v>
+      </c>
+      <c r="C370" t="str">
+        <v>Mostrar só os tickets atribuídos a mim</v>
+      </c>
+      <c r="D370" t="str">
+        <v>Mostrar solo los tickets asignados a mí</v>
+      </c>
+      <c r="E370" t="str">
+        <v>Afficher uniquement les tickets qui me sont assignés</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>Courses with activity</v>
+      </c>
+      <c r="B371" t="str">
+        <v>Courses with activity</v>
+      </c>
+      <c r="C371" t="str">
+        <v>Cursos com atividade</v>
+      </c>
+      <c r="D371" t="str">
+        <v>Cursos con actividad</v>
+      </c>
+      <c r="E371" t="str">
+        <v>Cours avec activité</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>Courses in progress</v>
+      </c>
+      <c r="B372" t="str">
+        <v>Courses in progress</v>
+      </c>
+      <c r="C372" t="str">
+        <v>Cursos em progresso</v>
+      </c>
+      <c r="D372" t="str">
+        <v>Cursos en progreso</v>
+      </c>
+      <c r="E372" t="str">
+        <v>Cours en cours</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>Completed courses</v>
+      </c>
+      <c r="B373" t="str">
+        <v>Completed courses</v>
+      </c>
+      <c r="C373" t="str">
+        <v>Cursos concluídos</v>
+      </c>
+      <c r="D373" t="str">
+        <v>Cursos completados</v>
+      </c>
+      <c r="E373" t="str">
+        <v>Cours terminés</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>No activity yet</v>
+      </c>
+      <c r="B374" t="str">
+        <v>No activity yet</v>
+      </c>
+      <c r="C374" t="str">
+        <v>Ainda sem atividade</v>
+      </c>
+      <c r="D374" t="str">
+        <v>Todavía sin actividad</v>
+      </c>
+      <c r="E374" t="str">
+        <v>Pas encore d'activité</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>Course identification, status and product</v>
+      </c>
+      <c r="B375" t="str">
+        <v>Course identification, status and product</v>
+      </c>
+      <c r="C375" t="str">
+        <v>Identificação, estado e produto do curso</v>
+      </c>
+      <c r="D375" t="str">
+        <v>Identificación, estado y producto del curso</v>
+      </c>
+      <c r="E375" t="str">
+        <v>Identification, état et produit du cours</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>The product this course belongs to</v>
+      </c>
+      <c r="B376" t="str">
+        <v>The product this course belongs to</v>
+      </c>
+      <c r="C376" t="str">
+        <v>O produto a que este curso pertence</v>
+      </c>
+      <c r="D376" t="str">
+        <v>El producto al que pertenece este curso</v>
+      </c>
+      <c r="E376" t="str">
+        <v>Le produit auquel ce cours appartient</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>{{count}} courses</v>
+      </c>
+      <c r="B377" t="str">
+        <v>{{count}} courses</v>
+      </c>
+      <c r="C377" t="str">
+        <v>{{count}} cursos</v>
+      </c>
+      <c r="D377" t="str">
+        <v>{{count}} cursos</v>
+      </c>
+      <c r="E377" t="str">
+        <v>{{count}} cours</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>{{count}} students evaluated</v>
+      </c>
+      <c r="B378" t="str">
+        <v>{{count}} students evaluated</v>
+      </c>
+      <c r="C378" t="str">
+        <v>{{count}} alunos avaliados</v>
+      </c>
+      <c r="D378" t="str">
+        <v>{{count}} alumnos evaluados</v>
+      </c>
+      <c r="E378" t="str">
+        <v>{{count}} apprenants évalués</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>Average score</v>
+      </c>
+      <c r="B379" t="str">
+        <v>Average score</v>
+      </c>
+      <c r="C379" t="str">
+        <v>Pontuação média</v>
+      </c>
+      <c r="D379" t="str">
+        <v>Puntuación media</v>
+      </c>
+      <c r="E379" t="str">
+        <v>Score moyen</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>Approval rate</v>
+      </c>
+      <c r="B380" t="str">
+        <v>Approval rate</v>
+      </c>
+      <c r="C380" t="str">
+        <v>Taxa de aprovação</v>
+      </c>
+      <c r="D380" t="str">
+        <v>Tasa de aprobación</v>
+      </c>
+      <c r="E380" t="str">
+        <v>Taux de réussite</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>Average score by country</v>
+      </c>
+      <c r="B381" t="str">
+        <v>Average score by country</v>
+      </c>
+      <c r="C381" t="str">
+        <v>Pontuação média por país</v>
+      </c>
+      <c r="D381" t="str">
+        <v>Puntuación media por país</v>
+      </c>
+      <c r="E381" t="str">
+        <v>Score moyen par pays</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>Average score by course</v>
+      </c>
+      <c r="B382" t="str">
+        <v>Average score by course</v>
+      </c>
+      <c r="C382" t="str">
+        <v>Pontuação média por curso</v>
+      </c>
+      <c r="D382" t="str">
+        <v>Puntuación media por curso</v>
+      </c>
+      <c r="E382" t="str">
+        <v>Score moyen par cours</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v>No product</v>
+      </c>
+      <c r="B383" t="str">
+        <v>No product</v>
+      </c>
+      <c r="C383" t="str">
+        <v>Sem produto</v>
+      </c>
+      <c r="D383" t="str">
+        <v>Sin producto</v>
+      </c>
+      <c r="E383" t="str">
+        <v>Sans produit</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v>Students evaluated</v>
+      </c>
+      <c r="B384" t="str">
+        <v>Students evaluated</v>
+      </c>
+      <c r="C384" t="str">
+        <v>Alunos avaliados</v>
+      </c>
+      <c r="D384" t="str">
+        <v>Alumnos evaluados</v>
+      </c>
+      <c r="E384" t="str">
+        <v>Apprenants évalués</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E222"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E384"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: monitoring migration and new translations
Adds the monitoring migration to the staging deploy guide and the pt/es/fr translations for the monitoring page, the certificate background hints and the e-mail templates (still to import into the language table).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E384"/>
+  <dimension ref="A1:E481"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6927,9 +6927,1658 @@
         <v>Apprenants évalués</v>
       </c>
     </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v>System monitoring</v>
+      </c>
+      <c r="B385" t="str">
+        <v>System monitoring</v>
+      </c>
+      <c r="C385" t="str">
+        <v>Monitorização do sistema</v>
+      </c>
+      <c r="D385" t="str">
+        <v>Monitorización del sistema</v>
+      </c>
+      <c r="E385" t="str">
+        <v>Surveillance du système</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v>Availability, server errors and e-mails sent by the platform</v>
+      </c>
+      <c r="B386" t="str">
+        <v>Availability, server errors and e-mails sent by the platform</v>
+      </c>
+      <c r="C386" t="str">
+        <v>Disponibilidade, erros do servidor e e-mails enviados pela plataforma</v>
+      </c>
+      <c r="D386" t="str">
+        <v>Disponibilidad, errores del servidor y correos electrónicos enviados por la plataforma</v>
+      </c>
+      <c r="E386" t="str">
+        <v>Disponibilité, erreurs du serveur et e-mails envoyés par la plateforme</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v>Availability</v>
+      </c>
+      <c r="B387" t="str">
+        <v>Availability</v>
+      </c>
+      <c r="C387" t="str">
+        <v>Disponibilidade</v>
+      </c>
+      <c r="D387" t="str">
+        <v>Disponibilidad</v>
+      </c>
+      <c r="E387" t="str">
+        <v>Disponibilité</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v>Server errors</v>
+      </c>
+      <c r="B388" t="str">
+        <v>Server errors</v>
+      </c>
+      <c r="C388" t="str">
+        <v>Erros do servidor</v>
+      </c>
+      <c r="D388" t="str">
+        <v>Errores del servidor</v>
+      </c>
+      <c r="E388" t="str">
+        <v>Erreurs du serveur</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v>E-mails</v>
+      </c>
+      <c r="B389" t="str">
+        <v>E-mails</v>
+      </c>
+      <c r="C389" t="str">
+        <v>E-mails</v>
+      </c>
+      <c r="D389" t="str">
+        <v>Correos electrónicos</v>
+      </c>
+      <c r="E389" t="str">
+        <v>E-mails</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v>Could not load the system status</v>
+      </c>
+      <c r="B390" t="str">
+        <v>Could not load the system status</v>
+      </c>
+      <c r="C390" t="str">
+        <v>Não foi possível carregar o estado do sistema</v>
+      </c>
+      <c r="D390" t="str">
+        <v>No se pudo cargar el estado del sistema</v>
+      </c>
+      <c r="E390" t="str">
+        <v>Impossible de charger l'état du système</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v>Server down</v>
+      </c>
+      <c r="B391" t="str">
+        <v>Server down</v>
+      </c>
+      <c r="C391" t="str">
+        <v>Servidor em baixo</v>
+      </c>
+      <c r="D391" t="str">
+        <v>Servidor caído</v>
+      </c>
+      <c r="E391" t="str">
+        <v>Serveur hors service</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v>Database unreachable</v>
+      </c>
+      <c r="B392" t="str">
+        <v>Database unreachable</v>
+      </c>
+      <c r="C392" t="str">
+        <v>Base de dados inacessível</v>
+      </c>
+      <c r="D392" t="str">
+        <v>Base de datos inaccesible</v>
+      </c>
+      <c r="E392" t="str">
+        <v>Base de données inaccessible</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v>Last 24 hours</v>
+      </c>
+      <c r="B393" t="str">
+        <v>Last 24 hours</v>
+      </c>
+      <c r="C393" t="str">
+        <v>Últimas 24 horas</v>
+      </c>
+      <c r="D393" t="str">
+        <v>Últimas 24 horas</v>
+      </c>
+      <c r="E393" t="str">
+        <v>Dernières 24 heures</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v>Last 7 days</v>
+      </c>
+      <c r="B394" t="str">
+        <v>Last 7 days</v>
+      </c>
+      <c r="C394" t="str">
+        <v>Últimos 7 dias</v>
+      </c>
+      <c r="D394" t="str">
+        <v>Últimos 7 días</v>
+      </c>
+      <c r="E394" t="str">
+        <v>7 derniers jours</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v>Last 30 days</v>
+      </c>
+      <c r="B395" t="str">
+        <v>Last 30 days</v>
+      </c>
+      <c r="C395" t="str">
+        <v>Últimos 30 dias</v>
+      </c>
+      <c r="D395" t="str">
+        <v>Últimos 30 días</v>
+      </c>
+      <c r="E395" t="str">
+        <v>30 derniers jours</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="str">
+        <v>Status now</v>
+      </c>
+      <c r="B396" t="str">
+        <v>Status now</v>
+      </c>
+      <c r="C396" t="str">
+        <v>Estado atual</v>
+      </c>
+      <c r="D396" t="str">
+        <v>Estado actual</v>
+      </c>
+      <c r="E396" t="str">
+        <v>État actuel</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="str">
+        <v>Online</v>
+      </c>
+      <c r="B397" t="str">
+        <v>Online</v>
+      </c>
+      <c r="C397" t="str">
+        <v>Online</v>
+      </c>
+      <c r="D397" t="str">
+        <v>En línea</v>
+      </c>
+      <c r="E397" t="str">
+        <v>En ligne</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="str">
+        <v>Server time</v>
+      </c>
+      <c r="B398" t="str">
+        <v>Server time</v>
+      </c>
+      <c r="C398" t="str">
+        <v>Hora do servidor</v>
+      </c>
+      <c r="D398" t="str">
+        <v>Hora del servidor</v>
+      </c>
+      <c r="E398" t="str">
+        <v>Heure du serveur</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="str">
+        <v>Running since the last restart</v>
+      </c>
+      <c r="B399" t="str">
+        <v>Running since the last restart</v>
+      </c>
+      <c r="C399" t="str">
+        <v>Em execução desde o último reinício</v>
+      </c>
+      <c r="D399" t="str">
+        <v>En ejecución desde el último reinicio</v>
+      </c>
+      <c r="E399" t="str">
+        <v>En fonctionnement depuis le dernier redémarrage</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="str">
+        <v>Started at</v>
+      </c>
+      <c r="B400" t="str">
+        <v>Started at</v>
+      </c>
+      <c r="C400" t="str">
+        <v>Iniciado em</v>
+      </c>
+      <c r="D400" t="str">
+        <v>Iniciado el</v>
+      </c>
+      <c r="E400" t="str">
+        <v>Démarré le</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="str">
+        <v>Unresolved errors</v>
+      </c>
+      <c r="B401" t="str">
+        <v>Unresolved errors</v>
+      </c>
+      <c r="C401" t="str">
+        <v>Erros por resolver</v>
+      </c>
+      <c r="D401" t="str">
+        <v>Errores sin resolver</v>
+      </c>
+      <c r="E401" t="str">
+        <v>Erreurs non résolues</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="str">
+        <v>{{count}} in the last 24 hours</v>
+      </c>
+      <c r="B402" t="str">
+        <v>{{count}} in the last 24 hours</v>
+      </c>
+      <c r="C402" t="str">
+        <v>{{count}} nas últimas 24 horas</v>
+      </c>
+      <c r="D402" t="str">
+        <v>{{count}} en las últimas 24 horas</v>
+      </c>
+      <c r="E402" t="str">
+        <v>{{count}} au cours des dernières 24 heures</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v>E-mail failures (24 hours)</v>
+      </c>
+      <c r="B403" t="str">
+        <v>E-mail failures (24 hours)</v>
+      </c>
+      <c r="C403" t="str">
+        <v>Falhas de e-mail (24 horas)</v>
+      </c>
+      <c r="D403" t="str">
+        <v>Fallos de correo (24 horas)</v>
+      </c>
+      <c r="E403" t="str">
+        <v>Échecs d'e-mail (24 heures)</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v>Downtime</v>
+      </c>
+      <c r="B404" t="str">
+        <v>Downtime</v>
+      </c>
+      <c r="C404" t="str">
+        <v>Tempo em baixo</v>
+      </c>
+      <c r="D404" t="str">
+        <v>Tiempo de inactividad</v>
+      </c>
+      <c r="E404" t="str">
+        <v>Temps d'arrêt</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="str">
+        <v>{{count}} incidents</v>
+      </c>
+      <c r="B405" t="str">
+        <v>{{count}} incidents</v>
+      </c>
+      <c r="C405" t="str">
+        <v>{{count}} incidentes</v>
+      </c>
+      <c r="D405" t="str">
+        <v>{{count}} incidentes</v>
+      </c>
+      <c r="E405" t="str">
+        <v>{{count}} incidents</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="str">
+        <v>Downtime incidents</v>
+      </c>
+      <c r="B406" t="str">
+        <v>Downtime incidents</v>
+      </c>
+      <c r="C406" t="str">
+        <v>Incidentes de indisponibilidade</v>
+      </c>
+      <c r="D406" t="str">
+        <v>Incidentes de indisponibilidad</v>
+      </c>
+      <c r="E406" t="str">
+        <v>Incidents d'indisponibilité</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="str">
+        <v>Public address for an external uptime monitor (it answers 200 when the server and the database are working)</v>
+      </c>
+      <c r="B407" t="str">
+        <v>Public address for an external uptime monitor (it answers 200 when the server and the database are working)</v>
+      </c>
+      <c r="C407" t="str">
+        <v>Endereço público para um monitor de disponibilidade externo (responde 200 quando o servidor e a base de dados estão a funcionar)</v>
+      </c>
+      <c r="D407" t="str">
+        <v>Dirección pública para un monitor de disponibilidad externo (responde 200 cuando el servidor y la base de datos funcionan)</v>
+      </c>
+      <c r="E407" t="str">
+        <v>Adresse publique pour un moniteur de disponibilité externe (répond 200 lorsque le serveur et la base de données fonctionnent)</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="str">
+        <v>No downtime recorded</v>
+      </c>
+      <c r="B408" t="str">
+        <v>No downtime recorded</v>
+      </c>
+      <c r="C408" t="str">
+        <v>Sem indisponibilidade registada</v>
+      </c>
+      <c r="D408" t="str">
+        <v>Sin inactividad registrada</v>
+      </c>
+      <c r="E408" t="str">
+        <v>Aucune indisponibilité enregistrée</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="str">
+        <v>Started</v>
+      </c>
+      <c r="B409" t="str">
+        <v>Started</v>
+      </c>
+      <c r="C409" t="str">
+        <v>Início</v>
+      </c>
+      <c r="D409" t="str">
+        <v>Inicio</v>
+      </c>
+      <c r="E409" t="str">
+        <v>Début</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="str">
+        <v>Ended</v>
+      </c>
+      <c r="B410" t="str">
+        <v>Ended</v>
+      </c>
+      <c r="C410" t="str">
+        <v>Fim</v>
+      </c>
+      <c r="D410" t="str">
+        <v>Fin</v>
+      </c>
+      <c r="E410" t="str">
+        <v>Fin</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="str">
+        <v>Duration</v>
+      </c>
+      <c r="B411" t="str">
+        <v>Duration</v>
+      </c>
+      <c r="C411" t="str">
+        <v>Duração</v>
+      </c>
+      <c r="D411" t="str">
+        <v>Duración</v>
+      </c>
+      <c r="E411" t="str">
+        <v>Durée</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="str">
+        <v>The downtime is calculated from the server heartbeat (every 30 seconds): when the server starts again, the time since its last heartbeat is recorded. Logs are kept for {{days}} days.</v>
+      </c>
+      <c r="B412" t="str">
+        <v>The downtime is calculated from the server heartbeat (every 30 seconds): when the server starts again, the time since its last heartbeat is recorded. Logs are kept for {{days}} days.</v>
+      </c>
+      <c r="C412" t="str">
+        <v>O tempo em baixo é calculado a partir do sinal de vida do servidor (a cada 30 segundos): quando o servidor volta a arrancar, regista-se o tempo desde o último sinal. Os registos são mantidos durante {{days}} dias.</v>
+      </c>
+      <c r="D412" t="str">
+        <v>El tiempo de inactividad se calcula a partir de la señal de vida del servidor (cada 30 segundos): cuando el servidor vuelve a arrancar, se registra el tiempo desde la última señal. Los registros se conservan durante {{days}} días.</v>
+      </c>
+      <c r="E412" t="str">
+        <v>Le temps d'arrêt est calculé à partir du signal de vie du serveur (toutes les 30 secondes) : lorsque le serveur redémarre, le temps écoulé depuis le dernier signal est enregistré. Les journaux sont conservés pendant {{days}} jours.</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="str">
+        <v>Could not load the data</v>
+      </c>
+      <c r="B413" t="str">
+        <v>Could not load the data</v>
+      </c>
+      <c r="C413" t="str">
+        <v>Não foi possível carregar os dados</v>
+      </c>
+      <c r="D413" t="str">
+        <v>No se pudieron cargar los datos</v>
+      </c>
+      <c r="E413" t="str">
+        <v>Impossible de charger les données</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="str">
+        <v>Request failed</v>
+      </c>
+      <c r="B414" t="str">
+        <v>Request failed</v>
+      </c>
+      <c r="C414" t="str">
+        <v>Pedido falhado</v>
+      </c>
+      <c r="D414" t="str">
+        <v>Solicitud fallida</v>
+      </c>
+      <c r="E414" t="str">
+        <v>Requête échouée</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="str">
+        <v>Unhandled rejection</v>
+      </c>
+      <c r="B415" t="str">
+        <v>Unhandled rejection</v>
+      </c>
+      <c r="C415" t="str">
+        <v>Rejeição não tratada</v>
+      </c>
+      <c r="D415" t="str">
+        <v>Rechazo no gestionado</v>
+      </c>
+      <c r="E415" t="str">
+        <v>Rejet non géré</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="str">
+        <v>Uncaught exception</v>
+      </c>
+      <c r="B416" t="str">
+        <v>Uncaught exception</v>
+      </c>
+      <c r="C416" t="str">
+        <v>Exceção não capturada</v>
+      </c>
+      <c r="D416" t="str">
+        <v>Excepción no capturada</v>
+      </c>
+      <c r="E416" t="str">
+        <v>Exception non interceptée</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="str">
+        <v>Marked as resolved</v>
+      </c>
+      <c r="B417" t="str">
+        <v>Marked as resolved</v>
+      </c>
+      <c r="C417" t="str">
+        <v>Marcado como resolvido</v>
+      </c>
+      <c r="D417" t="str">
+        <v>Marcado como resuelto</v>
+      </c>
+      <c r="E417" t="str">
+        <v>Marqué comme résolu</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="str">
+        <v>Marked as unresolved</v>
+      </c>
+      <c r="B418" t="str">
+        <v>Marked as unresolved</v>
+      </c>
+      <c r="C418" t="str">
+        <v>Marcado como por resolver</v>
+      </c>
+      <c r="D418" t="str">
+        <v>Marcado como sin resolver</v>
+      </c>
+      <c r="E418" t="str">
+        <v>Marqué comme non résolu</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="str">
+        <v>Could not update the errors</v>
+      </c>
+      <c r="B419" t="str">
+        <v>Could not update the errors</v>
+      </c>
+      <c r="C419" t="str">
+        <v>Não foi possível atualizar os erros</v>
+      </c>
+      <c r="D419" t="str">
+        <v>No se pudieron actualizar los errores</v>
+      </c>
+      <c r="E419" t="str">
+        <v>Impossible de mettre à jour les erreurs</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="str">
+        <v>Delete the selected logs?</v>
+      </c>
+      <c r="B420" t="str">
+        <v>Delete the selected logs?</v>
+      </c>
+      <c r="C420" t="str">
+        <v>Eliminar os registos selecionados?</v>
+      </c>
+      <c r="D420" t="str">
+        <v>¿Eliminar los registros seleccionados?</v>
+      </c>
+      <c r="E420" t="str">
+        <v>Supprimer les journaux sélectionnés ?</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="str">
+        <v>{{count}} log(s) will be permanently deleted.</v>
+      </c>
+      <c r="B421" t="str">
+        <v>{{count}} log(s) will be permanently deleted.</v>
+      </c>
+      <c r="C421" t="str">
+        <v>{{count}} registo(s) será(ão) eliminado(s) permanentemente.</v>
+      </c>
+      <c r="D421" t="str">
+        <v>{{count}} registro(s) se eliminará(n) permanentemente.</v>
+      </c>
+      <c r="E421" t="str">
+        <v>{{count}} journal(aux) sera(ont) supprimé(s) définitivement.</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="str">
+        <v>Logs deleted</v>
+      </c>
+      <c r="B422" t="str">
+        <v>Logs deleted</v>
+      </c>
+      <c r="C422" t="str">
+        <v>Registos eliminados</v>
+      </c>
+      <c r="D422" t="str">
+        <v>Registros eliminados</v>
+      </c>
+      <c r="E422" t="str">
+        <v>Journaux supprimés</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="str">
+        <v>Could not delete the logs</v>
+      </c>
+      <c r="B423" t="str">
+        <v>Could not delete the logs</v>
+      </c>
+      <c r="C423" t="str">
+        <v>Não foi possível eliminar os registos</v>
+      </c>
+      <c r="D423" t="str">
+        <v>No se pudieron eliminar los registros</v>
+      </c>
+      <c r="E423" t="str">
+        <v>Impossible de supprimer les journaux</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="str">
+        <v>Search by message or route...</v>
+      </c>
+      <c r="B424" t="str">
+        <v>Search by message or route...</v>
+      </c>
+      <c r="C424" t="str">
+        <v>Pesquisar por mensagem ou rota...</v>
+      </c>
+      <c r="D424" t="str">
+        <v>Buscar por mensaje o ruta...</v>
+      </c>
+      <c r="E424" t="str">
+        <v>Rechercher par message ou route...</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="str">
+        <v>Error</v>
+      </c>
+      <c r="B425" t="str">
+        <v>Error</v>
+      </c>
+      <c r="C425" t="str">
+        <v>Erro</v>
+      </c>
+      <c r="D425" t="str">
+        <v>Error</v>
+      </c>
+      <c r="E425" t="str">
+        <v>Erreur</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="str">
+        <v>Warning</v>
+      </c>
+      <c r="B426" t="str">
+        <v>Warning</v>
+      </c>
+      <c r="C426" t="str">
+        <v>Aviso</v>
+      </c>
+      <c r="D426" t="str">
+        <v>Advertencia</v>
+      </c>
+      <c r="E426" t="str">
+        <v>Avertissement</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="str">
+        <v>Source</v>
+      </c>
+      <c r="B427" t="str">
+        <v>Source</v>
+      </c>
+      <c r="C427" t="str">
+        <v>Origem</v>
+      </c>
+      <c r="D427" t="str">
+        <v>Origen</v>
+      </c>
+      <c r="E427" t="str">
+        <v>Source</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="str">
+        <v>Unresolved</v>
+      </c>
+      <c r="B428" t="str">
+        <v>Unresolved</v>
+      </c>
+      <c r="C428" t="str">
+        <v>Por resolver</v>
+      </c>
+      <c r="D428" t="str">
+        <v>Sin resolver</v>
+      </c>
+      <c r="E428" t="str">
+        <v>Non résolu</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="str">
+        <v>Resolved</v>
+      </c>
+      <c r="B429" t="str">
+        <v>Resolved</v>
+      </c>
+      <c r="C429" t="str">
+        <v>Resolvido</v>
+      </c>
+      <c r="D429" t="str">
+        <v>Resuelto</v>
+      </c>
+      <c r="E429" t="str">
+        <v>Résolu</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="str">
+        <v>All</v>
+      </c>
+      <c r="B430" t="str">
+        <v>All</v>
+      </c>
+      <c r="C430" t="str">
+        <v>Todos</v>
+      </c>
+      <c r="D430" t="str">
+        <v>Todos</v>
+      </c>
+      <c r="E430" t="str">
+        <v>Tous</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="str">
+        <v>Mark as resolved</v>
+      </c>
+      <c r="B431" t="str">
+        <v>Mark as resolved</v>
+      </c>
+      <c r="C431" t="str">
+        <v>Marcar como resolvido</v>
+      </c>
+      <c r="D431" t="str">
+        <v>Marcar como resuelto</v>
+      </c>
+      <c r="E431" t="str">
+        <v>Marquer comme résolu</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="str">
+        <v>of</v>
+      </c>
+      <c r="B432" t="str">
+        <v>of</v>
+      </c>
+      <c r="C432" t="str">
+        <v>de</v>
+      </c>
+      <c r="D432" t="str">
+        <v>de</v>
+      </c>
+      <c r="E432" t="str">
+        <v>sur</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="str">
+        <v>Message</v>
+      </c>
+      <c r="B433" t="str">
+        <v>Message</v>
+      </c>
+      <c r="C433" t="str">
+        <v>Mensagem</v>
+      </c>
+      <c r="D433" t="str">
+        <v>Mensaje</v>
+      </c>
+      <c r="E433" t="str">
+        <v>Message</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="str">
+        <v>No errors recorded</v>
+      </c>
+      <c r="B434" t="str">
+        <v>No errors recorded</v>
+      </c>
+      <c r="C434" t="str">
+        <v>Sem erros registados</v>
+      </c>
+      <c r="D434" t="str">
+        <v>Sin errores registrados</v>
+      </c>
+      <c r="E434" t="str">
+        <v>Aucune erreur enregistrée</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="str">
+        <v>Route</v>
+      </c>
+      <c r="B435" t="str">
+        <v>Route</v>
+      </c>
+      <c r="C435" t="str">
+        <v>Rota</v>
+      </c>
+      <c r="D435" t="str">
+        <v>Ruta</v>
+      </c>
+      <c r="E435" t="str">
+        <v>Route</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="str">
+        <v>Sent</v>
+      </c>
+      <c r="B436" t="str">
+        <v>Sent</v>
+      </c>
+      <c r="C436" t="str">
+        <v>Enviado</v>
+      </c>
+      <c r="D436" t="str">
+        <v>Enviado</v>
+      </c>
+      <c r="E436" t="str">
+        <v>Envoyé</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="str">
+        <v>Search by recipient, subject or error...</v>
+      </c>
+      <c r="B437" t="str">
+        <v>Search by recipient, subject or error...</v>
+      </c>
+      <c r="C437" t="str">
+        <v>Pesquisar por destinatário, assunto ou erro...</v>
+      </c>
+      <c r="D437" t="str">
+        <v>Buscar por destinatario, asunto o error...</v>
+      </c>
+      <c r="E437" t="str">
+        <v>Rechercher par destinataire, objet ou erreur...</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="str">
+        <v>SMTP response</v>
+      </c>
+      <c r="B438" t="str">
+        <v>SMTP response</v>
+      </c>
+      <c r="C438" t="str">
+        <v>Resposta SMTP</v>
+      </c>
+      <c r="D438" t="str">
+        <v>Respuesta SMTP</v>
+      </c>
+      <c r="E438" t="str">
+        <v>Réponse SMTP</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="str">
+        <v>No e-mails recorded</v>
+      </c>
+      <c r="B439" t="str">
+        <v>No e-mails recorded</v>
+      </c>
+      <c r="C439" t="str">
+        <v>Sem e-mails registados</v>
+      </c>
+      <c r="D439" t="str">
+        <v>Sin correos registrados</v>
+      </c>
+      <c r="E439" t="str">
+        <v>Aucun e-mail enregistré</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="str">
+        <v>Recipient</v>
+      </c>
+      <c r="B440" t="str">
+        <v>Recipient</v>
+      </c>
+      <c r="C440" t="str">
+        <v>Destinatário</v>
+      </c>
+      <c r="D440" t="str">
+        <v>Destinatario</v>
+      </c>
+      <c r="E440" t="str">
+        <v>Destinataire</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="str">
+        <v>Reason of the failure</v>
+      </c>
+      <c r="B441" t="str">
+        <v>Reason of the failure</v>
+      </c>
+      <c r="C441" t="str">
+        <v>Razão da falha</v>
+      </c>
+      <c r="D441" t="str">
+        <v>Motivo del fallo</v>
+      </c>
+      <c r="E441" t="str">
+        <v>Raison de l'échec</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="str">
+        <v>Subject</v>
+      </c>
+      <c r="B442" t="str">
+        <v>Subject</v>
+      </c>
+      <c r="C442" t="str">
+        <v>Assunto</v>
+      </c>
+      <c r="D442" t="str">
+        <v>Asunto</v>
+      </c>
+      <c r="E442" t="str">
+        <v>Objet</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="str">
+        <v>E-mail type</v>
+      </c>
+      <c r="B443" t="str">
+        <v>E-mail type</v>
+      </c>
+      <c r="C443" t="str">
+        <v>Tipo de e-mail</v>
+      </c>
+      <c r="D443" t="str">
+        <v>Tipo de correo</v>
+      </c>
+      <c r="E443" t="str">
+        <v>Type d'e-mail</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="str">
+        <v>System</v>
+      </c>
+      <c r="B444" t="str">
+        <v>System</v>
+      </c>
+      <c r="C444" t="str">
+        <v>Sistema</v>
+      </c>
+      <c r="D444" t="str">
+        <v>Sistema</v>
+      </c>
+      <c r="E444" t="str">
+        <v>Système</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="str">
+        <v>Recommended: A4 landscape (297 × 210 mm), {{size}} (300 dpi), PNG or JPG</v>
+      </c>
+      <c r="B445" t="str">
+        <v>Recommended: A4 landscape (297 × 210 mm), {{size}} (300 dpi), PNG or JPG</v>
+      </c>
+      <c r="C445" t="str">
+        <v>Recomendado: A4 horizontal (297 × 210 mm), {{size}} (300 dpi), PNG ou JPG</v>
+      </c>
+      <c r="D445" t="str">
+        <v>Recomendado: A4 horizontal (297 × 210 mm), {{size}} (300 ppp), PNG o JPG</v>
+      </c>
+      <c r="E445" t="str">
+        <v>Recommandé : A4 paysage (297 × 210 mm), {{size}} (300 dpi), PNG ou JPG</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="str">
+        <v>Chosen image: {{width}} × {{height}} px</v>
+      </c>
+      <c r="B446" t="str">
+        <v>Chosen image: {{width}} × {{height}} px</v>
+      </c>
+      <c r="C446" t="str">
+        <v>Imagem escolhida: {{width}} × {{height}} px</v>
+      </c>
+      <c r="D446" t="str">
+        <v>Imagen elegida: {{width}} × {{height}} px</v>
+      </c>
+      <c r="E446" t="str">
+        <v>Image choisie : {{width}} × {{height}} px</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="str">
+        <v>This image is not A4 landscape: it keeps its proportions and is cropped from the centre to fill the page, so the edges may be cut off</v>
+      </c>
+      <c r="B447" t="str">
+        <v>This image is not A4 landscape: it keeps its proportions and is cropped from the centre to fill the page, so the edges may be cut off</v>
+      </c>
+      <c r="C447" t="str">
+        <v>Esta imagem não é A4 horizontal: mantém as proporções e é cortada a partir do centro para preencher a página, por isso as margens podem ser cortadas</v>
+      </c>
+      <c r="D447" t="str">
+        <v>Esta imagen no es A4 horizontal: mantiene sus proporciones y se recorta desde el centro para llenar la página, por lo que los bordes pueden quedar cortados</v>
+      </c>
+      <c r="E447" t="str">
+        <v>Cette image n’est pas en A4 paysage : elle garde ses proportions et est recadrée depuis le centre pour remplir la page, les bords peuvent donc être coupés</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="str">
+        <v>This image is small for a printed certificate and may look blurry. Use at least {{width}} px wide</v>
+      </c>
+      <c r="B448" t="str">
+        <v>This image is small for a printed certificate and may look blurry. Use at least {{width}} px wide</v>
+      </c>
+      <c r="C448" t="str">
+        <v>Esta imagem é pequena para um certificado impresso e pode ficar desfocada. Use pelo menos {{width}} px de largura</v>
+      </c>
+      <c r="D448" t="str">
+        <v>Esta imagen es pequeña para un certificado impreso y puede verse borrosa. Use al menos {{width}} px de ancho</v>
+      </c>
+      <c r="E448" t="str">
+        <v>Cette image est petite pour un certificat imprimé et peut paraître floue. Utilisez au moins {{width}} px de large</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="str">
+        <v>Click to copy</v>
+      </c>
+      <c r="B449" t="str">
+        <v>Click to copy</v>
+      </c>
+      <c r="C449" t="str">
+        <v>Clique para copiar</v>
+      </c>
+      <c r="D449" t="str">
+        <v>Haga clic para copiar</v>
+      </c>
+      <c r="E449" t="str">
+        <v>Cliquez pour copier</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="str">
+        <v>Copied</v>
+      </c>
+      <c r="B450" t="str">
+        <v>Copied</v>
+      </c>
+      <c r="C450" t="str">
+        <v>Copiado</v>
+      </c>
+      <c r="D450" t="str">
+        <v>Copiado</v>
+      </c>
+      <c r="E450" t="str">
+        <v>Copié</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="str">
+        <v>Custom</v>
+      </c>
+      <c r="B451" t="str">
+        <v>Custom</v>
+      </c>
+      <c r="C451" t="str">
+        <v>Personalizado</v>
+      </c>
+      <c r="D451" t="str">
+        <v>Personalizado</v>
+      </c>
+      <c r="E451" t="str">
+        <v>Personnalisé</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="str">
+        <v>Design the e-mail with the editor. Use the eye icon in the editor to preview it on desktop and mobile</v>
+      </c>
+      <c r="B452" t="str">
+        <v>Design the e-mail with the editor. Use the eye icon in the editor to preview it on desktop and mobile</v>
+      </c>
+      <c r="C452" t="str">
+        <v>Crie o e-mail com o editor. Use o ícone do olho no editor para o pré-visualizar no computador e no telemóvel</v>
+      </c>
+      <c r="D452" t="str">
+        <v>Diseñe el correo con el editor. Use el icono del ojo en el editor para previsualizarlo en ordenador y móvil</v>
+      </c>
+      <c r="E452" t="str">
+        <v>Concevez l’e-mail avec l’éditeur. Utilisez l’icône en forme d’œil de l’éditeur pour l’aperçu sur ordinateur et mobile</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="str">
+        <v>Filled in with each person's data when the e-mail is sent. Use them in the subject and in the content</v>
+      </c>
+      <c r="B453" t="str">
+        <v>Filled in with each person's data when the e-mail is sent. Use them in the subject and in the content</v>
+      </c>
+      <c r="C453" t="str">
+        <v>Preenchidas com os dados de cada pessoa quando o e-mail é enviado. Use-as no assunto e no conteúdo</v>
+      </c>
+      <c r="D453" t="str">
+        <v>Se rellenan con los datos de cada persona al enviar el correo. Úselas en el asunto y en el contenido</v>
+      </c>
+      <c r="E453" t="str">
+        <v>Remplies avec les données de chaque personne lors de l’envoi de l’e-mail. Utilisez-les dans l’objet et dans le contenu</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="str">
+        <v>In the editor, the variables are also in the Merge Tags option of the text toolbar</v>
+      </c>
+      <c r="B454" t="str">
+        <v>In the editor, the variables are also in the Merge Tags option of the text toolbar</v>
+      </c>
+      <c r="C454" t="str">
+        <v>No editor, as variáveis também estão na opção Merge Tags da barra de ferramentas do texto</v>
+      </c>
+      <c r="D454" t="str">
+        <v>En el editor, las variables también están en la opción Merge Tags de la barra de herramientas del texto</v>
+      </c>
+      <c r="E454" t="str">
+        <v>Dans l’éditeur, les variables sont aussi dans l’option Merge Tags de la barre d’outils du texte</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="str">
+        <v>Last updated</v>
+      </c>
+      <c r="B455" t="str">
+        <v>Last updated</v>
+      </c>
+      <c r="C455" t="str">
+        <v>Última atualização</v>
+      </c>
+      <c r="D455" t="str">
+        <v>Última actualización</v>
+      </c>
+      <c r="E455" t="str">
+        <v>Dernière mise à jour</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="str">
+        <v>No subject</v>
+      </c>
+      <c r="B456" t="str">
+        <v>No subject</v>
+      </c>
+      <c r="C456" t="str">
+        <v>Sem assunto</v>
+      </c>
+      <c r="D456" t="str">
+        <v>Sin asunto</v>
+      </c>
+      <c r="E456" t="str">
+        <v>Sans objet</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="str">
+        <v>Reload</v>
+      </c>
+      <c r="B457" t="str">
+        <v>Reload</v>
+      </c>
+      <c r="C457" t="str">
+        <v>Recarregar</v>
+      </c>
+      <c r="D457" t="str">
+        <v>Recargar</v>
+      </c>
+      <c r="E457" t="str">
+        <v>Recharger</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="str">
+        <v>Search by name or subject...</v>
+      </c>
+      <c r="B458" t="str">
+        <v>Search by name or subject...</v>
+      </c>
+      <c r="C458" t="str">
+        <v>Pesquisar por nome ou assunto...</v>
+      </c>
+      <c r="D458" t="str">
+        <v>Buscar por nombre o asunto...</v>
+      </c>
+      <c r="E458" t="str">
+        <v>Rechercher par nom ou objet...</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="str">
+        <v>Send a test</v>
+      </c>
+      <c r="B459" t="str">
+        <v>Send a test</v>
+      </c>
+      <c r="C459" t="str">
+        <v>Enviar um teste</v>
+      </c>
+      <c r="D459" t="str">
+        <v>Enviar una prueba</v>
+      </c>
+      <c r="E459" t="str">
+        <v>Envoyer un test</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="str">
+        <v>Send test e-mail</v>
+      </c>
+      <c r="B460" t="str">
+        <v>Send test e-mail</v>
+      </c>
+      <c r="C460" t="str">
+        <v>Enviar e-mail de teste</v>
+      </c>
+      <c r="D460" t="str">
+        <v>Enviar correo de prueba</v>
+      </c>
+      <c r="E460" t="str">
+        <v>Envoyer un e-mail de test</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="str">
+        <v>Sends the template as it is in the editor (even unsaved), with example data. The result is recorded in System monitoring</v>
+      </c>
+      <c r="B461" t="str">
+        <v>Sends the template as it is in the editor (even unsaved), with example data. The result is recorded in System monitoring</v>
+      </c>
+      <c r="C461" t="str">
+        <v>Envia o template tal como está no editor (mesmo por guardar), com dados de exemplo. O resultado fica registado na Monitorização do sistema</v>
+      </c>
+      <c r="D461" t="str">
+        <v>Envía la plantilla tal como está en el editor (aunque no esté guardada), con datos de ejemplo. El resultado queda registrado en la Monitorización del sistema</v>
+      </c>
+      <c r="E461" t="str">
+        <v>Envoie le modèle tel qu’il est dans l’éditeur (même non enregistré), avec des données d’exemple. Le résultat est enregistré dans la Surveillance du système</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="str">
+        <v>Sent by the platform</v>
+      </c>
+      <c r="B462" t="str">
+        <v>Sent by the platform</v>
+      </c>
+      <c r="C462" t="str">
+        <v>Enviados pela plataforma</v>
+      </c>
+      <c r="D462" t="str">
+        <v>Enviados por la plataforma</v>
+      </c>
+      <c r="E462" t="str">
+        <v>Envoyés par la plateforme</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="str">
+        <v>Test e-mail sent to {{email}}</v>
+      </c>
+      <c r="B463" t="str">
+        <v>Test e-mail sent to {{email}}</v>
+      </c>
+      <c r="C463" t="str">
+        <v>E-mail de teste enviado para {{email}}</v>
+      </c>
+      <c r="D463" t="str">
+        <v>Correo de prueba enviado a {{email}}</v>
+      </c>
+      <c r="E463" t="str">
+        <v>E-mail de test envoyé à {{email}}</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="str">
+        <v>The image could not be uploaded</v>
+      </c>
+      <c r="B464" t="str">
+        <v>The image could not be uploaded</v>
+      </c>
+      <c r="C464" t="str">
+        <v>Não foi possível carregar a imagem</v>
+      </c>
+      <c r="D464" t="str">
+        <v>No se pudo subir la imagen</v>
+      </c>
+      <c r="E464" t="str">
+        <v>Impossible de téléverser l’image</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="str">
+        <v>The name only identifies this template in the dashboard. The subject is what the person sees in their inbox</v>
+      </c>
+      <c r="B465" t="str">
+        <v>The name only identifies this template in the dashboard. The subject is what the person sees in their inbox</v>
+      </c>
+      <c r="C465" t="str">
+        <v>O nome só identifica este template no backoffice. O assunto é o que a pessoa vê na caixa de entrada</v>
+      </c>
+      <c r="D465" t="str">
+        <v>El nombre solo identifica esta plantilla en el panel. El asunto es lo que la persona ve en su bandeja de entrada</v>
+      </c>
+      <c r="E465" t="str">
+        <v>Le nom identifie seulement ce modèle dans le back-office. L’objet est ce que la personne voit dans sa boîte de réception</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="str">
+        <v>The test e-mail could not be sent</v>
+      </c>
+      <c r="B466" t="str">
+        <v>The test e-mail could not be sent</v>
+      </c>
+      <c r="C466" t="str">
+        <v>Não foi possível enviar o e-mail de teste</v>
+      </c>
+      <c r="D466" t="str">
+        <v>No se pudo enviar el correo de prueba</v>
+      </c>
+      <c r="E466" t="str">
+        <v>Impossible d’envoyer l’e-mail de test</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="str">
+        <v>This e-mail is sent by the platform, so the template cannot be deleted</v>
+      </c>
+      <c r="B467" t="str">
+        <v>This e-mail is sent by the platform, so the template cannot be deleted</v>
+      </c>
+      <c r="C467" t="str">
+        <v>Este e-mail é enviado pela plataforma, por isso o template não pode ser eliminado</v>
+      </c>
+      <c r="D467" t="str">
+        <v>Este correo lo envía la plataforma, por lo que la plantilla no se puede eliminar</v>
+      </c>
+      <c r="E467" t="str">
+        <v>Cet e-mail est envoyé par la plateforme, le modèle ne peut donc pas être supprimé</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="str">
+        <v>Variables</v>
+      </c>
+      <c r="B468" t="str">
+        <v>Variables</v>
+      </c>
+      <c r="C468" t="str">
+        <v>Variáveis</v>
+      </c>
+      <c r="D468" t="str">
+        <v>Variables</v>
+      </c>
+      <c r="E468" t="str">
+        <v>Variables</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="str">
+        <v>New registration</v>
+      </c>
+      <c r="B469" t="str">
+        <v>New registration</v>
+      </c>
+      <c r="C469" t="str">
+        <v>Novo registo</v>
+      </c>
+      <c r="D469" t="str">
+        <v>Nuevo registro</v>
+      </c>
+      <c r="E469" t="str">
+        <v>Nouvelle inscription</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="str">
+        <v>Sent to a person when they create an account</v>
+      </c>
+      <c r="B470" t="str">
+        <v>Sent to a person when they create an account</v>
+      </c>
+      <c r="C470" t="str">
+        <v>Enviado a uma pessoa quando cria uma conta</v>
+      </c>
+      <c r="D470" t="str">
+        <v>Se envía a una persona cuando crea una cuenta</v>
+      </c>
+      <c r="E470" t="str">
+        <v>Envoyé à une personne lorsqu’elle crée un compte</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="str">
+        <v>Account status change</v>
+      </c>
+      <c r="B471" t="str">
+        <v>Account status change</v>
+      </c>
+      <c r="C471" t="str">
+        <v>Alteração do estado da conta</v>
+      </c>
+      <c r="D471" t="str">
+        <v>Cambio del estado de la cuenta</v>
+      </c>
+      <c r="E471" t="str">
+        <v>Changement du statut du compte</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="str">
+        <v>Sent to a person when an administrator changes the status of their account</v>
+      </c>
+      <c r="B472" t="str">
+        <v>Sent to a person when an administrator changes the status of their account</v>
+      </c>
+      <c r="C472" t="str">
+        <v>Enviado a uma pessoa quando um administrador altera o estado da sua conta</v>
+      </c>
+      <c r="D472" t="str">
+        <v>Se envía a una persona cuando un administrador cambia el estado de su cuenta</v>
+      </c>
+      <c r="E472" t="str">
+        <v>Envoyé à une personne lorsqu’un administrateur modifie le statut de son compte</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="str">
+        <v>Password recovery</v>
+      </c>
+      <c r="B473" t="str">
+        <v>Password recovery</v>
+      </c>
+      <c r="C473" t="str">
+        <v>Recuperação de password</v>
+      </c>
+      <c r="D473" t="str">
+        <v>Recuperación de contraseña</v>
+      </c>
+      <c r="E473" t="str">
+        <v>Récupération du mot de passe</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="str">
+        <v>Sent with the code to recover a password</v>
+      </c>
+      <c r="B474" t="str">
+        <v>Sent with the code to recover a password</v>
+      </c>
+      <c r="C474" t="str">
+        <v>Enviado com o código para recuperar a password</v>
+      </c>
+      <c r="D474" t="str">
+        <v>Se envía con el código para recuperar la contraseña</v>
+      </c>
+      <c r="E474" t="str">
+        <v>Envoyé avec le code pour récupérer le mot de passe</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="str">
+        <v>User created</v>
+      </c>
+      <c r="B475" t="str">
+        <v>User created</v>
+      </c>
+      <c r="C475" t="str">
+        <v>Utilizador criado</v>
+      </c>
+      <c r="D475" t="str">
+        <v>Usuario creado</v>
+      </c>
+      <c r="E475" t="str">
+        <v>Utilisateur créé</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="str">
+        <v>Sent when an administrator creates an account for someone</v>
+      </c>
+      <c r="B476" t="str">
+        <v>Sent when an administrator creates an account for someone</v>
+      </c>
+      <c r="C476" t="str">
+        <v>Enviado quando um administrador cria uma conta para alguém</v>
+      </c>
+      <c r="D476" t="str">
+        <v>Se envía cuando un administrador crea una cuenta para alguien</v>
+      </c>
+      <c r="E476" t="str">
+        <v>Envoyé lorsqu’un administrateur crée un compte pour quelqu’un</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="str">
+        <v>The name of the person receiving the e-mail</v>
+      </c>
+      <c r="B477" t="str">
+        <v>The name of the person receiving the e-mail</v>
+      </c>
+      <c r="C477" t="str">
+        <v>O nome da pessoa que recebe o e-mail</v>
+      </c>
+      <c r="D477" t="str">
+        <v>El nombre de la persona que recibe el correo</v>
+      </c>
+      <c r="E477" t="str">
+        <v>Le nom de la personne qui reçoit l’e-mail</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="str">
+        <v>The new status of the account</v>
+      </c>
+      <c r="B478" t="str">
+        <v>The new status of the account</v>
+      </c>
+      <c r="C478" t="str">
+        <v>O novo estado da conta</v>
+      </c>
+      <c r="D478" t="str">
+        <v>El nuevo estado de la cuenta</v>
+      </c>
+      <c r="E478" t="str">
+        <v>Le nouveau statut du compte</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="str">
+        <v>Code</v>
+      </c>
+      <c r="B479" t="str">
+        <v>Code</v>
+      </c>
+      <c r="C479" t="str">
+        <v>Código</v>
+      </c>
+      <c r="D479" t="str">
+        <v>Código</v>
+      </c>
+      <c r="E479" t="str">
+        <v>Code</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="str">
+        <v>The code to recover the password</v>
+      </c>
+      <c r="B480" t="str">
+        <v>The code to recover the password</v>
+      </c>
+      <c r="C480" t="str">
+        <v>O código para recuperar a password</v>
+      </c>
+      <c r="D480" t="str">
+        <v>El código para recuperar la contraseña</v>
+      </c>
+      <c r="E480" t="str">
+        <v>Le code pour récupérer le mot de passe</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="str">
+        <v>Created in the dashboard, not sent automatically</v>
+      </c>
+      <c r="B481" t="str">
+        <v>Created in the dashboard, not sent automatically</v>
+      </c>
+      <c r="C481" t="str">
+        <v>Criado no backoffice, não é enviado automaticamente</v>
+      </c>
+      <c r="D481" t="str">
+        <v>Creada en el panel, no se envía automáticamente</v>
+      </c>
+      <c r="E481" t="str">
+        <v>Créé dans le back-office, non envoyé automatiquement</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E384"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E481"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: deploy notes for communications and translations
Deploy guide: communications and click tracking migrations, API_PUBLIC_URL, the fonts folder and its public URL. Translations (pt/es/fr) for the Media library, the e-mail editor and its blocks, the template pages and the communications; already imported into the staging language table.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E481"/>
+  <dimension ref="A1:E651"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8576,9 +8576,2899 @@
         <v>Créé dans le back-office, non envoyé automatiquement</v>
       </c>
     </row>
+    <row r="482">
+      <c r="A482" t="str">
+        <v>1 column</v>
+      </c>
+      <c r="B482" t="str">
+        <v>1 column</v>
+      </c>
+      <c r="C482" t="str">
+        <v>1 coluna</v>
+      </c>
+      <c r="D482" t="str">
+        <v>1 columna</v>
+      </c>
+      <c r="E482" t="str">
+        <v>1 colonne</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="str">
+        <v>2 columns</v>
+      </c>
+      <c r="B483" t="str">
+        <v>2 columns</v>
+      </c>
+      <c r="C483" t="str">
+        <v>2 colunas</v>
+      </c>
+      <c r="D483" t="str">
+        <v>2 columnas</v>
+      </c>
+      <c r="E483" t="str">
+        <v>2 colonnes</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="str">
+        <v>3 columns</v>
+      </c>
+      <c r="B484" t="str">
+        <v>3 columns</v>
+      </c>
+      <c r="C484" t="str">
+        <v>3 colunas</v>
+      </c>
+      <c r="D484" t="str">
+        <v>3 columnas</v>
+      </c>
+      <c r="E484" t="str">
+        <v>3 colonnes</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="str">
+        <v>Banner</v>
+      </c>
+      <c r="B485" t="str">
+        <v>Banner</v>
+      </c>
+      <c r="C485" t="str">
+        <v>Banner</v>
+      </c>
+      <c r="D485" t="str">
+        <v>Banner</v>
+      </c>
+      <c r="E485" t="str">
+        <v>Bannière</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="str">
+        <v>Button</v>
+      </c>
+      <c r="B486" t="str">
+        <v>Button</v>
+      </c>
+      <c r="C486" t="str">
+        <v>Botão</v>
+      </c>
+      <c r="D486" t="str">
+        <v>Botón</v>
+      </c>
+      <c r="E486" t="str">
+        <v>Bouton</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="str">
+        <v>Click here</v>
+      </c>
+      <c r="B487" t="str">
+        <v>Click here</v>
+      </c>
+      <c r="C487" t="str">
+        <v>Clique aqui</v>
+      </c>
+      <c r="D487" t="str">
+        <v>Haga clic aquí</v>
+      </c>
+      <c r="E487" t="str">
+        <v>Cliquez ici</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="str">
+        <v>Column</v>
+      </c>
+      <c r="B488" t="str">
+        <v>Column</v>
+      </c>
+      <c r="C488" t="str">
+        <v>Coluna</v>
+      </c>
+      <c r="D488" t="str">
+        <v>Columna</v>
+      </c>
+      <c r="E488" t="str">
+        <v>Colonne</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="str">
+        <v>Divider</v>
+      </c>
+      <c r="B489" t="str">
+        <v>Divider</v>
+      </c>
+      <c r="C489" t="str">
+        <v>Separador</v>
+      </c>
+      <c r="D489" t="str">
+        <v>Separador</v>
+      </c>
+      <c r="E489" t="str">
+        <v>Séparateur</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="str">
+        <v>Footer</v>
+      </c>
+      <c r="B490" t="str">
+        <v>Footer</v>
+      </c>
+      <c r="C490" t="str">
+        <v>Rodapé</v>
+      </c>
+      <c r="D490" t="str">
+        <v>Pie de página</v>
+      </c>
+      <c r="E490" t="str">
+        <v>Pied de page</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="str">
+        <v>Greeting</v>
+      </c>
+      <c r="B491" t="str">
+        <v>Greeting</v>
+      </c>
+      <c r="C491" t="str">
+        <v>Saudação</v>
+      </c>
+      <c r="D491" t="str">
+        <v>Saludo</v>
+      </c>
+      <c r="E491" t="str">
+        <v>Salutation</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="str">
+        <v>Header</v>
+      </c>
+      <c r="B492" t="str">
+        <v>Header</v>
+      </c>
+      <c r="C492" t="str">
+        <v>Cabeçalho</v>
+      </c>
+      <c r="D492" t="str">
+        <v>Encabezado</v>
+      </c>
+      <c r="E492" t="str">
+        <v>En-tête</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="str">
+        <v>Hello</v>
+      </c>
+      <c r="B493" t="str">
+        <v>Hello</v>
+      </c>
+      <c r="C493" t="str">
+        <v>Olá</v>
+      </c>
+      <c r="D493" t="str">
+        <v>Hola</v>
+      </c>
+      <c r="E493" t="str">
+        <v>Bonjour</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="str">
+        <v>Image</v>
+      </c>
+      <c r="B494" t="str">
+        <v>Image</v>
+      </c>
+      <c r="C494" t="str">
+        <v>Imagem</v>
+      </c>
+      <c r="D494" t="str">
+        <v>Imagen</v>
+      </c>
+      <c r="E494" t="str">
+        <v>Image</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="str">
+        <v>Image and text</v>
+      </c>
+      <c r="B495" t="str">
+        <v>Image and text</v>
+      </c>
+      <c r="C495" t="str">
+        <v>Imagem e texto</v>
+      </c>
+      <c r="D495" t="str">
+        <v>Imagen y texto</v>
+      </c>
+      <c r="E495" t="str">
+        <v>Image et texte</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="str">
+        <v>Insert variable</v>
+      </c>
+      <c r="B496" t="str">
+        <v>Insert variable</v>
+      </c>
+      <c r="C496" t="str">
+        <v>Inserir variável</v>
+      </c>
+      <c r="D496" t="str">
+        <v>Insertar variable</v>
+      </c>
+      <c r="E496" t="str">
+        <v>Insérer une variable</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="str">
+        <v>Layout</v>
+      </c>
+      <c r="B497" t="str">
+        <v>Layout</v>
+      </c>
+      <c r="C497" t="str">
+        <v>Estrutura</v>
+      </c>
+      <c r="D497" t="str">
+        <v>Estructura</v>
+      </c>
+      <c r="E497" t="str">
+        <v>Mise en page</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="str">
+        <v>Ready-made</v>
+      </c>
+      <c r="B498" t="str">
+        <v>Ready-made</v>
+      </c>
+      <c r="C498" t="str">
+        <v>Prontos a usar</v>
+      </c>
+      <c r="D498" t="str">
+        <v>Listos para usar</v>
+      </c>
+      <c r="E498" t="str">
+        <v>Prêts à l’emploi</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="str">
+        <v>Rebuild</v>
+      </c>
+      <c r="B499" t="str">
+        <v>Rebuild</v>
+      </c>
+      <c r="C499" t="str">
+        <v>Refazer</v>
+      </c>
+      <c r="D499" t="str">
+        <v>Rehacer</v>
+      </c>
+      <c r="E499" t="str">
+        <v>Refaire</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="str">
+        <v>Rebuild in the new editor</v>
+      </c>
+      <c r="B500" t="str">
+        <v>Rebuild in the new editor</v>
+      </c>
+      <c r="C500" t="str">
+        <v>Refazer no editor novo</v>
+      </c>
+      <c r="D500" t="str">
+        <v>Rehacer en el editor nuevo</v>
+      </c>
+      <c r="E500" t="str">
+        <v>Refaire dans le nouvel éditeur</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="str">
+        <v>Rebuild this template in the new editor?</v>
+      </c>
+      <c r="B501" t="str">
+        <v>Rebuild this template in the new editor?</v>
+      </c>
+      <c r="C501" t="str">
+        <v>Refazer este template no editor novo?</v>
+      </c>
+      <c r="D501" t="str">
+        <v>¿Rehacer esta plantilla en el editor nuevo?</v>
+      </c>
+      <c r="E501" t="str">
+        <v>Refaire ce modèle dans le nouvel éditeur ?</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="str">
+        <v>It keeps working and can still be edited here. To use the new editor (blocks, columns, saved styles) it has to be rebuilt from scratch: the current content is only replaced when you save</v>
+      </c>
+      <c r="B502" t="str">
+        <v>It keeps working and can still be edited here. To use the new editor (blocks, columns, saved styles) it has to be rebuilt from scratch: the current content is only replaced when you save</v>
+      </c>
+      <c r="C502" t="str">
+        <v>Continua a funcionar e ainda se pode editar aqui. Para usar o editor novo (blocos, colunas, estilos) tem de ser refeito de raiz: o conteúdo atual só é substituído quando guardar</v>
+      </c>
+      <c r="D502" t="str">
+        <v>Sigue funcionando y todavía se puede editar aquí. Para usar el editor nuevo (bloques, columnas, estilos) hay que rehacerla desde cero: el contenido actual solo se reemplaza al guardar</v>
+      </c>
+      <c r="E502" t="str">
+        <v>Il continue de fonctionner et peut encore être modifié ici. Pour utiliser le nouvel éditeur (blocs, colonnes, styles), il doit être refait de zéro : le contenu actuel n’est remplacé qu’à l’enregistrement</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="str">
+        <v>The design starts from a new base. The current content stays saved until you click Save</v>
+      </c>
+      <c r="B503" t="str">
+        <v>The design starts from a new base. The current content stays saved until you click Save</v>
+      </c>
+      <c r="C503" t="str">
+        <v>O desenho começa de uma base nova. O conteúdo atual fica guardado até clicar em Guardar</v>
+      </c>
+      <c r="D503" t="str">
+        <v>El diseño empieza desde una base nueva. El contenido actual sigue guardado hasta que haga clic en Guardar</v>
+      </c>
+      <c r="E503" t="str">
+        <v>Le design repart d’une base neuve. Le contenu actuel reste enregistré jusqu’à ce que vous cliquiez sur Enregistrer</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="str">
+        <v>This e-mail was sent automatically, please do not reply</v>
+      </c>
+      <c r="B504" t="str">
+        <v>This e-mail was sent automatically, please do not reply</v>
+      </c>
+      <c r="C504" t="str">
+        <v>Este e-mail foi enviado automaticamente, por favor não responda</v>
+      </c>
+      <c r="D504" t="str">
+        <v>Este correo se envió automáticamente, por favor no responda</v>
+      </c>
+      <c r="E504" t="str">
+        <v>Cet e-mail a été envoyé automatiquement, merci de ne pas répondre</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="str">
+        <v>This template was made in the previous editor</v>
+      </c>
+      <c r="B505" t="str">
+        <v>This template was made in the previous editor</v>
+      </c>
+      <c r="C505" t="str">
+        <v>Este template foi feito no editor anterior</v>
+      </c>
+      <c r="D505" t="str">
+        <v>Esta plantilla se creó en el editor anterior</v>
+      </c>
+      <c r="E505" t="str">
+        <v>Ce modèle a été créé dans l’ancien éditeur</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="str">
+        <v>Social</v>
+      </c>
+      <c r="B506" t="str">
+        <v>Social</v>
+      </c>
+      <c r="C506" t="str">
+        <v>Redes sociais</v>
+      </c>
+      <c r="D506" t="str">
+        <v>Redes sociales</v>
+      </c>
+      <c r="E506" t="str">
+        <v>Réseaux sociaux</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="str">
+        <v>Spacer</v>
+      </c>
+      <c r="B507" t="str">
+        <v>Spacer</v>
+      </c>
+      <c r="C507" t="str">
+        <v>Espaço</v>
+      </c>
+      <c r="D507" t="str">
+        <v>Espacio</v>
+      </c>
+      <c r="E507" t="str">
+        <v>Espace</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="str">
+        <v>Text</v>
+      </c>
+      <c r="B508" t="str">
+        <v>Text</v>
+      </c>
+      <c r="C508" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D508" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="E508" t="str">
+        <v>Texte</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="str">
+        <v>Title</v>
+      </c>
+      <c r="B509" t="str">
+        <v>Title</v>
+      </c>
+      <c r="C509" t="str">
+        <v>Título</v>
+      </c>
+      <c r="D509" t="str">
+        <v>Título</v>
+      </c>
+      <c r="E509" t="str">
+        <v>Titre</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="B510" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="C510" t="str">
+        <v>Variável</v>
+      </c>
+      <c r="D510" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="E510" t="str">
+        <v>Variable</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="str">
+        <v>Write your text here</v>
+      </c>
+      <c r="B511" t="str">
+        <v>Write your text here</v>
+      </c>
+      <c r="C511" t="str">
+        <v>Escreva aqui o seu texto</v>
+      </c>
+      <c r="D511" t="str">
+        <v>Escriba aquí su texto</v>
+      </c>
+      <c r="E511" t="str">
+        <v>Écrivez votre texte ici</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="str">
+        <v>Your title</v>
+      </c>
+      <c r="B512" t="str">
+        <v>Your title</v>
+      </c>
+      <c r="C512" t="str">
+        <v>O seu título</v>
+      </c>
+      <c r="D512" t="str">
+        <v>Su título</v>
+      </c>
+      <c r="E512" t="str">
+        <v>Votre titre</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="str">
+        <v>Communications</v>
+      </c>
+      <c r="B513" t="str">
+        <v>Communications</v>
+      </c>
+      <c r="C513" t="str">
+        <v>Comunicações</v>
+      </c>
+      <c r="D513" t="str">
+        <v>Comunicaciones</v>
+      </c>
+      <c r="E513" t="str">
+        <v>Communications</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="str">
+        <v>Communication</v>
+      </c>
+      <c r="B514" t="str">
+        <v>Communication</v>
+      </c>
+      <c r="C514" t="str">
+        <v>Comunicação</v>
+      </c>
+      <c r="D514" t="str">
+        <v>Comunicación</v>
+      </c>
+      <c r="E514" t="str">
+        <v>Communication</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="str">
+        <v>E-mails sent by the platform to the users you choose</v>
+      </c>
+      <c r="B515" t="str">
+        <v>E-mails sent by the platform to the users you choose</v>
+      </c>
+      <c r="C515" t="str">
+        <v>E-mails enviados pela plataforma aos utilizadores que escolher</v>
+      </c>
+      <c r="D515" t="str">
+        <v>Correos enviados por la plataforma a los usuarios que elija</v>
+      </c>
+      <c r="E515" t="str">
+        <v>E-mails envoyés par la plateforme aux utilisateurs de votre choix</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="str">
+        <v>New communication</v>
+      </c>
+      <c r="B516" t="str">
+        <v>New communication</v>
+      </c>
+      <c r="C516" t="str">
+        <v>Nova comunicação</v>
+      </c>
+      <c r="D516" t="str">
+        <v>Nueva comunicación</v>
+      </c>
+      <c r="E516" t="str">
+        <v>Nouvelle communication</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="str">
+        <v>Only identifies the communication in the dashboard</v>
+      </c>
+      <c r="B517" t="str">
+        <v>Only identifies the communication in the dashboard</v>
+      </c>
+      <c r="C517" t="str">
+        <v>Só identifica a comunicação no backoffice</v>
+      </c>
+      <c r="D517" t="str">
+        <v>Solo identifica la comunicación en el panel</v>
+      </c>
+      <c r="E517" t="str">
+        <v>Identifie seulement la communication dans le back-office</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="str">
+        <v>Audience</v>
+      </c>
+      <c r="B518" t="str">
+        <v>Audience</v>
+      </c>
+      <c r="C518" t="str">
+        <v>Público</v>
+      </c>
+      <c r="D518" t="str">
+        <v>Audiencia</v>
+      </c>
+      <c r="E518" t="str">
+        <v>Audience</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="str">
+        <v>Delivery</v>
+      </c>
+      <c r="B519" t="str">
+        <v>Delivery</v>
+      </c>
+      <c r="C519" t="str">
+        <v>Envio</v>
+      </c>
+      <c r="D519" t="str">
+        <v>Envío</v>
+      </c>
+      <c r="E519" t="str">
+        <v>Envoi</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="str">
+        <v>Draft</v>
+      </c>
+      <c r="B520" t="str">
+        <v>Draft</v>
+      </c>
+      <c r="C520" t="str">
+        <v>Rascunho</v>
+      </c>
+      <c r="D520" t="str">
+        <v>Borrador</v>
+      </c>
+      <c r="E520" t="str">
+        <v>Brouillon</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="str">
+        <v>Scheduled</v>
+      </c>
+      <c r="B521" t="str">
+        <v>Scheduled</v>
+      </c>
+      <c r="C521" t="str">
+        <v>Agendada</v>
+      </c>
+      <c r="D521" t="str">
+        <v>Programada</v>
+      </c>
+      <c r="E521" t="str">
+        <v>Planifiée</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="str">
+        <v>Sending</v>
+      </c>
+      <c r="B522" t="str">
+        <v>Sending</v>
+      </c>
+      <c r="C522" t="str">
+        <v>A enviar</v>
+      </c>
+      <c r="D522" t="str">
+        <v>Enviando</v>
+      </c>
+      <c r="E522" t="str">
+        <v>En cours d’envoi</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="str">
+        <v>Cancelled</v>
+      </c>
+      <c r="B523" t="str">
+        <v>Cancelled</v>
+      </c>
+      <c r="C523" t="str">
+        <v>Cancelada</v>
+      </c>
+      <c r="D523" t="str">
+        <v>Cancelada</v>
+      </c>
+      <c r="E523" t="str">
+        <v>Annulée</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="B524" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="C524" t="str">
+        <v>Pendente</v>
+      </c>
+      <c r="D524" t="str">
+        <v>Pendiente</v>
+      </c>
+      <c r="E524" t="str">
+        <v>En attente</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="str">
+        <v>Duplicate</v>
+      </c>
+      <c r="B525" t="str">
+        <v>Duplicate</v>
+      </c>
+      <c r="C525" t="str">
+        <v>Duplicar</v>
+      </c>
+      <c r="D525" t="str">
+        <v>Duplicar</v>
+      </c>
+      <c r="E525" t="str">
+        <v>Dupliquer</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="str">
+        <v>Delete this communication?</v>
+      </c>
+      <c r="B526" t="str">
+        <v>Delete this communication?</v>
+      </c>
+      <c r="C526" t="str">
+        <v>Eliminar esta comunicação?</v>
+      </c>
+      <c r="D526" t="str">
+        <v>¿Eliminar esta comunicación?</v>
+      </c>
+      <c r="E526" t="str">
+        <v>Supprimer cette communication ?</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="str">
+        <v>The communication and its list of recipients will be permanently deleted. The e-mails already sent are not recalled</v>
+      </c>
+      <c r="B527" t="str">
+        <v>The communication and its list of recipients will be permanently deleted. The e-mails already sent are not recalled</v>
+      </c>
+      <c r="C527" t="str">
+        <v>A comunicação e a lista de destinatários serão eliminadas permanentemente. Os e-mails já enviados não são recolhidos</v>
+      </c>
+      <c r="D527" t="str">
+        <v>La comunicación y su lista de destinatarios se eliminarán permanentemente. Los correos ya enviados no se retiran</v>
+      </c>
+      <c r="E527" t="str">
+        <v>La communication et sa liste de destinataires seront supprimées définitivement. Les e-mails déjà envoyés ne sont pas rappelés</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="str">
+        <v>Communication deleted</v>
+      </c>
+      <c r="B528" t="str">
+        <v>Communication deleted</v>
+      </c>
+      <c r="C528" t="str">
+        <v>Comunicação eliminada</v>
+      </c>
+      <c r="D528" t="str">
+        <v>Comunicación eliminada</v>
+      </c>
+      <c r="E528" t="str">
+        <v>Communication supprimée</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="str">
+        <v>Communication saved</v>
+      </c>
+      <c r="B529" t="str">
+        <v>Communication saved</v>
+      </c>
+      <c r="C529" t="str">
+        <v>Comunicação guardada</v>
+      </c>
+      <c r="D529" t="str">
+        <v>Comunicación guardada</v>
+      </c>
+      <c r="E529" t="str">
+        <v>Communication enregistrée</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="str">
+        <v>Communication scheduled for {{date}}</v>
+      </c>
+      <c r="B530" t="str">
+        <v>Communication scheduled for {{date}}</v>
+      </c>
+      <c r="C530" t="str">
+        <v>Comunicação agendada para {{date}}</v>
+      </c>
+      <c r="D530" t="str">
+        <v>Comunicación programada para {{date}}</v>
+      </c>
+      <c r="E530" t="str">
+        <v>Communication planifiée pour le {{date}}</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="str">
+        <v>Sending to {{count}} recipients</v>
+      </c>
+      <c r="B531" t="str">
+        <v>Sending to {{count}} recipients</v>
+      </c>
+      <c r="C531" t="str">
+        <v>A enviar para {{count}} destinatários</v>
+      </c>
+      <c r="D531" t="str">
+        <v>Enviando a {{count}} destinatarios</v>
+      </c>
+      <c r="E531" t="str">
+        <v>Envoi à {{count}} destinataires</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="str">
+        <v>Send this communication now?</v>
+      </c>
+      <c r="B532" t="str">
+        <v>Send this communication now?</v>
+      </c>
+      <c r="C532" t="str">
+        <v>Enviar esta comunicação agora?</v>
+      </c>
+      <c r="D532" t="str">
+        <v>¿Enviar esta comunicación ahora?</v>
+      </c>
+      <c r="E532" t="str">
+        <v>Envoyer cette communication maintenant ?</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="str">
+        <v>It will be sent to {{count}} recipients. This cannot be undone</v>
+      </c>
+      <c r="B533" t="str">
+        <v>It will be sent to {{count}} recipients. This cannot be undone</v>
+      </c>
+      <c r="C533" t="str">
+        <v>Será enviada a {{count}} destinatários. Isto não pode ser desfeito</v>
+      </c>
+      <c r="D533" t="str">
+        <v>Se enviará a {{count}} destinatarios. Esto no se puede deshacer</v>
+      </c>
+      <c r="E533" t="str">
+        <v>Elle sera envoyée à {{count}} destinataires. Cette action est irréversible</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="str">
+        <v>It will be sent to {{count}} recipients on the chosen date and time</v>
+      </c>
+      <c r="B534" t="str">
+        <v>It will be sent to {{count}} recipients on the chosen date and time</v>
+      </c>
+      <c r="C534" t="str">
+        <v>Será enviada a {{count}} destinatários na data e hora escolhidas</v>
+      </c>
+      <c r="D534" t="str">
+        <v>Se enviará a {{count}} destinatarios en la fecha y hora elegidas</v>
+      </c>
+      <c r="E534" t="str">
+        <v>Elle sera envoyée à {{count}} destinataires à la date et à l’heure choisies</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="str">
+        <v>Send now</v>
+      </c>
+      <c r="B535" t="str">
+        <v>Send now</v>
+      </c>
+      <c r="C535" t="str">
+        <v>Enviar agora</v>
+      </c>
+      <c r="D535" t="str">
+        <v>Enviar ahora</v>
+      </c>
+      <c r="E535" t="str">
+        <v>Envoyer maintenant</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="str">
+        <v>Schedule</v>
+      </c>
+      <c r="B536" t="str">
+        <v>Schedule</v>
+      </c>
+      <c r="C536" t="str">
+        <v>Agendar</v>
+      </c>
+      <c r="D536" t="str">
+        <v>Programar</v>
+      </c>
+      <c r="E536" t="str">
+        <v>Planifier</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="str">
+        <v>Schedule the sending</v>
+      </c>
+      <c r="B537" t="str">
+        <v>Schedule the sending</v>
+      </c>
+      <c r="C537" t="str">
+        <v>Agendar o envio</v>
+      </c>
+      <c r="D537" t="str">
+        <v>Programar el envío</v>
+      </c>
+      <c r="E537" t="str">
+        <v>Planifier l’envoi</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="str">
+        <v>Send</v>
+      </c>
+      <c r="B538" t="str">
+        <v>Send</v>
+      </c>
+      <c r="C538" t="str">
+        <v>Enviar</v>
+      </c>
+      <c r="D538" t="str">
+        <v>Enviar</v>
+      </c>
+      <c r="E538" t="str">
+        <v>Envoyer</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="str">
+        <v>Send a test to yourself first. The communication is saved when you send or schedule it</v>
+      </c>
+      <c r="B539" t="str">
+        <v>Send a test to yourself first. The communication is saved when you send or schedule it</v>
+      </c>
+      <c r="C539" t="str">
+        <v>Envie primeiro um teste para si. A comunicação é guardada quando a enviar ou agendar</v>
+      </c>
+      <c r="D539" t="str">
+        <v>Envíese primero una prueba. La comunicación se guarda al enviarla o programarla</v>
+      </c>
+      <c r="E539" t="str">
+        <v>Envoyez d’abord un test à vous-même. La communication est enregistrée lorsque vous l’envoyez ou la planifiez</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="str">
+        <v>Cancel scheduling</v>
+      </c>
+      <c r="B540" t="str">
+        <v>Cancel scheduling</v>
+      </c>
+      <c r="C540" t="str">
+        <v>Cancelar agendamento</v>
+      </c>
+      <c r="D540" t="str">
+        <v>Cancelar programación</v>
+      </c>
+      <c r="E540" t="str">
+        <v>Annuler la planification</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="str">
+        <v>Cancel sending</v>
+      </c>
+      <c r="B541" t="str">
+        <v>Cancel sending</v>
+      </c>
+      <c r="C541" t="str">
+        <v>Cancelar envio</v>
+      </c>
+      <c r="D541" t="str">
+        <v>Cancelar envío</v>
+      </c>
+      <c r="E541" t="str">
+        <v>Annuler l’envoi</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="str">
+        <v>Cancel the scheduling?</v>
+      </c>
+      <c r="B542" t="str">
+        <v>Cancel the scheduling?</v>
+      </c>
+      <c r="C542" t="str">
+        <v>Cancelar o agendamento?</v>
+      </c>
+      <c r="D542" t="str">
+        <v>¿Cancelar la programación?</v>
+      </c>
+      <c r="E542" t="str">
+        <v>Annuler la planification ?</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="str">
+        <v>Cancel the sending?</v>
+      </c>
+      <c r="B543" t="str">
+        <v>Cancel the sending?</v>
+      </c>
+      <c r="C543" t="str">
+        <v>Cancelar o envio?</v>
+      </c>
+      <c r="D543" t="str">
+        <v>¿Cancelar el envío?</v>
+      </c>
+      <c r="E543" t="str">
+        <v>Annuler l’envoi ?</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="str">
+        <v>The communication goes back to draft</v>
+      </c>
+      <c r="B544" t="str">
+        <v>The communication goes back to draft</v>
+      </c>
+      <c r="C544" t="str">
+        <v>A comunicação volta a rascunho</v>
+      </c>
+      <c r="D544" t="str">
+        <v>La comunicación vuelve a borrador</v>
+      </c>
+      <c r="E544" t="str">
+        <v>La communication redevient un brouillon</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="str">
+        <v>The e-mails already sent are not recalled; the remaining ones will not be sent</v>
+      </c>
+      <c r="B545" t="str">
+        <v>The e-mails already sent are not recalled; the remaining ones will not be sent</v>
+      </c>
+      <c r="C545" t="str">
+        <v>Os e-mails já enviados não são recolhidos; os restantes não serão enviados</v>
+      </c>
+      <c r="D545" t="str">
+        <v>Los correos ya enviados no se retiran; el resto no se enviará</v>
+      </c>
+      <c r="E545" t="str">
+        <v>Les e-mails déjà envoyés ne sont pas rappelés ; les autres ne seront pas envoyés</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="str">
+        <v>Yes, cancel</v>
+      </c>
+      <c r="B546" t="str">
+        <v>Yes, cancel</v>
+      </c>
+      <c r="C546" t="str">
+        <v>Sim, cancelar</v>
+      </c>
+      <c r="D546" t="str">
+        <v>Sí, cancelar</v>
+      </c>
+      <c r="E546" t="str">
+        <v>Oui, annuler</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="str">
+        <v>The sending failed</v>
+      </c>
+      <c r="B547" t="str">
+        <v>The sending failed</v>
+      </c>
+      <c r="C547" t="str">
+        <v>O envio falhou</v>
+      </c>
+      <c r="D547" t="str">
+        <v>El envío falló</v>
+      </c>
+      <c r="E547" t="str">
+        <v>L’envoi a échoué</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="str">
+        <v>{{sent}} of {{total}} sent</v>
+      </c>
+      <c r="B548" t="str">
+        <v>{{sent}} of {{total}} sent</v>
+      </c>
+      <c r="C548" t="str">
+        <v>{{sent}} de {{total}} enviados</v>
+      </c>
+      <c r="D548" t="str">
+        <v>{{sent}} de {{total}} enviados</v>
+      </c>
+      <c r="E548" t="str">
+        <v>{{sent}} sur {{total}} envoyés</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="str">
+        <v>{{count}} failed</v>
+      </c>
+      <c r="B549" t="str">
+        <v>{{count}} failed</v>
+      </c>
+      <c r="C549" t="str">
+        <v>{{count}} falharam</v>
+      </c>
+      <c r="D549" t="str">
+        <v>{{count}} fallaron</v>
+      </c>
+      <c r="E549" t="str">
+        <v>{{count}} en échec</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="str">
+        <v>{{count}} pending</v>
+      </c>
+      <c r="B550" t="str">
+        <v>{{count}} pending</v>
+      </c>
+      <c r="C550" t="str">
+        <v>{{count}} pendentes</v>
+      </c>
+      <c r="D550" t="str">
+        <v>{{count}} pendientes</v>
+      </c>
+      <c r="E550" t="str">
+        <v>{{count}} en attente</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="str">
+        <v>Try the failed again</v>
+      </c>
+      <c r="B551" t="str">
+        <v>Try the failed again</v>
+      </c>
+      <c r="C551" t="str">
+        <v>Tentar de novo os que falharam</v>
+      </c>
+      <c r="D551" t="str">
+        <v>Reintentar los que fallaron</v>
+      </c>
+      <c r="E551" t="str">
+        <v>Réessayer ceux qui ont échoué</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="str">
+        <v>Retrying the failed recipients</v>
+      </c>
+      <c r="B552" t="str">
+        <v>Retrying the failed recipients</v>
+      </c>
+      <c r="C552" t="str">
+        <v>A tentar de novo os destinatários que falharam</v>
+      </c>
+      <c r="D552" t="str">
+        <v>Reintentando los destinatarios que fallaron</v>
+      </c>
+      <c r="E552" t="str">
+        <v>Nouvelle tentative pour les destinataires en échec</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="str">
+        <v>The name only identifies the communication in the dashboard. The subject is what the person sees in their inbox</v>
+      </c>
+      <c r="B553" t="str">
+        <v>The name only identifies the communication in the dashboard. The subject is what the person sees in their inbox</v>
+      </c>
+      <c r="C553" t="str">
+        <v>O nome só identifica a comunicação no backoffice. O assunto é o que a pessoa vê na caixa de entrada</v>
+      </c>
+      <c r="D553" t="str">
+        <v>El nombre solo identifica la comunicación en el panel. El asunto es lo que la persona ve en su bandeja de entrada</v>
+      </c>
+      <c r="E553" t="str">
+        <v>Le nom identifie seulement la communication dans le back-office. L’objet est ce que la personne voit dans sa boîte de réception</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="str">
+        <v>You can use {{name}} to put each person's name</v>
+      </c>
+      <c r="B554" t="str">
+        <v>You can use {{name}} to put each person's name</v>
+      </c>
+      <c r="C554" t="str">
+        <v>Pode usar {{name}} para pôr o nome de cada pessoa</v>
+      </c>
+      <c r="D554" t="str">
+        <v>Puede usar {{name}} para poner el nombre de cada persona</v>
+      </c>
+      <c r="E554" t="str">
+        <v>Vous pouvez utiliser {{name}} pour insérer le nom de chaque personne</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="str">
+        <v>Who receives this communication</v>
+      </c>
+      <c r="B555" t="str">
+        <v>Who receives this communication</v>
+      </c>
+      <c r="C555" t="str">
+        <v>Quem recebe esta comunicação</v>
+      </c>
+      <c r="D555" t="str">
+        <v>Quién recibe esta comunicación</v>
+      </c>
+      <c r="E555" t="str">
+        <v>Qui reçoit cette communication</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="str">
+        <v>All users</v>
+      </c>
+      <c r="B556" t="str">
+        <v>All users</v>
+      </c>
+      <c r="C556" t="str">
+        <v>Todos os utilizadores</v>
+      </c>
+      <c r="D556" t="str">
+        <v>Todos los usuarios</v>
+      </c>
+      <c r="E556" t="str">
+        <v>Tous les utilisateurs</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="str">
+        <v>Selected users</v>
+      </c>
+      <c r="B557" t="str">
+        <v>Selected users</v>
+      </c>
+      <c r="C557" t="str">
+        <v>Utilizadores selecionados</v>
+      </c>
+      <c r="D557" t="str">
+        <v>Usuarios seleccionados</v>
+      </c>
+      <c r="E557" t="str">
+        <v>Utilisateurs sélectionnés</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="str">
+        <v>Sent to the people you pick, the members of the groups and everyone with access to the courses</v>
+      </c>
+      <c r="B558" t="str">
+        <v>Sent to the people you pick, the members of the groups and everyone with access to the courses</v>
+      </c>
+      <c r="C558" t="str">
+        <v>Enviada às pessoas que escolher, aos membros dos grupos e a quem tem acesso aos cursos</v>
+      </c>
+      <c r="D558" t="str">
+        <v>Se envía a las personas que elija, a los miembros de los grupos y a quienes tienen acceso a los cursos</v>
+      </c>
+      <c r="E558" t="str">
+        <v>Envoyée aux personnes choisies, aux membres des groupes et à toutes les personnes ayant accès aux cours</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="str">
+        <v>Search users by name or e-mail</v>
+      </c>
+      <c r="B559" t="str">
+        <v>Search users by name or e-mail</v>
+      </c>
+      <c r="C559" t="str">
+        <v>Pesquisar utilizadores por nome ou e-mail</v>
+      </c>
+      <c r="D559" t="str">
+        <v>Buscar usuarios por nombre o correo</v>
+      </c>
+      <c r="E559" t="str">
+        <v>Rechercher des utilisateurs par nom ou e-mail</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="str">
+        <v>Courses (everyone with access)</v>
+      </c>
+      <c r="B560" t="str">
+        <v>Courses (everyone with access)</v>
+      </c>
+      <c r="C560" t="str">
+        <v>Cursos (todos os que têm acesso)</v>
+      </c>
+      <c r="D560" t="str">
+        <v>Cursos (todos los que tienen acceso)</v>
+      </c>
+      <c r="E560" t="str">
+        <v>Cours (toutes les personnes ayant accès)</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="str">
+        <v>Narrow the audience (optional)</v>
+      </c>
+      <c r="B561" t="str">
+        <v>Narrow the audience (optional)</v>
+      </c>
+      <c r="C561" t="str">
+        <v>Restringir o público (opcional)</v>
+      </c>
+      <c r="D561" t="str">
+        <v>Restringir la audiencia (opcional)</v>
+      </c>
+      <c r="E561" t="str">
+        <v>Restreindre l’audience (facultatif)</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="str">
+        <v>Role</v>
+      </c>
+      <c r="B562" t="str">
+        <v>Role</v>
+      </c>
+      <c r="C562" t="str">
+        <v>Função</v>
+      </c>
+      <c r="D562" t="str">
+        <v>Rol</v>
+      </c>
+      <c r="E562" t="str">
+        <v>Rôle</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="str">
+        <v>Country</v>
+      </c>
+      <c r="B563" t="str">
+        <v>Country</v>
+      </c>
+      <c r="C563" t="str">
+        <v>País</v>
+      </c>
+      <c r="D563" t="str">
+        <v>País</v>
+      </c>
+      <c r="E563" t="str">
+        <v>Pays</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="str">
+        <v>Language</v>
+      </c>
+      <c r="B564" t="str">
+        <v>Language</v>
+      </c>
+      <c r="C564" t="str">
+        <v>Idioma</v>
+      </c>
+      <c r="D564" t="str">
+        <v>Idioma</v>
+      </c>
+      <c r="E564" t="str">
+        <v>Langue</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="str">
+        <v>{{count}} recipients</v>
+      </c>
+      <c r="B565" t="str">
+        <v>{{count}} recipients</v>
+      </c>
+      <c r="C565" t="str">
+        <v>{{count}} destinatários</v>
+      </c>
+      <c r="D565" t="str">
+        <v>{{count}} destinatarios</v>
+      </c>
+      <c r="E565" t="str">
+        <v>{{count}} destinataires</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="str">
+        <v>{{count}} selected</v>
+      </c>
+      <c r="B566" t="str">
+        <v>{{count}} selected</v>
+      </c>
+      <c r="C566" t="str">
+        <v>{{count}} selecionados</v>
+      </c>
+      <c r="D566" t="str">
+        <v>{{count}} seleccionados</v>
+      </c>
+      <c r="E566" t="str">
+        <v>{{count}} sélectionnés</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="str">
+        <v>{{count}} filters</v>
+      </c>
+      <c r="B567" t="str">
+        <v>{{count}} filters</v>
+      </c>
+      <c r="C567" t="str">
+        <v>{{count}} filtros</v>
+      </c>
+      <c r="D567" t="str">
+        <v>{{count}} filtros</v>
+      </c>
+      <c r="E567" t="str">
+        <v>{{count}} filtres</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="str">
+        <v>Only approved users with a valid e-mail receive it</v>
+      </c>
+      <c r="B568" t="str">
+        <v>Only approved users with a valid e-mail receive it</v>
+      </c>
+      <c r="C568" t="str">
+        <v>Só recebem os utilizadores aprovados com um e-mail válido</v>
+      </c>
+      <c r="D568" t="str">
+        <v>Solo lo reciben los usuarios aprobados con un correo válido</v>
+      </c>
+      <c r="E568" t="str">
+        <v>Seuls les utilisateurs approuvés avec une adresse e-mail valide la reçoivent</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="str">
+        <v>The e-mail that was sent</v>
+      </c>
+      <c r="B569" t="str">
+        <v>The e-mail that was sent</v>
+      </c>
+      <c r="C569" t="str">
+        <v>O e-mail que foi enviado</v>
+      </c>
+      <c r="D569" t="str">
+        <v>El correo que se envió</v>
+      </c>
+      <c r="E569" t="str">
+        <v>L’e-mail qui a été envoyé</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="str">
+        <v>Recipients</v>
+      </c>
+      <c r="B570" t="str">
+        <v>Recipients</v>
+      </c>
+      <c r="C570" t="str">
+        <v>Destinatários</v>
+      </c>
+      <c r="D570" t="str">
+        <v>Destinatarios</v>
+      </c>
+      <c r="E570" t="str">
+        <v>Destinataires</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="str">
+        <v>Who received it and, when it failed, why</v>
+      </c>
+      <c r="B571" t="str">
+        <v>Who received it and, when it failed, why</v>
+      </c>
+      <c r="C571" t="str">
+        <v>Quem o recebeu e, quando falhou, porquê</v>
+      </c>
+      <c r="D571" t="str">
+        <v>Quién lo recibió y, cuando falló, por qué</v>
+      </c>
+      <c r="E571" t="str">
+        <v>Qui l’a reçu et, en cas d’échec, pourquoi</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="str">
+        <v>Search by name, e-mail or error...</v>
+      </c>
+      <c r="B572" t="str">
+        <v>Search by name, e-mail or error...</v>
+      </c>
+      <c r="C572" t="str">
+        <v>Pesquisar por nome, e-mail ou erro...</v>
+      </c>
+      <c r="D572" t="str">
+        <v>Buscar por nombre, correo o error...</v>
+      </c>
+      <c r="E572" t="str">
+        <v>Rechercher par nom, e-mail ou erreur...</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="str">
+        <v>Sends the e-mail as it is in the editor (even unsaved), with example data. The result is recorded in System monitoring</v>
+      </c>
+      <c r="B573" t="str">
+        <v>Sends the e-mail as it is in the editor (even unsaved), with example data. The result is recorded in System monitoring</v>
+      </c>
+      <c r="C573" t="str">
+        <v>Envia o e-mail tal como está no editor (mesmo por guardar), com dados de exemplo. O resultado fica registado na Monitorização do sistema</v>
+      </c>
+      <c r="D573" t="str">
+        <v>Envía el correo tal como está en el editor (aunque no esté guardado), con datos de ejemplo. El resultado queda registrado en la Monitorización del sistema</v>
+      </c>
+      <c r="E573" t="str">
+        <v>Envoie l’e-mail tel qu’il est dans l’éditeur (même non enregistré), avec des données d’exemple. Le résultat est enregistré dans la Surveillance du système</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="str">
+        <v>The communication is saved when you send or schedule it</v>
+      </c>
+      <c r="B574" t="str">
+        <v>The communication is saved when you send or schedule it</v>
+      </c>
+      <c r="C574" t="str">
+        <v>A comunicação é guardada quando a enviar ou agendar</v>
+      </c>
+      <c r="D574" t="str">
+        <v>La comunicación se guarda al enviarla o programarla</v>
+      </c>
+      <c r="E574" t="str">
+        <v>La communication est enregistrée lorsque vous l’envoyez ou la planifiez</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="str">
+        <v>The selected file is not an image.</v>
+      </c>
+      <c r="B575" t="str">
+        <v>The selected file is not an image.</v>
+      </c>
+      <c r="C575" t="str">
+        <v>O ficheiro selecionado não é uma imagem.</v>
+      </c>
+      <c r="D575" t="str">
+        <v>El archivo seleccionado no es una imagen.</v>
+      </c>
+      <c r="E575" t="str">
+        <v>Le fichier sélectionné n’est pas une image.</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="str">
+        <v>Search by file name...</v>
+      </c>
+      <c r="B576" t="str">
+        <v>Search by file name...</v>
+      </c>
+      <c r="C576" t="str">
+        <v>Pesquisar por nome do ficheiro...</v>
+      </c>
+      <c r="D576" t="str">
+        <v>Buscar por nombre de archivo...</v>
+      </c>
+      <c r="E576" t="str">
+        <v>Rechercher par nom de fichier...</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="str">
+        <v>Images</v>
+      </c>
+      <c r="B577" t="str">
+        <v>Images</v>
+      </c>
+      <c r="C577" t="str">
+        <v>Imagens</v>
+      </c>
+      <c r="D577" t="str">
+        <v>Imágenes</v>
+      </c>
+      <c r="E577" t="str">
+        <v>Images</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="str">
+        <v>Documents</v>
+      </c>
+      <c r="B578" t="str">
+        <v>Documents</v>
+      </c>
+      <c r="C578" t="str">
+        <v>Documentos</v>
+      </c>
+      <c r="D578" t="str">
+        <v>Documentos</v>
+      </c>
+      <c r="E578" t="str">
+        <v>Documents</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="str">
+        <v>Newest first</v>
+      </c>
+      <c r="B579" t="str">
+        <v>Newest first</v>
+      </c>
+      <c r="C579" t="str">
+        <v>Mais recentes primeiro</v>
+      </c>
+      <c r="D579" t="str">
+        <v>Más recientes primero</v>
+      </c>
+      <c r="E579" t="str">
+        <v>Plus récents d’abord</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="str">
+        <v>Oldest first</v>
+      </c>
+      <c r="B580" t="str">
+        <v>Oldest first</v>
+      </c>
+      <c r="C580" t="str">
+        <v>Mais antigos primeiro</v>
+      </c>
+      <c r="D580" t="str">
+        <v>Más antiguos primero</v>
+      </c>
+      <c r="E580" t="str">
+        <v>Plus anciens d’abord</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="str">
+        <v>Name (A-Z)</v>
+      </c>
+      <c r="B581" t="str">
+        <v>Name (A-Z)</v>
+      </c>
+      <c r="C581" t="str">
+        <v>Nome (A-Z)</v>
+      </c>
+      <c r="D581" t="str">
+        <v>Nombre (A-Z)</v>
+      </c>
+      <c r="E581" t="str">
+        <v>Nom (A-Z)</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="str">
+        <v>Upload</v>
+      </c>
+      <c r="B582" t="str">
+        <v>Upload</v>
+      </c>
+      <c r="C582" t="str">
+        <v>Carregar</v>
+      </c>
+      <c r="D582" t="str">
+        <v>Subir</v>
+      </c>
+      <c r="E582" t="str">
+        <v>Téléverser</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="str">
+        <v>Upload files</v>
+      </c>
+      <c r="B583" t="str">
+        <v>Upload files</v>
+      </c>
+      <c r="C583" t="str">
+        <v>Carregar ficheiros</v>
+      </c>
+      <c r="D583" t="str">
+        <v>Subir archivos</v>
+      </c>
+      <c r="E583" t="str">
+        <v>Téléverser des fichiers</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="str">
+        <v>Uploading</v>
+      </c>
+      <c r="B584" t="str">
+        <v>Uploading</v>
+      </c>
+      <c r="C584" t="str">
+        <v>A carregar</v>
+      </c>
+      <c r="D584" t="str">
+        <v>Subiendo</v>
+      </c>
+      <c r="E584" t="str">
+        <v>Téléversement</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="str">
+        <v>Preview</v>
+      </c>
+      <c r="B585" t="str">
+        <v>Preview</v>
+      </c>
+      <c r="C585" t="str">
+        <v>Pré-visualizar</v>
+      </c>
+      <c r="D585" t="str">
+        <v>Previsualizar</v>
+      </c>
+      <c r="E585" t="str">
+        <v>Aperçu</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="str">
+        <v>The library has no files yet</v>
+      </c>
+      <c r="B586" t="str">
+        <v>The library has no files yet</v>
+      </c>
+      <c r="C586" t="str">
+        <v>A biblioteca ainda não tem ficheiros</v>
+      </c>
+      <c r="D586" t="str">
+        <v>La biblioteca aún no tiene archivos</v>
+      </c>
+      <c r="E586" t="str">
+        <v>La bibliothèque ne contient encore aucun fichier</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="str">
+        <v>No files match your search</v>
+      </c>
+      <c r="B587" t="str">
+        <v>No files match your search</v>
+      </c>
+      <c r="C587" t="str">
+        <v>Nenhum ficheiro corresponde à pesquisa</v>
+      </c>
+      <c r="D587" t="str">
+        <v>Ningún archivo coincide con la búsqueda</v>
+      </c>
+      <c r="E587" t="str">
+        <v>Aucun fichier ne correspond à la recherche</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="str">
+        <v>Select a file. Double click to choose it right away</v>
+      </c>
+      <c r="B588" t="str">
+        <v>Select a file. Double click to choose it right away</v>
+      </c>
+      <c r="C588" t="str">
+        <v>Selecione um ficheiro. Duplo clique para o escolher logo</v>
+      </c>
+      <c r="D588" t="str">
+        <v>Seleccione un archivo. Doble clic para elegirlo al instante</v>
+      </c>
+      <c r="E588" t="str">
+        <v>Sélectionnez un fichier. Double-cliquez pour le choisir directement</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="str">
+        <v>Choose</v>
+      </c>
+      <c r="B589" t="str">
+        <v>Choose</v>
+      </c>
+      <c r="C589" t="str">
+        <v>Escolher</v>
+      </c>
+      <c r="D589" t="str">
+        <v>Elegir</v>
+      </c>
+      <c r="E589" t="str">
+        <v>Choisir</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="str">
+        <v>Cancel</v>
+      </c>
+      <c r="B590" t="str">
+        <v>Cancel</v>
+      </c>
+      <c r="C590" t="str">
+        <v>Cancelar</v>
+      </c>
+      <c r="D590" t="str">
+        <v>Cancelar</v>
+      </c>
+      <c r="E590" t="str">
+        <v>Annuler</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="str">
+        <v>Drop the files to upload them</v>
+      </c>
+      <c r="B591" t="str">
+        <v>Drop the files to upload them</v>
+      </c>
+      <c r="C591" t="str">
+        <v>Largue os ficheiros para os carregar</v>
+      </c>
+      <c r="D591" t="str">
+        <v>Suelte los archivos para subirlos</v>
+      </c>
+      <c r="E591" t="str">
+        <v>Déposez les fichiers pour les téléverser</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="str">
+        <v>File uploaded successfully.</v>
+      </c>
+      <c r="B592" t="str">
+        <v>File uploaded successfully.</v>
+      </c>
+      <c r="C592" t="str">
+        <v>Ficheiro carregado com sucesso.</v>
+      </c>
+      <c r="D592" t="str">
+        <v>Archivo subido correctamente.</v>
+      </c>
+      <c r="E592" t="str">
+        <v>Fichier téléversé avec succès.</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="str">
+        <v>{{count}} files uploaded successfully.</v>
+      </c>
+      <c r="B593" t="str">
+        <v>{{count}} files uploaded successfully.</v>
+      </c>
+      <c r="C593" t="str">
+        <v>{{count}} ficheiros carregados com sucesso.</v>
+      </c>
+      <c r="D593" t="str">
+        <v>{{count}} archivos subidos correctamente.</v>
+      </c>
+      <c r="E593" t="str">
+        <v>{{count}} fichiers téléversés avec succès.</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="str">
+        <v>The upload failed</v>
+      </c>
+      <c r="B594" t="str">
+        <v>The upload failed</v>
+      </c>
+      <c r="C594" t="str">
+        <v>O carregamento falhou</v>
+      </c>
+      <c r="D594" t="str">
+        <v>La subida falló</v>
+      </c>
+      <c r="E594" t="str">
+        <v>Le téléversement a échoué</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="str">
+        <v>Computer</v>
+      </c>
+      <c r="B595" t="str">
+        <v>Computer</v>
+      </c>
+      <c r="C595" t="str">
+        <v>Computador</v>
+      </c>
+      <c r="D595" t="str">
+        <v>Ordenador</v>
+      </c>
+      <c r="E595" t="str">
+        <v>Ordinateur</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="str">
+        <v>Mobile</v>
+      </c>
+      <c r="B596" t="str">
+        <v>Mobile</v>
+      </c>
+      <c r="C596" t="str">
+        <v>Telemóvel</v>
+      </c>
+      <c r="D596" t="str">
+        <v>Móvil</v>
+      </c>
+      <c r="E596" t="str">
+        <v>Mobile</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="str">
+        <v>Edit content</v>
+      </c>
+      <c r="B597" t="str">
+        <v>Edit content</v>
+      </c>
+      <c r="C597" t="str">
+        <v>Editar conteúdo</v>
+      </c>
+      <c r="D597" t="str">
+        <v>Editar contenido</v>
+      </c>
+      <c r="E597" t="str">
+        <v>Modifier le contenu</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="str">
+        <v>This e-mail has no content yet</v>
+      </c>
+      <c r="B598" t="str">
+        <v>This e-mail has no content yet</v>
+      </c>
+      <c r="C598" t="str">
+        <v>Este e-mail ainda não tem conteúdo</v>
+      </c>
+      <c r="D598" t="str">
+        <v>Este correo aún no tiene contenido</v>
+      </c>
+      <c r="E598" t="str">
+        <v>Cet e-mail n’a pas encore de contenu</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="str">
+        <v>Content saved</v>
+      </c>
+      <c r="B599" t="str">
+        <v>Content saved</v>
+      </c>
+      <c r="C599" t="str">
+        <v>Conteúdo guardado</v>
+      </c>
+      <c r="D599" t="str">
+        <v>Contenido guardado</v>
+      </c>
+      <c r="E599" t="str">
+        <v>Contenu enregistré</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="str">
+        <v>Save and close</v>
+      </c>
+      <c r="B600" t="str">
+        <v>Save and close</v>
+      </c>
+      <c r="C600" t="str">
+        <v>Guardar e fechar</v>
+      </c>
+      <c r="D600" t="str">
+        <v>Guardar y cerrar</v>
+      </c>
+      <c r="E600" t="str">
+        <v>Enregistrer et fermer</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="str">
+        <v>Leave without saving?</v>
+      </c>
+      <c r="B601" t="str">
+        <v>Leave without saving?</v>
+      </c>
+      <c r="C601" t="str">
+        <v>Sair sem guardar?</v>
+      </c>
+      <c r="D601" t="str">
+        <v>¿Salir sin guardar?</v>
+      </c>
+      <c r="E601" t="str">
+        <v>Quitter sans enregistrer ?</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="str">
+        <v>The changes made to the content will be lost</v>
+      </c>
+      <c r="B602" t="str">
+        <v>The changes made to the content will be lost</v>
+      </c>
+      <c r="C602" t="str">
+        <v>As alterações feitas ao conteúdo serão perdidas</v>
+      </c>
+      <c r="D602" t="str">
+        <v>Los cambios realizados en el contenido se perderán</v>
+      </c>
+      <c r="E602" t="str">
+        <v>Les modifications apportées au contenu seront perdues</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="str">
+        <v>Leave</v>
+      </c>
+      <c r="B603" t="str">
+        <v>Leave</v>
+      </c>
+      <c r="C603" t="str">
+        <v>Sair</v>
+      </c>
+      <c r="D603" t="str">
+        <v>Salir</v>
+      </c>
+      <c r="E603" t="str">
+        <v>Quitter</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="str">
+        <v>Stay</v>
+      </c>
+      <c r="B604" t="str">
+        <v>Stay</v>
+      </c>
+      <c r="C604" t="str">
+        <v>Ficar</v>
+      </c>
+      <c r="D604" t="str">
+        <v>Quedarse</v>
+      </c>
+      <c r="E604" t="str">
+        <v>Rester</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="str">
+        <v>How the saved e-mail looks, with example data</v>
+      </c>
+      <c r="B605" t="str">
+        <v>How the saved e-mail looks, with example data</v>
+      </c>
+      <c r="C605" t="str">
+        <v>Como fica o e-mail guardado, com dados de exemplo</v>
+      </c>
+      <c r="D605" t="str">
+        <v>Cómo queda el correo guardado, con datos de ejemplo</v>
+      </c>
+      <c r="E605" t="str">
+        <v>Aperçu de l’e-mail enregistré, avec des données d’exemple</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="str">
+        <v>Sends the saved template to an address, with example data. The result is recorded in System monitoring</v>
+      </c>
+      <c r="B606" t="str">
+        <v>Sends the saved template to an address, with example data. The result is recorded in System monitoring</v>
+      </c>
+      <c r="C606" t="str">
+        <v>Envia o template guardado para um endereço, com dados de exemplo. O resultado fica registado na Monitorização do sistema</v>
+      </c>
+      <c r="D606" t="str">
+        <v>Envía la plantilla guardada a una dirección, con datos de ejemplo. El resultado queda registrado en la Monitorización del sistema</v>
+      </c>
+      <c r="E606" t="str">
+        <v>Envoie le modèle enregistré à une adresse, avec des données d’exemple. Le résultat est enregistré dans la Surveillance du système</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="str">
+        <v>Sends the saved e-mail to an address, with example data. The result is recorded in System monitoring</v>
+      </c>
+      <c r="B607" t="str">
+        <v>Sends the saved e-mail to an address, with example data. The result is recorded in System monitoring</v>
+      </c>
+      <c r="C607" t="str">
+        <v>Envia o e-mail guardado para um endereço, com dados de exemplo. O resultado fica registado na Monitorização do sistema</v>
+      </c>
+      <c r="D607" t="str">
+        <v>Envía el correo guardado a una dirección, con datos de ejemplo. El resultado queda registrado en la Monitorización del sistema</v>
+      </c>
+      <c r="E607" t="str">
+        <v>Envoie l’e-mail enregistré à une adresse, avec des données d’exemple. Le résultat est enregistré dans la Surveillance du système</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="str">
+        <v>HTML</v>
+      </c>
+      <c r="B608" t="str">
+        <v>HTML</v>
+      </c>
+      <c r="C608" t="str">
+        <v>HTML</v>
+      </c>
+      <c r="D608" t="str">
+        <v>HTML</v>
+      </c>
+      <c r="E608" t="str">
+        <v>HTML</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="str">
+        <v>Edit HTML</v>
+      </c>
+      <c r="B609" t="str">
+        <v>Edit HTML</v>
+      </c>
+      <c r="C609" t="str">
+        <v>Editar HTML</v>
+      </c>
+      <c r="D609" t="str">
+        <v>Editar HTML</v>
+      </c>
+      <c r="E609" t="str">
+        <v>Modifier le HTML</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="str">
+        <v>Your HTML here</v>
+      </c>
+      <c r="B610" t="str">
+        <v>Your HTML here</v>
+      </c>
+      <c r="C610" t="str">
+        <v>O seu HTML aqui</v>
+      </c>
+      <c r="D610" t="str">
+        <v>Su HTML aquí</v>
+      </c>
+      <c r="E610" t="str">
+        <v>Votre HTML ici</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="str">
+        <v>Write the HTML of this block. E-mail clients ignore scripts and most CSS, so use inline styles and simple tables</v>
+      </c>
+      <c r="B611" t="str">
+        <v>Write the HTML of this block. E-mail clients ignore scripts and most CSS, so use inline styles and simple tables</v>
+      </c>
+      <c r="C611" t="str">
+        <v>Escreva o HTML deste bloco. Os clientes de e-mail ignoram scripts e quase todo o CSS, por isso use estilos em linha e tabelas simples</v>
+      </c>
+      <c r="D611" t="str">
+        <v>Escriba el HTML de este bloque. Los clientes de correo ignoran los scripts y la mayoría del CSS, así que use estilos en línea y tablas simples</v>
+      </c>
+      <c r="E611" t="str">
+        <v>Écrivez le HTML de ce bloc. Les clients de messagerie ignorent les scripts et la plupart du CSS : utilisez des styles en ligne et des tableaux simples</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="str">
+        <v>Narrow + wide</v>
+      </c>
+      <c r="B612" t="str">
+        <v>Narrow + wide</v>
+      </c>
+      <c r="C612" t="str">
+        <v>Estreita + larga</v>
+      </c>
+      <c r="D612" t="str">
+        <v>Estrecha + ancha</v>
+      </c>
+      <c r="E612" t="str">
+        <v>Étroite + large</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="str">
+        <v>Side by side on mobile</v>
+      </c>
+      <c r="B613" t="str">
+        <v>Side by side on mobile</v>
+      </c>
+      <c r="C613" t="str">
+        <v>Lado a lado no telemóvel</v>
+      </c>
+      <c r="D613" t="str">
+        <v>Lado a lado en el móvil</v>
+      </c>
+      <c r="E613" t="str">
+        <v>Côte à côte sur mobile</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="str">
+        <v>List</v>
+      </c>
+      <c r="B614" t="str">
+        <v>List</v>
+      </c>
+      <c r="C614" t="str">
+        <v>Lista</v>
+      </c>
+      <c r="D614" t="str">
+        <v>Lista</v>
+      </c>
+      <c r="E614" t="str">
+        <v>Liste</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="str">
+        <v>First item</v>
+      </c>
+      <c r="B615" t="str">
+        <v>First item</v>
+      </c>
+      <c r="C615" t="str">
+        <v>Primeiro item</v>
+      </c>
+      <c r="D615" t="str">
+        <v>Primer elemento</v>
+      </c>
+      <c r="E615" t="str">
+        <v>Premier élément</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="str">
+        <v>Second item</v>
+      </c>
+      <c r="B616" t="str">
+        <v>Second item</v>
+      </c>
+      <c r="C616" t="str">
+        <v>Segundo item</v>
+      </c>
+      <c r="D616" t="str">
+        <v>Segundo elemento</v>
+      </c>
+      <c r="E616" t="str">
+        <v>Deuxième élément</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="str">
+        <v>Third item</v>
+      </c>
+      <c r="B617" t="str">
+        <v>Third item</v>
+      </c>
+      <c r="C617" t="str">
+        <v>Terceiro item</v>
+      </c>
+      <c r="D617" t="str">
+        <v>Tercer elemento</v>
+      </c>
+      <c r="E617" t="str">
+        <v>Troisième élément</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="str">
+        <v>Table</v>
+      </c>
+      <c r="B618" t="str">
+        <v>Table</v>
+      </c>
+      <c r="C618" t="str">
+        <v>Tabela</v>
+      </c>
+      <c r="D618" t="str">
+        <v>Tabla</v>
+      </c>
+      <c r="E618" t="str">
+        <v>Tableau</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="str">
+        <v>Item</v>
+      </c>
+      <c r="B619" t="str">
+        <v>Item</v>
+      </c>
+      <c r="C619" t="str">
+        <v>Item</v>
+      </c>
+      <c r="D619" t="str">
+        <v>Elemento</v>
+      </c>
+      <c r="E619" t="str">
+        <v>Élément</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="str">
+        <v>Value</v>
+      </c>
+      <c r="B620" t="str">
+        <v>Value</v>
+      </c>
+      <c r="C620" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="D620" t="str">
+        <v>Valor</v>
+      </c>
+      <c r="E620" t="str">
+        <v>Valeur</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="str">
+        <v>Menu</v>
+      </c>
+      <c r="B621" t="str">
+        <v>Menu</v>
+      </c>
+      <c r="C621" t="str">
+        <v>Menu</v>
+      </c>
+      <c r="D621" t="str">
+        <v>Menú</v>
+      </c>
+      <c r="E621" t="str">
+        <v>Menu</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="str">
+        <v>Link</v>
+      </c>
+      <c r="B622" t="str">
+        <v>Link</v>
+      </c>
+      <c r="C622" t="str">
+        <v>Ligação</v>
+      </c>
+      <c r="D622" t="str">
+        <v>Enlace</v>
+      </c>
+      <c r="E622" t="str">
+        <v>Lien</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="str">
+        <v>Banner with image</v>
+      </c>
+      <c r="B623" t="str">
+        <v>Banner with image</v>
+      </c>
+      <c r="C623" t="str">
+        <v>Banner com imagem</v>
+      </c>
+      <c r="D623" t="str">
+        <v>Banner con imagen</v>
+      </c>
+      <c r="E623" t="str">
+        <v>Bannière avec image</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="str">
+        <v>Call to action</v>
+      </c>
+      <c r="B624" t="str">
+        <v>Call to action</v>
+      </c>
+      <c r="C624" t="str">
+        <v>Chamada à ação</v>
+      </c>
+      <c r="D624" t="str">
+        <v>Llamada a la acción</v>
+      </c>
+      <c r="E624" t="str">
+        <v>Appel à l’action</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="str">
+        <v>Two images</v>
+      </c>
+      <c r="B625" t="str">
+        <v>Two images</v>
+      </c>
+      <c r="C625" t="str">
+        <v>Duas imagens</v>
+      </c>
+      <c r="D625" t="str">
+        <v>Dos imágenes</v>
+      </c>
+      <c r="E625" t="str">
+        <v>Deux images</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="str">
+        <v>Quote</v>
+      </c>
+      <c r="B626" t="str">
+        <v>Quote</v>
+      </c>
+      <c r="C626" t="str">
+        <v>Citação</v>
+      </c>
+      <c r="D626" t="str">
+        <v>Cita</v>
+      </c>
+      <c r="E626" t="str">
+        <v>Citation</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="str">
+        <v>Write the quote here</v>
+      </c>
+      <c r="B627" t="str">
+        <v>Write the quote here</v>
+      </c>
+      <c r="C627" t="str">
+        <v>Escreva aqui a citação</v>
+      </c>
+      <c r="D627" t="str">
+        <v>Escriba aquí la cita</v>
+      </c>
+      <c r="E627" t="str">
+        <v>Écrivez la citation ici</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="str">
+        <v>Signature</v>
+      </c>
+      <c r="B628" t="str">
+        <v>Signature</v>
+      </c>
+      <c r="C628" t="str">
+        <v>Assinatura</v>
+      </c>
+      <c r="D628" t="str">
+        <v>Firma</v>
+      </c>
+      <c r="E628" t="str">
+        <v>Signature</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="str">
+        <v>Best regards</v>
+      </c>
+      <c r="B629" t="str">
+        <v>Best regards</v>
+      </c>
+      <c r="C629" t="str">
+        <v>Com os melhores cumprimentos</v>
+      </c>
+      <c r="D629" t="str">
+        <v>Atentamente</v>
+      </c>
+      <c r="E629" t="str">
+        <v>Cordialement</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="str">
+        <v>The Bial Regional Academy team</v>
+      </c>
+      <c r="B630" t="str">
+        <v>The Bial Regional Academy team</v>
+      </c>
+      <c r="C630" t="str">
+        <v>A equipa da Bial Regional Academy</v>
+      </c>
+      <c r="D630" t="str">
+        <v>El equipo de Bial Regional Academy</v>
+      </c>
+      <c r="E630" t="str">
+        <v>L’équipe de Bial Regional Academy</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="str">
+        <v>Add a subject to send or schedule the communication</v>
+      </c>
+      <c r="B631" t="str">
+        <v>Add a subject to send or schedule the communication</v>
+      </c>
+      <c r="C631" t="str">
+        <v>Adicione um assunto para enviar ou agendar a comunicação</v>
+      </c>
+      <c r="D631" t="str">
+        <v>Añada un asunto para enviar o programar la comunicación</v>
+      </c>
+      <c r="E631" t="str">
+        <v>Ajoutez un objet pour envoyer ou planifier la communication</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="str">
+        <v>Add content to send or schedule the communication</v>
+      </c>
+      <c r="B632" t="str">
+        <v>Add content to send or schedule the communication</v>
+      </c>
+      <c r="C632" t="str">
+        <v>Adicione conteúdo para enviar ou agendar a comunicação</v>
+      </c>
+      <c r="D632" t="str">
+        <v>Añada contenido para enviar o programar la comunicación</v>
+      </c>
+      <c r="E632" t="str">
+        <v>Ajoutez du contenu pour envoyer ou planifier la communication</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="str">
+        <v>Required to send or schedule. You can use {{name}} to put each person's name</v>
+      </c>
+      <c r="B633" t="str">
+        <v>Required to send or schedule. You can use {{name}} to put each person's name</v>
+      </c>
+      <c r="C633" t="str">
+        <v>Obrigatório para enviar ou agendar. Pode usar {{name}} para pôr o nome de cada pessoa</v>
+      </c>
+      <c r="D633" t="str">
+        <v>Obligatorio para enviar o programar. Puede usar {{name}} para poner el nombre de cada persona</v>
+      </c>
+      <c r="E633" t="str">
+        <v>Obligatoire pour envoyer ou planifier. Vous pouvez utiliser {{name}} pour insérer le nom de chaque personne</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="str">
+        <v>Accepted by the mail server. It does not guarantee it reached the inbox</v>
+      </c>
+      <c r="B634" t="str">
+        <v>Accepted by the mail server. It does not guarantee it reached the inbox</v>
+      </c>
+      <c r="C634" t="str">
+        <v>Aceites pelo servidor de e-mail. Não garante que chegaram à caixa de entrada</v>
+      </c>
+      <c r="D634" t="str">
+        <v>Aceptados por el servidor de correo. No garantiza que llegaran a la bandeja de entrada</v>
+      </c>
+      <c r="E634" t="str">
+        <v>Acceptés par le serveur de messagerie. Cela ne garantit pas l’arrivée dans la boîte de réception</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="str">
+        <v>Opened</v>
+      </c>
+      <c r="B635" t="str">
+        <v>Opened</v>
+      </c>
+      <c r="C635" t="str">
+        <v>Abertos</v>
+      </c>
+      <c r="D635" t="str">
+        <v>Abiertos</v>
+      </c>
+      <c r="E635" t="str">
+        <v>Ouverts</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="str">
+        <v>Clicked</v>
+      </c>
+      <c r="B636" t="str">
+        <v>Clicked</v>
+      </c>
+      <c r="C636" t="str">
+        <v>Clicaram</v>
+      </c>
+      <c r="D636" t="str">
+        <v>Hicieron clic</v>
+      </c>
+      <c r="E636" t="str">
+        <v>Ont cliqué</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="str">
+        <v>Not opened</v>
+      </c>
+      <c r="B637" t="str">
+        <v>Not opened</v>
+      </c>
+      <c r="C637" t="str">
+        <v>Não abertos</v>
+      </c>
+      <c r="D637" t="str">
+        <v>No abiertos</v>
+      </c>
+      <c r="E637" t="str">
+        <v>Non ouverts</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="str">
+        <v>Opens and clicks</v>
+      </c>
+      <c r="B638" t="str">
+        <v>Opens and clicks</v>
+      </c>
+      <c r="C638" t="str">
+        <v>Aberturas e cliques</v>
+      </c>
+      <c r="D638" t="str">
+        <v>Aperturas y clics</v>
+      </c>
+      <c r="E638" t="str">
+        <v>Ouvertures et clics</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="str">
+        <v>People who opened it, out of the e-mails sent. It is approximate: some mail apps load images by themselves or block them</v>
+      </c>
+      <c r="B639" t="str">
+        <v>People who opened it, out of the e-mails sent. It is approximate: some mail apps load images by themselves or block them</v>
+      </c>
+      <c r="C639" t="str">
+        <v>Pessoas que o abriram, em relação aos e-mails enviados. É aproximado: há programas de e-mail que carregam as imagens sozinhos ou as bloqueiam</v>
+      </c>
+      <c r="D639" t="str">
+        <v>Personas que lo abrieron, sobre los correos enviados. Es aproximado: algunas aplicaciones de correo cargan las imágenes solas o las bloquean</v>
+      </c>
+      <c r="E639" t="str">
+        <v>Personnes l’ayant ouvert, par rapport aux e-mails envoyés. C’est approximatif : certaines applications de messagerie chargent les images seules ou les bloquent</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="str">
+        <v>People who clicked at least one link, out of the e-mails sent</v>
+      </c>
+      <c r="B640" t="str">
+        <v>People who clicked at least one link, out of the e-mails sent</v>
+      </c>
+      <c r="C640" t="str">
+        <v>Pessoas que clicaram em pelo menos um link, em relação aos e-mails enviados</v>
+      </c>
+      <c r="D640" t="str">
+        <v>Personas que hicieron clic en al menos un enlace, sobre los correos enviados</v>
+      </c>
+      <c r="E640" t="str">
+        <v>Personnes ayant cliqué sur au moins un lien, par rapport aux e-mails envoyés</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="str">
+        <v>Opens and clicks are not tracked for this communication</v>
+      </c>
+      <c r="B641" t="str">
+        <v>Opens and clicks are not tracked for this communication</v>
+      </c>
+      <c r="C641" t="str">
+        <v>As aberturas e os cliques não são rastreados nesta comunicação</v>
+      </c>
+      <c r="D641" t="str">
+        <v>Las aperturas y los clics no se rastrean en esta comunicación</v>
+      </c>
+      <c r="E641" t="str">
+        <v>Les ouvertures et les clics ne sont pas suivis pour cette communication</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="str">
+        <v>Most clicked links</v>
+      </c>
+      <c r="B642" t="str">
+        <v>Most clicked links</v>
+      </c>
+      <c r="C642" t="str">
+        <v>Links mais clicados</v>
+      </c>
+      <c r="D642" t="str">
+        <v>Enlaces más clicados</v>
+      </c>
+      <c r="E642" t="str">
+        <v>Liens les plus cliqués</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="str">
+        <v>People</v>
+      </c>
+      <c r="B643" t="str">
+        <v>People</v>
+      </c>
+      <c r="C643" t="str">
+        <v>Pessoas</v>
+      </c>
+      <c r="D643" t="str">
+        <v>Personas</v>
+      </c>
+      <c r="E643" t="str">
+        <v>Personnes</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="str">
+        <v>Clicks</v>
+      </c>
+      <c r="B644" t="str">
+        <v>Clicks</v>
+      </c>
+      <c r="C644" t="str">
+        <v>Cliques</v>
+      </c>
+      <c r="D644" t="str">
+        <v>Clics</v>
+      </c>
+      <c r="E644" t="str">
+        <v>Clics</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="str">
+        <v>Track opens and clicks</v>
+      </c>
+      <c r="B645" t="str">
+        <v>Track opens and clicks</v>
+      </c>
+      <c r="C645" t="str">
+        <v>Rastrear aberturas e cliques</v>
+      </c>
+      <c r="D645" t="str">
+        <v>Rastrear aperturas y clics</v>
+      </c>
+      <c r="E645" t="str">
+        <v>Suivre les ouvertures et les clics</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="str">
+        <v>Shows who opened the e-mail and clicked its links. Adds an invisible image and passes the links through the platform</v>
+      </c>
+      <c r="B646" t="str">
+        <v>Shows who opened the e-mail and clicked its links. Adds an invisible image and passes the links through the platform</v>
+      </c>
+      <c r="C646" t="str">
+        <v>Mostra quem abriu o e-mail e clicou nos links. Acrescenta uma imagem invisível e faz os links passar pela plataforma</v>
+      </c>
+      <c r="D646" t="str">
+        <v>Muestra quién abrió el correo y hizo clic en sus enlaces. Añade una imagen invisible y hace pasar los enlaces por la plataforma</v>
+      </c>
+      <c r="E646" t="str">
+        <v>Montre qui a ouvert l’e-mail et cliqué sur ses liens. Ajoute une image invisible et fait passer les liens par la plateforme</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="str">
+        <v>Export</v>
+      </c>
+      <c r="B647" t="str">
+        <v>Export</v>
+      </c>
+      <c r="C647" t="str">
+        <v>Exportar</v>
+      </c>
+      <c r="D647" t="str">
+        <v>Exportar</v>
+      </c>
+      <c r="E647" t="str">
+        <v>Exporter</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="str">
+        <v>Track clicks</v>
+      </c>
+      <c r="B648" t="str">
+        <v>Track clicks</v>
+      </c>
+      <c r="C648" t="str">
+        <v>Rastrear cliques</v>
+      </c>
+      <c r="D648" t="str">
+        <v>Rastrear clics</v>
+      </c>
+      <c r="E648" t="str">
+        <v>Suivre les clics</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="str">
+        <v>Shows who clicked the links. The links pass through the platform before opening the original address</v>
+      </c>
+      <c r="B649" t="str">
+        <v>Shows who clicked the links. The links pass through the platform before opening the original address</v>
+      </c>
+      <c r="C649" t="str">
+        <v>Mostra quem clicou nos links. Os links passam pela plataforma antes de abrir o endereço original</v>
+      </c>
+      <c r="D649" t="str">
+        <v>Muestra quién hizo clic en los enlaces. Los enlaces pasan por la plataforma antes de abrir la dirección original</v>
+      </c>
+      <c r="E649" t="str">
+        <v>Montre qui a cliqué sur les liens. Les liens passent par la plateforme avant d’ouvrir l’adresse d’origine</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="str">
+        <v>Not clicked</v>
+      </c>
+      <c r="B650" t="str">
+        <v>Not clicked</v>
+      </c>
+      <c r="C650" t="str">
+        <v>Não clicaram</v>
+      </c>
+      <c r="D650" t="str">
+        <v>No hicieron clic</v>
+      </c>
+      <c r="E650" t="str">
+        <v>N’ont pas cliqué</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="str">
+        <v>Clicks are not tracked for this communication</v>
+      </c>
+      <c r="B651" t="str">
+        <v>Clicks are not tracked for this communication</v>
+      </c>
+      <c r="C651" t="str">
+        <v>Os cliques não são rastreados nesta comunicação</v>
+      </c>
+      <c r="D651" t="str">
+        <v>Los clics no se rastrean en esta comunicación</v>
+      </c>
+      <c r="E651" t="str">
+        <v>Les clics ne sont pas suivis pour cette communication</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E481"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E651"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: shared config, endpoints, translations source and deploy notes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E651"/>
+  <dimension ref="A1:E892"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11466,9 +11466,4106 @@
         <v>Les clics ne sont pas suivis pour cette communication</v>
       </c>
     </row>
+    <row r="652">
+      <c r="A652" t="str">
+        <v>Start from a template</v>
+      </c>
+      <c r="B652" t="str">
+        <v>Start from a template</v>
+      </c>
+      <c r="C652" t="str">
+        <v>Começar a partir de um modelo</v>
+      </c>
+      <c r="D652" t="str">
+        <v>Empezar desde una plantilla</v>
+      </c>
+      <c r="E652" t="str">
+        <v>Commencer à partir d’un modèle</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="str">
+        <v>Templates and saved blocks</v>
+      </c>
+      <c r="B653" t="str">
+        <v>Templates and saved blocks</v>
+      </c>
+      <c r="C653" t="str">
+        <v>Modelos e blocos guardados</v>
+      </c>
+      <c r="D653" t="str">
+        <v>Plantillas y bloques guardados</v>
+      </c>
+      <c r="E653" t="str">
+        <v>Modèles et blocs enregistrés</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="str">
+        <v>Choose a ready-made e-mail to start from, or close this window to start from the basic one. You can change everything afterwards</v>
+      </c>
+      <c r="B654" t="str">
+        <v>Choose a ready-made e-mail to start from, or close this window to start from the basic one. You can change everything afterwards</v>
+      </c>
+      <c r="C654" t="str">
+        <v>Escolha um e-mail pronto para começar, ou feche esta janela para começar pelo modelo base. Pode alterar tudo depois</v>
+      </c>
+      <c r="D654" t="str">
+        <v>Elija un correo ya hecho para empezar, o cierre esta ventana para empezar con el básico. Puede cambiarlo todo después</v>
+      </c>
+      <c r="E654" t="str">
+        <v>Choisissez un e-mail prêt à l’emploi pour commencer, ou fermez cette fenêtre pour partir du modèle de base. Vous pourrez tout modifier ensuite</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="str">
+        <v>Gallery</v>
+      </c>
+      <c r="B655" t="str">
+        <v>Gallery</v>
+      </c>
+      <c r="C655" t="str">
+        <v>Galeria</v>
+      </c>
+      <c r="D655" t="str">
+        <v>Galería</v>
+      </c>
+      <c r="E655" t="str">
+        <v>Galerie</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="str">
+        <v>Team templates</v>
+      </c>
+      <c r="B656" t="str">
+        <v>Team templates</v>
+      </c>
+      <c r="C656" t="str">
+        <v>Modelos da equipa</v>
+      </c>
+      <c r="D656" t="str">
+        <v>Plantillas del equipo</v>
+      </c>
+      <c r="E656" t="str">
+        <v>Modèles de l’équipe</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="str">
+        <v>Saved blocks</v>
+      </c>
+      <c r="B657" t="str">
+        <v>Saved blocks</v>
+      </c>
+      <c r="C657" t="str">
+        <v>Blocos guardados</v>
+      </c>
+      <c r="D657" t="str">
+        <v>Bloques guardados</v>
+      </c>
+      <c r="E657" t="str">
+        <v>Blocs enregistrés</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="str">
+        <v>Use this template</v>
+      </c>
+      <c r="B658" t="str">
+        <v>Use this template</v>
+      </c>
+      <c r="C658" t="str">
+        <v>Usar este modelo</v>
+      </c>
+      <c r="D658" t="str">
+        <v>Usar esta plantilla</v>
+      </c>
+      <c r="E658" t="str">
+        <v>Utiliser ce modèle</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="str">
+        <v>The team library is not available yet</v>
+      </c>
+      <c r="B659" t="str">
+        <v>The team library is not available yet</v>
+      </c>
+      <c r="C659" t="str">
+        <v>A biblioteca da equipa ainda não está disponível</v>
+      </c>
+      <c r="D659" t="str">
+        <v>La biblioteca del equipo aún no está disponible</v>
+      </c>
+      <c r="E659" t="str">
+        <v>La bibliothèque de l’équipe n’est pas encore disponible</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="str">
+        <v>No templates saved by the team yet. Use "Save as template" in the editor toolbar</v>
+      </c>
+      <c r="B660" t="str">
+        <v>No templates saved by the team yet. Use "Save as template" in the editor toolbar</v>
+      </c>
+      <c r="C660" t="str">
+        <v>Ainda não há modelos guardados pela equipa. Use "Guardar como modelo" na barra do editor</v>
+      </c>
+      <c r="D660" t="str">
+        <v>Aún no hay plantillas guardadas por el equipo. Use "Guardar como plantilla" en la barra del editor</v>
+      </c>
+      <c r="E660" t="str">
+        <v>Aucun modèle enregistré par l’équipe pour l’instant. Utilisez "Enregistrer comme modèle" dans la barre de l’éditeur</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="str">
+        <v>No blocks saved yet. Select a section in the e-mail and use the bookmark button in its toolbar</v>
+      </c>
+      <c r="B661" t="str">
+        <v>No blocks saved yet. Select a section in the e-mail and use the bookmark button in its toolbar</v>
+      </c>
+      <c r="C661" t="str">
+        <v>Ainda não há blocos guardados. Selecione uma secção do e-mail e use o botão do marcador na sua barra</v>
+      </c>
+      <c r="D661" t="str">
+        <v>Aún no hay bloques guardados. Seleccione una sección del correo y use el botón del marcador en su barra</v>
+      </c>
+      <c r="E661" t="str">
+        <v>Aucun bloc enregistré pour l’instant. Sélectionnez une section de l’e-mail et utilisez le bouton marque-page de sa barre</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="str">
+        <v>Saved blocks appear in the blocks panel, in the "Saved blocks" group. Drag them into the e-mail</v>
+      </c>
+      <c r="B662" t="str">
+        <v>Saved blocks appear in the blocks panel, in the "Saved blocks" group. Drag them into the e-mail</v>
+      </c>
+      <c r="C662" t="str">
+        <v>Os blocos guardados aparecem no painel de blocos, no grupo "Blocos guardados". Arraste-os para o e-mail</v>
+      </c>
+      <c r="D662" t="str">
+        <v>Los bloques guardados aparecen en el panel de bloques, en el grupo "Bloques guardados". Arrástrelos al correo</v>
+      </c>
+      <c r="E662" t="str">
+        <v>Les blocs enregistrés apparaissent dans le panneau des blocs, dans le groupe "Blocs enregistrés". Faites-les glisser dans l’e-mail</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="str">
+        <v>Delete this item for the whole team?</v>
+      </c>
+      <c r="B663" t="str">
+        <v>Delete this item for the whole team?</v>
+      </c>
+      <c r="C663" t="str">
+        <v>Eliminar este item para toda a equipa?</v>
+      </c>
+      <c r="D663" t="str">
+        <v>¿Eliminar este elemento para todo el equipo?</v>
+      </c>
+      <c r="E663" t="str">
+        <v>Supprimer cet élément pour toute l’équipe ?</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="str">
+        <v>Deleted</v>
+      </c>
+      <c r="B664" t="str">
+        <v>Deleted</v>
+      </c>
+      <c r="C664" t="str">
+        <v>Eliminado</v>
+      </c>
+      <c r="D664" t="str">
+        <v>Eliminado</v>
+      </c>
+      <c r="E664" t="str">
+        <v>Supprimé</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="str">
+        <v>Rename</v>
+      </c>
+      <c r="B665" t="str">
+        <v>Rename</v>
+      </c>
+      <c r="C665" t="str">
+        <v>Mudar o nome</v>
+      </c>
+      <c r="D665" t="str">
+        <v>Cambiar el nombre</v>
+      </c>
+      <c r="E665" t="str">
+        <v>Renommer</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="str">
+        <v>Save as block</v>
+      </c>
+      <c r="B666" t="str">
+        <v>Save as block</v>
+      </c>
+      <c r="C666" t="str">
+        <v>Guardar como bloco</v>
+      </c>
+      <c r="D666" t="str">
+        <v>Guardar como bloque</v>
+      </c>
+      <c r="E666" t="str">
+        <v>Enregistrer comme bloc</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="str">
+        <v>Save as template</v>
+      </c>
+      <c r="B667" t="str">
+        <v>Save as template</v>
+      </c>
+      <c r="C667" t="str">
+        <v>Guardar como modelo</v>
+      </c>
+      <c r="D667" t="str">
+        <v>Guardar como plantilla</v>
+      </c>
+      <c r="E667" t="str">
+        <v>Enregistrer comme modèle</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="str">
+        <v>Block saved for the team</v>
+      </c>
+      <c r="B668" t="str">
+        <v>Block saved for the team</v>
+      </c>
+      <c r="C668" t="str">
+        <v>Bloco guardado para a equipa</v>
+      </c>
+      <c r="D668" t="str">
+        <v>Bloque guardado para el equipo</v>
+      </c>
+      <c r="E668" t="str">
+        <v>Bloc enregistré pour l’équipe</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="str">
+        <v>Template saved for the team</v>
+      </c>
+      <c r="B669" t="str">
+        <v>Template saved for the team</v>
+      </c>
+      <c r="C669" t="str">
+        <v>Modelo guardado para a equipa</v>
+      </c>
+      <c r="D669" t="str">
+        <v>Plantilla guardada para el equipo</v>
+      </c>
+      <c r="E669" t="str">
+        <v>Modèle enregistré pour l’équipe</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="str">
+        <v>The selected section becomes a block that the whole team can reuse in any e-mail</v>
+      </c>
+      <c r="B670" t="str">
+        <v>The selected section becomes a block that the whole team can reuse in any e-mail</v>
+      </c>
+      <c r="C670" t="str">
+        <v>A secção selecionada passa a ser um bloco que toda a equipa pode reutilizar em qualquer e-mail</v>
+      </c>
+      <c r="D670" t="str">
+        <v>La sección seleccionada pasa a ser un bloque que todo el equipo puede reutilizar en cualquier correo</v>
+      </c>
+      <c r="E670" t="str">
+        <v>La section sélectionnée devient un bloc que toute l’équipe peut réutiliser dans n’importe quel e-mail</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="str">
+        <v>The e-mail as it is now becomes a template that the whole team can start from</v>
+      </c>
+      <c r="B671" t="str">
+        <v>The e-mail as it is now becomes a template that the whole team can start from</v>
+      </c>
+      <c r="C671" t="str">
+        <v>O e-mail tal como está agora passa a ser um modelo a partir do qual toda a equipa pode começar</v>
+      </c>
+      <c r="D671" t="str">
+        <v>El correo tal como está ahora pasa a ser una plantilla desde la que todo el equipo puede empezar</v>
+      </c>
+      <c r="E671" t="str">
+        <v>L’e-mail tel qu’il est maintenant devient un modèle dont toute l’équipe peut partir</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="str">
+        <v>Replace the current content?</v>
+      </c>
+      <c r="B672" t="str">
+        <v>Replace the current content?</v>
+      </c>
+      <c r="C672" t="str">
+        <v>Substituir o conteúdo atual?</v>
+      </c>
+      <c r="D672" t="str">
+        <v>¿Reemplazar el contenido actual?</v>
+      </c>
+      <c r="E672" t="str">
+        <v>Remplacer le contenu actuel ?</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="str">
+        <v>The e-mail you are editing is replaced by this template. You can undo it with Ctrl+Z</v>
+      </c>
+      <c r="B673" t="str">
+        <v>The e-mail you are editing is replaced by this template. You can undo it with Ctrl+Z</v>
+      </c>
+      <c r="C673" t="str">
+        <v>O e-mail que está a editar é substituído por este modelo. Pode desfazer com Ctrl+Z</v>
+      </c>
+      <c r="D673" t="str">
+        <v>El correo que está editando se reemplaza por esta plantilla. Puede deshacerlo con Ctrl+Z</v>
+      </c>
+      <c r="E673" t="str">
+        <v>L’e-mail en cours de modification est remplacé par ce modèle. Vous pouvez annuler avec Ctrl+Z</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="str">
+        <v>Welcome</v>
+      </c>
+      <c r="B674" t="str">
+        <v>Welcome</v>
+      </c>
+      <c r="C674" t="str">
+        <v>Bem-vindo</v>
+      </c>
+      <c r="D674" t="str">
+        <v>Bienvenida</v>
+      </c>
+      <c r="E674" t="str">
+        <v>Bienvenue</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="str">
+        <v>Welcomes a person to the Academy with a button to access it</v>
+      </c>
+      <c r="B675" t="str">
+        <v>Welcomes a person to the Academy with a button to access it</v>
+      </c>
+      <c r="C675" t="str">
+        <v>Dá as boas-vindas à Academy com um botão para aceder</v>
+      </c>
+      <c r="D675" t="str">
+        <v>Da la bienvenida a la Academy con un botón para acceder</v>
+      </c>
+      <c r="E675" t="str">
+        <v>Accueille une personne à l’Academy avec un bouton d’accès</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="str">
+        <v>Welcome to the Academy</v>
+      </c>
+      <c r="B676" t="str">
+        <v>Welcome to the Academy</v>
+      </c>
+      <c r="C676" t="str">
+        <v>Bem-vindo à Academy</v>
+      </c>
+      <c r="D676" t="str">
+        <v>Bienvenido a la Academy</v>
+      </c>
+      <c r="E676" t="str">
+        <v>Bienvenue à l’Academy</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="str">
+        <v>Training made for you, wherever you are</v>
+      </c>
+      <c r="B677" t="str">
+        <v>Training made for you, wherever you are</v>
+      </c>
+      <c r="C677" t="str">
+        <v>Formação feita para si, onde quer que esteja</v>
+      </c>
+      <c r="D677" t="str">
+        <v>Formación hecha para usted, esté donde esté</v>
+      </c>
+      <c r="E677" t="str">
+        <v>Une formation faite pour vous, où que vous soyez</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="str">
+        <v>Your account is ready. Access the platform to see the courses available for you.</v>
+      </c>
+      <c r="B678" t="str">
+        <v>Your account is ready. Access the platform to see the courses available for you.</v>
+      </c>
+      <c r="C678" t="str">
+        <v>A sua conta está pronta. Aceda à plataforma para ver os cursos disponíveis para si.</v>
+      </c>
+      <c r="D678" t="str">
+        <v>Su cuenta está lista. Acceda a la plataforma para ver los cursos disponibles para usted.</v>
+      </c>
+      <c r="E678" t="str">
+        <v>Votre compte est prêt. Accédez à la plateforme pour voir les cours disponibles pour vous.</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="str">
+        <v>Access the platform</v>
+      </c>
+      <c r="B679" t="str">
+        <v>Access the platform</v>
+      </c>
+      <c r="C679" t="str">
+        <v>Aceder à plataforma</v>
+      </c>
+      <c r="D679" t="str">
+        <v>Acceder a la plataforma</v>
+      </c>
+      <c r="E679" t="str">
+        <v>Accéder à la plateforme</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="str">
+        <v>Newsletter</v>
+      </c>
+      <c r="B680" t="str">
+        <v>Newsletter</v>
+      </c>
+      <c r="C680" t="str">
+        <v>Newsletter</v>
+      </c>
+      <c r="D680" t="str">
+        <v>Boletín</v>
+      </c>
+      <c r="E680" t="str">
+        <v>Newsletter</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="str">
+        <v>A banner, two articles with image and a footer with social links</v>
+      </c>
+      <c r="B681" t="str">
+        <v>A banner, two articles with image and a footer with social links</v>
+      </c>
+      <c r="C681" t="str">
+        <v>Um banner, dois artigos com imagem e um rodapé com redes sociais</v>
+      </c>
+      <c r="D681" t="str">
+        <v>Un banner, dos artículos con imagen y un pie con redes sociales</v>
+      </c>
+      <c r="E681" t="str">
+        <v>Une bannière, deux articles avec image et un pied de page avec les réseaux sociaux</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="str">
+        <v>Newsletter title</v>
+      </c>
+      <c r="B682" t="str">
+        <v>Newsletter title</v>
+      </c>
+      <c r="C682" t="str">
+        <v>Título da newsletter</v>
+      </c>
+      <c r="D682" t="str">
+        <v>Título del boletín</v>
+      </c>
+      <c r="E682" t="str">
+        <v>Titre de la newsletter</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="str">
+        <v>here is what is new this month</v>
+      </c>
+      <c r="B683" t="str">
+        <v>here is what is new this month</v>
+      </c>
+      <c r="C683" t="str">
+        <v>eis as novidades deste mês</v>
+      </c>
+      <c r="D683" t="str">
+        <v>estas son las novedades de este mes</v>
+      </c>
+      <c r="E683" t="str">
+        <v>voici les nouveautés de ce mois-ci</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="str">
+        <v>First article</v>
+      </c>
+      <c r="B684" t="str">
+        <v>First article</v>
+      </c>
+      <c r="C684" t="str">
+        <v>Primeiro artigo</v>
+      </c>
+      <c r="D684" t="str">
+        <v>Primer artículo</v>
+      </c>
+      <c r="E684" t="str">
+        <v>Premier article</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="str">
+        <v>Second article</v>
+      </c>
+      <c r="B685" t="str">
+        <v>Second article</v>
+      </c>
+      <c r="C685" t="str">
+        <v>Segundo artigo</v>
+      </c>
+      <c r="D685" t="str">
+        <v>Segundo artículo</v>
+      </c>
+      <c r="E685" t="str">
+        <v>Deuxième article</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="str">
+        <v>Write a short summary of the article here.</v>
+      </c>
+      <c r="B686" t="str">
+        <v>Write a short summary of the article here.</v>
+      </c>
+      <c r="C686" t="str">
+        <v>Escreva aqui um pequeno resumo do artigo.</v>
+      </c>
+      <c r="D686" t="str">
+        <v>Escriba aquí un breve resumen del artículo.</v>
+      </c>
+      <c r="E686" t="str">
+        <v>Écrivez ici un court résumé de l’article.</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="str">
+        <v>New course</v>
+      </c>
+      <c r="B687" t="str">
+        <v>New course</v>
+      </c>
+      <c r="C687" t="str">
+        <v>Novo curso</v>
+      </c>
+      <c r="D687" t="str">
+        <v>Nuevo curso</v>
+      </c>
+      <c r="E687" t="str">
+        <v>Nouveau cours</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="str">
+        <v>Announces a course with its main details and a button to enrol</v>
+      </c>
+      <c r="B688" t="str">
+        <v>Announces a course with its main details and a button to enrol</v>
+      </c>
+      <c r="C688" t="str">
+        <v>Anuncia um curso com os dados principais e um botão para aceder</v>
+      </c>
+      <c r="D688" t="str">
+        <v>Anuncia un curso con sus datos principales y un botón para acceder</v>
+      </c>
+      <c r="E688" t="str">
+        <v>Annonce un cours avec ses informations principales et un bouton d’accès</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="str">
+        <v>New course available</v>
+      </c>
+      <c r="B689" t="str">
+        <v>New course available</v>
+      </c>
+      <c r="C689" t="str">
+        <v>Novo curso disponível</v>
+      </c>
+      <c r="D689" t="str">
+        <v>Nuevo curso disponible</v>
+      </c>
+      <c r="E689" t="str">
+        <v>Nouveau cours disponible</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="str">
+        <v>A new course is now available on the Academy.</v>
+      </c>
+      <c r="B690" t="str">
+        <v>A new course is now available on the Academy.</v>
+      </c>
+      <c r="C690" t="str">
+        <v>Está disponível um novo curso na Academy.</v>
+      </c>
+      <c r="D690" t="str">
+        <v>Hay un nuevo curso disponible en la Academy.</v>
+      </c>
+      <c r="E690" t="str">
+        <v>Un nouveau cours est disponible sur l’Academy.</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="str">
+        <v>Course</v>
+      </c>
+      <c r="B691" t="str">
+        <v>Course</v>
+      </c>
+      <c r="C691" t="str">
+        <v>Curso</v>
+      </c>
+      <c r="D691" t="str">
+        <v>Curso</v>
+      </c>
+      <c r="E691" t="str">
+        <v>Cours</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="str">
+        <v>Available from</v>
+      </c>
+      <c r="B692" t="str">
+        <v>Available from</v>
+      </c>
+      <c r="C692" t="str">
+        <v>Disponível a partir de</v>
+      </c>
+      <c r="D692" t="str">
+        <v>Disponible desde</v>
+      </c>
+      <c r="E692" t="str">
+        <v>Disponible à partir du</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="str">
+        <v>See the course</v>
+      </c>
+      <c r="B693" t="str">
+        <v>See the course</v>
+      </c>
+      <c r="C693" t="str">
+        <v>Ver o curso</v>
+      </c>
+      <c r="D693" t="str">
+        <v>Ver el curso</v>
+      </c>
+      <c r="E693" t="str">
+        <v>Voir le cours</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="str">
+        <v>Reminder</v>
+      </c>
+      <c r="B694" t="str">
+        <v>Reminder</v>
+      </c>
+      <c r="C694" t="str">
+        <v>Lembrete</v>
+      </c>
+      <c r="D694" t="str">
+        <v>Recordatorio</v>
+      </c>
+      <c r="E694" t="str">
+        <v>Rappel</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="str">
+        <v>A short reminder with a highlighted box and a button</v>
+      </c>
+      <c r="B695" t="str">
+        <v>A short reminder with a highlighted box and a button</v>
+      </c>
+      <c r="C695" t="str">
+        <v>Um lembrete curto com uma caixa em destaque e um botão</v>
+      </c>
+      <c r="D695" t="str">
+        <v>Un recordatorio corto con un recuadro destacado y un botón</v>
+      </c>
+      <c r="E695" t="str">
+        <v>Un court rappel avec un encadré mis en avant et un bouton</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="str">
+        <v>We would like to remind you of something important.</v>
+      </c>
+      <c r="B696" t="str">
+        <v>We would like to remind you of something important.</v>
+      </c>
+      <c r="C696" t="str">
+        <v>Gostaríamos de lhe recordar algo importante.</v>
+      </c>
+      <c r="D696" t="str">
+        <v>Nos gustaría recordarle algo importante.</v>
+      </c>
+      <c r="E696" t="str">
+        <v>Nous souhaitons vous rappeler quelque chose d’important.</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="str">
+        <v>Write the reminder here</v>
+      </c>
+      <c r="B697" t="str">
+        <v>Write the reminder here</v>
+      </c>
+      <c r="C697" t="str">
+        <v>Escreva aqui o lembrete</v>
+      </c>
+      <c r="D697" t="str">
+        <v>Escriba aquí el recordatorio</v>
+      </c>
+      <c r="E697" t="str">
+        <v>Écrivez ici le rappel</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="str">
+        <v>Announcement</v>
+      </c>
+      <c r="B698" t="str">
+        <v>Announcement</v>
+      </c>
+      <c r="C698" t="str">
+        <v>Anúncio</v>
+      </c>
+      <c r="D698" t="str">
+        <v>Anuncio</v>
+      </c>
+      <c r="E698" t="str">
+        <v>Annonce</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="str">
+        <v>A big title, an image, a text and a button</v>
+      </c>
+      <c r="B699" t="str">
+        <v>A big title, an image, a text and a button</v>
+      </c>
+      <c r="C699" t="str">
+        <v>Um título grande, uma imagem, um texto e um botão</v>
+      </c>
+      <c r="D699" t="str">
+        <v>Un título grande, una imagen, un texto y un botón</v>
+      </c>
+      <c r="E699" t="str">
+        <v>Un grand titre, une image, un texte et un bouton</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="str">
+        <v>Your announcement</v>
+      </c>
+      <c r="B700" t="str">
+        <v>Your announcement</v>
+      </c>
+      <c r="C700" t="str">
+        <v>O seu anúncio</v>
+      </c>
+      <c r="D700" t="str">
+        <v>Su anuncio</v>
+      </c>
+      <c r="E700" t="str">
+        <v>Votre annonce</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="str">
+        <v>Read more</v>
+      </c>
+      <c r="B701" t="str">
+        <v>Read more</v>
+      </c>
+      <c r="C701" t="str">
+        <v>Ler mais</v>
+      </c>
+      <c r="D701" t="str">
+        <v>Leer más</v>
+      </c>
+      <c r="E701" t="str">
+        <v>En savoir plus</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="str">
+        <v>Event invitation</v>
+      </c>
+      <c r="B702" t="str">
+        <v>Event invitation</v>
+      </c>
+      <c r="C702" t="str">
+        <v>Convite para evento</v>
+      </c>
+      <c r="D702" t="str">
+        <v>Invitación a un evento</v>
+      </c>
+      <c r="E702" t="str">
+        <v>Invitation à un événement</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="str">
+        <v>Invites to an event with date, time and place</v>
+      </c>
+      <c r="B703" t="str">
+        <v>Invites to an event with date, time and place</v>
+      </c>
+      <c r="C703" t="str">
+        <v>Convida para um evento com data, hora e local</v>
+      </c>
+      <c r="D703" t="str">
+        <v>Invita a un evento con fecha, hora y lugar</v>
+      </c>
+      <c r="E703" t="str">
+        <v>Invite à un événement avec date, heure et lieu</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="str">
+        <v>You are invited</v>
+      </c>
+      <c r="B704" t="str">
+        <v>You are invited</v>
+      </c>
+      <c r="C704" t="str">
+        <v>Está convidado</v>
+      </c>
+      <c r="D704" t="str">
+        <v>Está invitado</v>
+      </c>
+      <c r="E704" t="str">
+        <v>Vous êtes invité</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="str">
+        <v>Event name</v>
+      </c>
+      <c r="B705" t="str">
+        <v>Event name</v>
+      </c>
+      <c r="C705" t="str">
+        <v>Nome do evento</v>
+      </c>
+      <c r="D705" t="str">
+        <v>Nombre del evento</v>
+      </c>
+      <c r="E705" t="str">
+        <v>Nom de l’événement</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="str">
+        <v>we would like to have you with us.</v>
+      </c>
+      <c r="B706" t="str">
+        <v>we would like to have you with us.</v>
+      </c>
+      <c r="C706" t="str">
+        <v>gostaríamos de contar consigo.</v>
+      </c>
+      <c r="D706" t="str">
+        <v>nos gustaría contar con usted.</v>
+      </c>
+      <c r="E706" t="str">
+        <v>nous serions ravis de vous compter parmi nous.</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B707" t="str">
+        <v>Date</v>
+      </c>
+      <c r="C707" t="str">
+        <v>Data</v>
+      </c>
+      <c r="D707" t="str">
+        <v>Fecha</v>
+      </c>
+      <c r="E707" t="str">
+        <v>Date</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="str">
+        <v>Time</v>
+      </c>
+      <c r="B708" t="str">
+        <v>Time</v>
+      </c>
+      <c r="C708" t="str">
+        <v>Hora</v>
+      </c>
+      <c r="D708" t="str">
+        <v>Hora</v>
+      </c>
+      <c r="E708" t="str">
+        <v>Heure</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="str">
+        <v>Place</v>
+      </c>
+      <c r="B709" t="str">
+        <v>Place</v>
+      </c>
+      <c r="C709" t="str">
+        <v>Local</v>
+      </c>
+      <c r="D709" t="str">
+        <v>Lugar</v>
+      </c>
+      <c r="E709" t="str">
+        <v>Lieu</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="str">
+        <v>Place name</v>
+      </c>
+      <c r="B710" t="str">
+        <v>Place name</v>
+      </c>
+      <c r="C710" t="str">
+        <v>Nome do local</v>
+      </c>
+      <c r="D710" t="str">
+        <v>Nombre del lugar</v>
+      </c>
+      <c r="E710" t="str">
+        <v>Nom du lieu</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="str">
+        <v>Confirm attendance</v>
+      </c>
+      <c r="B711" t="str">
+        <v>Confirm attendance</v>
+      </c>
+      <c r="C711" t="str">
+        <v>Confirmar presença</v>
+      </c>
+      <c r="D711" t="str">
+        <v>Confirmar asistencia</v>
+      </c>
+      <c r="E711" t="str">
+        <v>Confirmer la présence</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="str">
+        <v>Congratulations</v>
+      </c>
+      <c r="B712" t="str">
+        <v>Congratulations</v>
+      </c>
+      <c r="C712" t="str">
+        <v>Parabéns</v>
+      </c>
+      <c r="D712" t="str">
+        <v>Felicidades</v>
+      </c>
+      <c r="E712" t="str">
+        <v>Félicitations</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="str">
+        <v>Celebrates a person's achievement, such as finishing a course</v>
+      </c>
+      <c r="B713" t="str">
+        <v>Celebrates a person's achievement, such as finishing a course</v>
+      </c>
+      <c r="C713" t="str">
+        <v>Celebra uma conquista, como terminar um curso</v>
+      </c>
+      <c r="D713" t="str">
+        <v>Celebra un logro, como terminar un curso</v>
+      </c>
+      <c r="E713" t="str">
+        <v>Célèbre une réussite, comme la fin d’un cours</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="str">
+        <v>You have completed the course.</v>
+      </c>
+      <c r="B714" t="str">
+        <v>You have completed the course.</v>
+      </c>
+      <c r="C714" t="str">
+        <v>Concluiu o curso.</v>
+      </c>
+      <c r="D714" t="str">
+        <v>Ha completado el curso.</v>
+      </c>
+      <c r="E714" t="str">
+        <v>Vous avez terminé le cours.</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="str">
+        <v>Thank you for your dedication. Your certificate is available on the platform.</v>
+      </c>
+      <c r="B715" t="str">
+        <v>Thank you for your dedication. Your certificate is available on the platform.</v>
+      </c>
+      <c r="C715" t="str">
+        <v>Obrigado pela sua dedicação. O seu certificado está disponível na plataforma.</v>
+      </c>
+      <c r="D715" t="str">
+        <v>Gracias por su dedicación. Su certificado está disponible en la plataforma.</v>
+      </c>
+      <c r="E715" t="str">
+        <v>Merci pour votre engagement. Votre certificat est disponible sur la plateforme.</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="str">
+        <v>See my certificate</v>
+      </c>
+      <c r="B716" t="str">
+        <v>See my certificate</v>
+      </c>
+      <c r="C716" t="str">
+        <v>Ver o meu certificado</v>
+      </c>
+      <c r="D716" t="str">
+        <v>Ver mi certificado</v>
+      </c>
+      <c r="E716" t="str">
+        <v>Voir mon certificat</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="str">
+        <v>Simple message</v>
+      </c>
+      <c r="B717" t="str">
+        <v>Simple message</v>
+      </c>
+      <c r="C717" t="str">
+        <v>Mensagem simples</v>
+      </c>
+      <c r="D717" t="str">
+        <v>Mensaje sencillo</v>
+      </c>
+      <c r="E717" t="str">
+        <v>Message simple</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="str">
+        <v>Just a greeting, your text and a signature</v>
+      </c>
+      <c r="B718" t="str">
+        <v>Just a greeting, your text and a signature</v>
+      </c>
+      <c r="C718" t="str">
+        <v>Só uma saudação, o seu texto e uma assinatura</v>
+      </c>
+      <c r="D718" t="str">
+        <v>Solo un saludo, su texto y una firma</v>
+      </c>
+      <c r="E718" t="str">
+        <v>Juste une salutation, votre texte et une signature</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="str">
+        <v>The mail server the platform uses to send e-mails</v>
+      </c>
+      <c r="B719" t="str">
+        <v>The mail server the platform uses to send e-mails</v>
+      </c>
+      <c r="C719" t="str">
+        <v>O servidor de e-mail que a plataforma usa para enviar e-mails</v>
+      </c>
+      <c r="D719" t="str">
+        <v>El servidor de correo que usa la plataforma para enviar correos</v>
+      </c>
+      <c r="E719" t="str">
+        <v>Le serveur de messagerie que la plateforme utilise pour envoyer les e-mails</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="str">
+        <v>Configured</v>
+      </c>
+      <c r="B720" t="str">
+        <v>Configured</v>
+      </c>
+      <c r="C720" t="str">
+        <v>Configurado</v>
+      </c>
+      <c r="D720" t="str">
+        <v>Configurado</v>
+      </c>
+      <c r="E720" t="str">
+        <v>Configuré</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="str">
+        <v>Not configured</v>
+      </c>
+      <c r="B721" t="str">
+        <v>Not configured</v>
+      </c>
+      <c r="C721" t="str">
+        <v>Por configurar</v>
+      </c>
+      <c r="D721" t="str">
+        <v>Sin configurar</v>
+      </c>
+      <c r="E721" t="str">
+        <v>Non configuré</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="str">
+        <v>Server</v>
+      </c>
+      <c r="B722" t="str">
+        <v>Server</v>
+      </c>
+      <c r="C722" t="str">
+        <v>Servidor</v>
+      </c>
+      <c r="D722" t="str">
+        <v>Servidor</v>
+      </c>
+      <c r="E722" t="str">
+        <v>Serveur</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="str">
+        <v>Where the e-mails are sent from. Your hosting or e-mail service gives you these values</v>
+      </c>
+      <c r="B723" t="str">
+        <v>Where the e-mails are sent from. Your hosting or e-mail service gives you these values</v>
+      </c>
+      <c r="C723" t="str">
+        <v>De onde os e-mails são enviados. O alojamento ou o serviço de e-mail dá-lhe estes valores</v>
+      </c>
+      <c r="D723" t="str">
+        <v>Desde dónde se envían los correos. Su alojamiento o servicio de correo le da estos valores</v>
+      </c>
+      <c r="E723" t="str">
+        <v>D’où les e-mails sont envoyés. Votre hébergeur ou service de messagerie vous fournit ces valeurs</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="str">
+        <v>Quick setup</v>
+      </c>
+      <c r="B724" t="str">
+        <v>Quick setup</v>
+      </c>
+      <c r="C724" t="str">
+        <v>Configuração rápida</v>
+      </c>
+      <c r="D724" t="str">
+        <v>Configuración rápida</v>
+      </c>
+      <c r="E724" t="str">
+        <v>Configuration rapide</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="str">
+        <v>Choose a common setup</v>
+      </c>
+      <c r="B725" t="str">
+        <v>Choose a common setup</v>
+      </c>
+      <c r="C725" t="str">
+        <v>Escolha uma configuração comum</v>
+      </c>
+      <c r="D725" t="str">
+        <v>Elija una configuración común</v>
+      </c>
+      <c r="E725" t="str">
+        <v>Choisissez une configuration courante</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="str">
+        <v>Fills in the port and the secure connection. The server and the account are yours to fill in</v>
+      </c>
+      <c r="B726" t="str">
+        <v>Fills in the port and the secure connection. The server and the account are yours to fill in</v>
+      </c>
+      <c r="C726" t="str">
+        <v>Preenche a porta e a ligação segura. O servidor e a conta são consigo</v>
+      </c>
+      <c r="D726" t="str">
+        <v>Rellena el puerto y la conexión segura. El servidor y la cuenta los rellena usted</v>
+      </c>
+      <c r="E726" t="str">
+        <v>Remplit le port et la connexion sécurisée. Le serveur et le compte sont à compléter par vous</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="str">
+        <v>Host</v>
+      </c>
+      <c r="B727" t="str">
+        <v>Host</v>
+      </c>
+      <c r="C727" t="str">
+        <v>Servidor (host)</v>
+      </c>
+      <c r="D727" t="str">
+        <v>Servidor (host)</v>
+      </c>
+      <c r="E727" t="str">
+        <v>Hôte</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="str">
+        <v>For example mail.yourdomain.com</v>
+      </c>
+      <c r="B728" t="str">
+        <v>For example mail.yourdomain.com</v>
+      </c>
+      <c r="C728" t="str">
+        <v>Por exemplo mail.seudominio.com</v>
+      </c>
+      <c r="D728" t="str">
+        <v>Por ejemplo mail.sudominio.com</v>
+      </c>
+      <c r="E728" t="str">
+        <v>Par exemple mail.votredomaine.com</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="str">
+        <v>Port</v>
+      </c>
+      <c r="B729" t="str">
+        <v>Port</v>
+      </c>
+      <c r="C729" t="str">
+        <v>Porta</v>
+      </c>
+      <c r="D729" t="str">
+        <v>Puerto</v>
+      </c>
+      <c r="E729" t="str">
+        <v>Port</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="str">
+        <v>Use only numbers</v>
+      </c>
+      <c r="B730" t="str">
+        <v>Use only numbers</v>
+      </c>
+      <c r="C730" t="str">
+        <v>Use só números</v>
+      </c>
+      <c r="D730" t="str">
+        <v>Use solo números</v>
+      </c>
+      <c r="E730" t="str">
+        <v>Utilisez uniquement des chiffres</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="str">
+        <v>Secure connection (SSL/TLS)</v>
+      </c>
+      <c r="B731" t="str">
+        <v>Secure connection (SSL/TLS)</v>
+      </c>
+      <c r="C731" t="str">
+        <v>Ligação segura (SSL/TLS)</v>
+      </c>
+      <c r="D731" t="str">
+        <v>Conexión segura (SSL/TLS)</v>
+      </c>
+      <c r="E731" t="str">
+        <v>Connexion sécurisée (SSL/TLS)</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="str">
+        <v>On for port 465. Off for 587, which switches to a secure connection by itself (STARTTLS)</v>
+      </c>
+      <c r="B732" t="str">
+        <v>On for port 465. Off for 587, which switches to a secure connection by itself (STARTTLS)</v>
+      </c>
+      <c r="C732" t="str">
+        <v>Ligada na porta 465. Desligada na 587, que passa sozinha a ligação segura (STARTTLS)</v>
+      </c>
+      <c r="D732" t="str">
+        <v>Activada en el puerto 465. Desactivada en el 587, que cambia sola a conexión segura (STARTTLS)</v>
+      </c>
+      <c r="E732" t="str">
+        <v>Activée pour le port 465. Désactivée pour le 587, qui passe seul en connexion sécurisée (STARTTLS)</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="str">
+        <v>Account and sender</v>
+      </c>
+      <c r="B733" t="str">
+        <v>Account and sender</v>
+      </c>
+      <c r="C733" t="str">
+        <v>Conta e remetente</v>
+      </c>
+      <c r="D733" t="str">
+        <v>Cuenta y remitente</v>
+      </c>
+      <c r="E733" t="str">
+        <v>Compte et expéditeur</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="str">
+        <v>The account used to log in and the name that appears as the sender</v>
+      </c>
+      <c r="B734" t="str">
+        <v>The account used to log in and the name that appears as the sender</v>
+      </c>
+      <c r="C734" t="str">
+        <v>A conta usada para iniciar sessão e o nome que aparece como remetente</v>
+      </c>
+      <c r="D734" t="str">
+        <v>La cuenta usada para iniciar sesión y el nombre que aparece como remitente</v>
+      </c>
+      <c r="E734" t="str">
+        <v>Le compte utilisé pour se connecter et le nom qui apparaît comme expéditeur</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="str">
+        <v>E-mail</v>
+      </c>
+      <c r="B735" t="str">
+        <v>E-mail</v>
+      </c>
+      <c r="C735" t="str">
+        <v>E-mail</v>
+      </c>
+      <c r="D735" t="str">
+        <v>Correo electrónico</v>
+      </c>
+      <c r="E735" t="str">
+        <v>E-mail</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="str">
+        <v>Used to log in and as the sender address</v>
+      </c>
+      <c r="B736" t="str">
+        <v>Used to log in and as the sender address</v>
+      </c>
+      <c r="C736" t="str">
+        <v>Usado para iniciar sessão e como endereço do remetente</v>
+      </c>
+      <c r="D736" t="str">
+        <v>Se usa para iniciar sesión y como dirección del remitente</v>
+      </c>
+      <c r="E736" t="str">
+        <v>Utilisé pour se connecter et comme adresse de l’expéditeur</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="str">
+        <v>Enter a valid e-mail address</v>
+      </c>
+      <c r="B737" t="str">
+        <v>Enter a valid e-mail address</v>
+      </c>
+      <c r="C737" t="str">
+        <v>Introduza um endereço de e-mail válido</v>
+      </c>
+      <c r="D737" t="str">
+        <v>Introduzca una dirección de correo válida</v>
+      </c>
+      <c r="E737" t="str">
+        <v>Saisissez une adresse e-mail valide</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="str">
+        <v>Sender name</v>
+      </c>
+      <c r="B738" t="str">
+        <v>Sender name</v>
+      </c>
+      <c r="C738" t="str">
+        <v>Nome do remetente</v>
+      </c>
+      <c r="D738" t="str">
+        <v>Nombre del remitente</v>
+      </c>
+      <c r="E738" t="str">
+        <v>Nom de l’expéditeur</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="str">
+        <v>What the person sees as the sender, for example Bial Academy</v>
+      </c>
+      <c r="B739" t="str">
+        <v>What the person sees as the sender, for example Bial Academy</v>
+      </c>
+      <c r="C739" t="str">
+        <v>O que a pessoa vê como remetente, por exemplo Bial Academy</v>
+      </c>
+      <c r="D739" t="str">
+        <v>Lo que la persona ve como remitente, por ejemplo Bial Academy</v>
+      </c>
+      <c r="E739" t="str">
+        <v>Ce que la personne voit comme expéditeur, par exemple Bial Academy</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="str">
+        <v>Password</v>
+      </c>
+      <c r="B740" t="str">
+        <v>Password</v>
+      </c>
+      <c r="C740" t="str">
+        <v>Palavra-passe</v>
+      </c>
+      <c r="D740" t="str">
+        <v>Contraseña</v>
+      </c>
+      <c r="E740" t="str">
+        <v>Mot de passe</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="str">
+        <v>Test the settings</v>
+      </c>
+      <c r="B741" t="str">
+        <v>Test the settings</v>
+      </c>
+      <c r="C741" t="str">
+        <v>Testar as definições</v>
+      </c>
+      <c r="D741" t="str">
+        <v>Probar la configuración</v>
+      </c>
+      <c r="E741" t="str">
+        <v>Tester les paramètres</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="str">
+        <v>Sends a test e-mail with the values above, even if you have not saved them yet</v>
+      </c>
+      <c r="B742" t="str">
+        <v>Sends a test e-mail with the values above, even if you have not saved them yet</v>
+      </c>
+      <c r="C742" t="str">
+        <v>Envia um e-mail de teste com os valores acima, mesmo que ainda não os tenha guardado</v>
+      </c>
+      <c r="D742" t="str">
+        <v>Envía un correo de prueba con los valores de arriba, aunque aún no los haya guardado</v>
+      </c>
+      <c r="E742" t="str">
+        <v>Envoie un e-mail de test avec les valeurs ci-dessus, même si vous ne les avez pas encore enregistrées</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="str">
+        <v>Send the test to</v>
+      </c>
+      <c r="B743" t="str">
+        <v>Send the test to</v>
+      </c>
+      <c r="C743" t="str">
+        <v>Enviar o teste para</v>
+      </c>
+      <c r="D743" t="str">
+        <v>Enviar la prueba a</v>
+      </c>
+      <c r="E743" t="str">
+        <v>Envoyer le test à</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="str">
+        <v>Check the inbox (and the spam folder) of that address</v>
+      </c>
+      <c r="B744" t="str">
+        <v>Check the inbox (and the spam folder) of that address</v>
+      </c>
+      <c r="C744" t="str">
+        <v>Verifique a caixa de entrada (e o spam) desse endereço</v>
+      </c>
+      <c r="D744" t="str">
+        <v>Revise la bandeja de entrada (y el spam) de esa dirección</v>
+      </c>
+      <c r="E744" t="str">
+        <v>Vérifiez la boîte de réception (et les spams) de cette adresse</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="str">
+        <v>Where it is used</v>
+      </c>
+      <c r="B745" t="str">
+        <v>Where it is used</v>
+      </c>
+      <c r="C745" t="str">
+        <v>Onde é usado</v>
+      </c>
+      <c r="D745" t="str">
+        <v>Dónde se usa</v>
+      </c>
+      <c r="E745" t="str">
+        <v>Où il est utilisé</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="str">
+        <v>Everything the platform sends goes through this server</v>
+      </c>
+      <c r="B746" t="str">
+        <v>Everything the platform sends goes through this server</v>
+      </c>
+      <c r="C746" t="str">
+        <v>Tudo o que a plataforma envia passa por este servidor</v>
+      </c>
+      <c r="D746" t="str">
+        <v>Todo lo que envía la plataforma pasa por este servidor</v>
+      </c>
+      <c r="E746" t="str">
+        <v>Tout ce que la plateforme envoie passe par ce serveur</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="str">
+        <v>Account e-mails (registration, status, password recovery)</v>
+      </c>
+      <c r="B747" t="str">
+        <v>Account e-mails (registration, status, password recovery)</v>
+      </c>
+      <c r="C747" t="str">
+        <v>E-mails da conta (registo, estado, recuperação de password)</v>
+      </c>
+      <c r="D747" t="str">
+        <v>Correos de la cuenta (registro, estado, recuperación de contraseña)</v>
+      </c>
+      <c r="E747" t="str">
+        <v>E-mails du compte (inscription, statut, récupération du mot de passe)</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="str">
+        <v>Templates and their test e-mails</v>
+      </c>
+      <c r="B748" t="str">
+        <v>Templates and their test e-mails</v>
+      </c>
+      <c r="C748" t="str">
+        <v>Templates e os respetivos e-mails de teste</v>
+      </c>
+      <c r="D748" t="str">
+        <v>Plantillas y sus correos de prueba</v>
+      </c>
+      <c r="E748" t="str">
+        <v>Modèles et leurs e-mails de test</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="str">
+        <v>Communications, sent in batches</v>
+      </c>
+      <c r="B749" t="str">
+        <v>Communications, sent in batches</v>
+      </c>
+      <c r="C749" t="str">
+        <v>Comunicações, enviadas em lotes</v>
+      </c>
+      <c r="D749" t="str">
+        <v>Comunicaciones, enviadas por lotes</v>
+      </c>
+      <c r="E749" t="str">
+        <v>Communications, envoyées par lots</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="str">
+        <v>Hosting servers limit how many e-mails can be sent per hour. For many recipients, a dedicated e-mail service (for example Brevo) delivers better</v>
+      </c>
+      <c r="B750" t="str">
+        <v>Hosting servers limit how many e-mails can be sent per hour. For many recipients, a dedicated e-mail service (for example Brevo) delivers better</v>
+      </c>
+      <c r="C750" t="str">
+        <v>Os servidores de alojamento limitam os e-mails enviados por hora. Para muitos destinatários, um serviço de e-mail dedicado (por exemplo o Brevo) entrega melhor</v>
+      </c>
+      <c r="D750" t="str">
+        <v>Los servidores de alojamiento limitan los correos enviados por hora. Para muchos destinatarios, un servicio de correo dedicado (por ejemplo Brevo) entrega mejor</v>
+      </c>
+      <c r="E750" t="str">
+        <v>Les serveurs d’hébergement limitent le nombre d’e-mails envoyés par heure. Pour de nombreux destinataires, un service d’e-mail dédié (par exemple Brevo) délivre mieux</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="str">
+        <v>file</v>
+      </c>
+      <c r="B751" t="str">
+        <v>file</v>
+      </c>
+      <c r="C751" t="str">
+        <v>ficheiro</v>
+      </c>
+      <c r="D751" t="str">
+        <v>archivo</v>
+      </c>
+      <c r="E751" t="str">
+        <v>fichier</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="str">
+        <v>files</v>
+      </c>
+      <c r="B752" t="str">
+        <v>files</v>
+      </c>
+      <c r="C752" t="str">
+        <v>ficheiros</v>
+      </c>
+      <c r="D752" t="str">
+        <v>archivos</v>
+      </c>
+      <c r="E752" t="str">
+        <v>fichiers</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="str">
+        <v>Files</v>
+      </c>
+      <c r="B753" t="str">
+        <v>Files</v>
+      </c>
+      <c r="C753" t="str">
+        <v>Ficheiros</v>
+      </c>
+      <c r="D753" t="str">
+        <v>Archivos</v>
+      </c>
+      <c r="E753" t="str">
+        <v>Fichiers</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="str">
+        <v>Accepted</v>
+      </c>
+      <c r="B754" t="str">
+        <v>Accepted</v>
+      </c>
+      <c r="C754" t="str">
+        <v>Aceite</v>
+      </c>
+      <c r="D754" t="str">
+        <v>Aceptada</v>
+      </c>
+      <c r="E754" t="str">
+        <v>Acceptée</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="str">
+        <v>Not given</v>
+      </c>
+      <c r="B755" t="str">
+        <v>Not given</v>
+      </c>
+      <c r="C755" t="str">
+        <v>Não dada</v>
+      </c>
+      <c r="D755" t="str">
+        <v>No otorgada</v>
+      </c>
+      <c r="E755" t="str">
+        <v>Non donnée</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="str">
+        <v>Privacy consent</v>
+      </c>
+      <c r="B756" t="str">
+        <v>Privacy consent</v>
+      </c>
+      <c r="C756" t="str">
+        <v>Consentimento de privacidade</v>
+      </c>
+      <c r="D756" t="str">
+        <v>Consentimiento de privacidad</v>
+      </c>
+      <c r="E756" t="str">
+        <v>Consentement à la confidentialité</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="str">
+        <v>Received</v>
+      </c>
+      <c r="B757" t="str">
+        <v>Received</v>
+      </c>
+      <c r="C757" t="str">
+        <v>Recebida</v>
+      </c>
+      <c r="D757" t="str">
+        <v>Recibida</v>
+      </c>
+      <c r="E757" t="str">
+        <v>Reçue</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="str">
+        <v>Received on {{date}}</v>
+      </c>
+      <c r="B758" t="str">
+        <v>Received on {{date}}</v>
+      </c>
+      <c r="C758" t="str">
+        <v>Recebida em {{date}}</v>
+      </c>
+      <c r="D758" t="str">
+        <v>Recibida el {{date}}</v>
+      </c>
+      <c r="E758" t="str">
+        <v>Reçue le {{date}}</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="str">
+        <v>Reply by e-mail</v>
+      </c>
+      <c r="B759" t="str">
+        <v>Reply by e-mail</v>
+      </c>
+      <c r="C759" t="str">
+        <v>Responder por e-mail</v>
+      </c>
+      <c r="D759" t="str">
+        <v>Responder por correo</v>
+      </c>
+      <c r="E759" t="str">
+        <v>Répondre par e-mail</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="str">
+        <v>What the person wrote in the contact form</v>
+      </c>
+      <c r="B760" t="str">
+        <v>What the person wrote in the contact form</v>
+      </c>
+      <c r="C760" t="str">
+        <v>O que a pessoa escreveu no formulário de contacto</v>
+      </c>
+      <c r="D760" t="str">
+        <v>Lo que la persona escribió en el formulario de contacto</v>
+      </c>
+      <c r="E760" t="str">
+        <v>Ce que la personne a écrit dans le formulaire de contact</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="str">
+        <v>The message is empty</v>
+      </c>
+      <c r="B761" t="str">
+        <v>The message is empty</v>
+      </c>
+      <c r="C761" t="str">
+        <v>A mensagem está vazia</v>
+      </c>
+      <c r="D761" t="str">
+        <v>El mensaje está vacío</v>
+      </c>
+      <c r="E761" t="str">
+        <v>Le message est vide</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="str">
+        <v>Sender</v>
+      </c>
+      <c r="B762" t="str">
+        <v>Sender</v>
+      </c>
+      <c r="C762" t="str">
+        <v>Remetente</v>
+      </c>
+      <c r="D762" t="str">
+        <v>Remitente</v>
+      </c>
+      <c r="E762" t="str">
+        <v>Expéditeur</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="str">
+        <v>Who sent the message</v>
+      </c>
+      <c r="B763" t="str">
+        <v>Who sent the message</v>
+      </c>
+      <c r="C763" t="str">
+        <v>Quem enviou a mensagem</v>
+      </c>
+      <c r="D763" t="str">
+        <v>Quién envió el mensaje</v>
+      </c>
+      <c r="E763" t="str">
+        <v>Qui a envoyé le message</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="str">
+        <v>Registered user</v>
+      </c>
+      <c r="B764" t="str">
+        <v>Registered user</v>
+      </c>
+      <c r="C764" t="str">
+        <v>Utilizador registado</v>
+      </c>
+      <c r="D764" t="str">
+        <v>Usuario registrado</v>
+      </c>
+      <c r="E764" t="str">
+        <v>Utilisateur inscrit</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="str">
+        <v>Not a registered user</v>
+      </c>
+      <c r="B765" t="str">
+        <v>Not a registered user</v>
+      </c>
+      <c r="C765" t="str">
+        <v>Não é um utilizador registado</v>
+      </c>
+      <c r="D765" t="str">
+        <v>No es un usuario registrado</v>
+      </c>
+      <c r="E765" t="str">
+        <v>Ce n’est pas un utilisateur inscrit</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="str">
+        <v>Submission</v>
+      </c>
+      <c r="B766" t="str">
+        <v>Submission</v>
+      </c>
+      <c r="C766" t="str">
+        <v>Submissão</v>
+      </c>
+      <c r="D766" t="str">
+        <v>Envío</v>
+      </c>
+      <c r="E766" t="str">
+        <v>Soumission</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="str">
+        <v>Data of this submission</v>
+      </c>
+      <c r="B767" t="str">
+        <v>Data of this submission</v>
+      </c>
+      <c r="C767" t="str">
+        <v>Dados desta submissão</v>
+      </c>
+      <c r="D767" t="str">
+        <v>Datos de este envío</v>
+      </c>
+      <c r="E767" t="str">
+        <v>Données de cette soumission</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="str">
+        <v>Submission deleted</v>
+      </c>
+      <c r="B768" t="str">
+        <v>Submission deleted</v>
+      </c>
+      <c r="C768" t="str">
+        <v>Submissão eliminada</v>
+      </c>
+      <c r="D768" t="str">
+        <v>Envío eliminado</v>
+      </c>
+      <c r="E768" t="str">
+        <v>Soumission supprimée</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="str">
+        <v>Copy</v>
+      </c>
+      <c r="B769" t="str">
+        <v>Copy</v>
+      </c>
+      <c r="C769" t="str">
+        <v>Copiar</v>
+      </c>
+      <c r="D769" t="str">
+        <v>Copiar</v>
+      </c>
+      <c r="E769" t="str">
+        <v>Copier</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="str">
+        <v>Change</v>
+      </c>
+      <c r="B770" t="str">
+        <v>Change</v>
+      </c>
+      <c r="C770" t="str">
+        <v>Trocar</v>
+      </c>
+      <c r="D770" t="str">
+        <v>Cambiar</v>
+      </c>
+      <c r="E770" t="str">
+        <v>Changer</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="str">
+        <v>Remove</v>
+      </c>
+      <c r="B771" t="str">
+        <v>Remove</v>
+      </c>
+      <c r="C771" t="str">
+        <v>Remover</v>
+      </c>
+      <c r="D771" t="str">
+        <v>Quitar</v>
+      </c>
+      <c r="E771" t="str">
+        <v>Retirer</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="str">
+        <v>Choose an image</v>
+      </c>
+      <c r="B772" t="str">
+        <v>Choose an image</v>
+      </c>
+      <c r="C772" t="str">
+        <v>Escolher uma imagem</v>
+      </c>
+      <c r="D772" t="str">
+        <v>Elegir una imagen</v>
+      </c>
+      <c r="E772" t="str">
+        <v>Choisir une image</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="str">
+        <v>Choose a file</v>
+      </c>
+      <c r="B773" t="str">
+        <v>Choose a file</v>
+      </c>
+      <c r="C773" t="str">
+        <v>Escolher um ficheiro</v>
+      </c>
+      <c r="D773" t="str">
+        <v>Elegir un archivo</v>
+      </c>
+      <c r="E773" t="str">
+        <v>Choisir un fichier</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="str">
+        <v>Default role</v>
+      </c>
+      <c r="B774" t="str">
+        <v>Default role</v>
+      </c>
+      <c r="C774" t="str">
+        <v>Função por omissão</v>
+      </c>
+      <c r="D774" t="str">
+        <v>Rol por defecto</v>
+      </c>
+      <c r="E774" t="str">
+        <v>Rôle par défaut</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="str">
+        <v>This is the role given at registration: its name is fixed, only its permissions can be changed</v>
+      </c>
+      <c r="B775" t="str">
+        <v>This is the role given at registration: its name is fixed, only its permissions can be changed</v>
+      </c>
+      <c r="C775" t="str">
+        <v>Esta é a função atribuída no registo: o nome é fixo, só se podem alterar as permissões</v>
+      </c>
+      <c r="D775" t="str">
+        <v>Este es el rol que se asigna al registrarse: su nombre es fijo, solo se pueden cambiar sus permisos</v>
+      </c>
+      <c r="E775" t="str">
+        <v>C’est le rôle attribué à l’inscription : son nom est fixe, seules ses permissions peuvent être modifiées</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="str">
+        <v>Uploaded</v>
+      </c>
+      <c r="B776" t="str">
+        <v>Uploaded</v>
+      </c>
+      <c r="C776" t="str">
+        <v>Carregado</v>
+      </c>
+      <c r="D776" t="str">
+        <v>Subido</v>
+      </c>
+      <c r="E776" t="str">
+        <v>Téléversé</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="str">
+        <v>Account access</v>
+      </c>
+      <c r="B777" t="str">
+        <v>Account access</v>
+      </c>
+      <c r="C777" t="str">
+        <v>Acesso à conta</v>
+      </c>
+      <c r="D777" t="str">
+        <v>Acceso a la cuenta</v>
+      </c>
+      <c r="E777" t="str">
+        <v>Accès au compte</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="str">
+        <v>Account approved</v>
+      </c>
+      <c r="B778" t="str">
+        <v>Account approved</v>
+      </c>
+      <c r="C778" t="str">
+        <v>Conta aprovada</v>
+      </c>
+      <c r="D778" t="str">
+        <v>Cuenta aprobada</v>
+      </c>
+      <c r="E778" t="str">
+        <v>Compte approuvé</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="str">
+        <v>Account not approved</v>
+      </c>
+      <c r="B779" t="str">
+        <v>Account not approved</v>
+      </c>
+      <c r="C779" t="str">
+        <v>Conta não aprovada</v>
+      </c>
+      <c r="D779" t="str">
+        <v>Cuenta no aprobada</v>
+      </c>
+      <c r="E779" t="str">
+        <v>Compte non approuvé</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="str">
+        <v>Button link</v>
+      </c>
+      <c r="B780" t="str">
+        <v>Button link</v>
+      </c>
+      <c r="C780" t="str">
+        <v>Ligação do botão</v>
+      </c>
+      <c r="D780" t="str">
+        <v>Enlace del botón</v>
+      </c>
+      <c r="E780" t="str">
+        <v>Lien du bouton</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="str">
+        <v>Contact message received</v>
+      </c>
+      <c r="B781" t="str">
+        <v>Contact message received</v>
+      </c>
+      <c r="C781" t="str">
+        <v>Mensagem de contacto recebida</v>
+      </c>
+      <c r="D781" t="str">
+        <v>Mensaje de contacto recibido</v>
+      </c>
+      <c r="E781" t="str">
+        <v>Message de contact reçu</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="str">
+        <v>Course completed</v>
+      </c>
+      <c r="B782" t="str">
+        <v>Course completed</v>
+      </c>
+      <c r="C782" t="str">
+        <v>Curso concluído</v>
+      </c>
+      <c r="D782" t="str">
+        <v>Curso completado</v>
+      </c>
+      <c r="E782" t="str">
+        <v>Cours terminé</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="str">
+        <v>New contact message (team)</v>
+      </c>
+      <c r="B783" t="str">
+        <v>New contact message (team)</v>
+      </c>
+      <c r="C783" t="str">
+        <v>Nova mensagem de contacto (equipa)</v>
+      </c>
+      <c r="D783" t="str">
+        <v>Nuevo mensaje de contacto (equipo)</v>
+      </c>
+      <c r="E783" t="str">
+        <v>Nouveau message de contact (équipe)</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="str">
+        <v>Password changed</v>
+      </c>
+      <c r="B784" t="str">
+        <v>Password changed</v>
+      </c>
+      <c r="C784" t="str">
+        <v>Password alterada</v>
+      </c>
+      <c r="D784" t="str">
+        <v>Contraseña cambiada</v>
+      </c>
+      <c r="E784" t="str">
+        <v>Mot de passe modifié</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="str">
+        <v>Registration received</v>
+      </c>
+      <c r="B785" t="str">
+        <v>Registration received</v>
+      </c>
+      <c r="C785" t="str">
+        <v>Registo recebido</v>
+      </c>
+      <c r="D785" t="str">
+        <v>Registro recibido</v>
+      </c>
+      <c r="E785" t="str">
+        <v>Inscription reçue</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="str">
+        <v>Reply to the request</v>
+      </c>
+      <c r="B786" t="str">
+        <v>Reply to the request</v>
+      </c>
+      <c r="C786" t="str">
+        <v>Resposta ao pedido</v>
+      </c>
+      <c r="D786" t="str">
+        <v>Respuesta a la solicitud</v>
+      </c>
+      <c r="E786" t="str">
+        <v>Réponse à la demande</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="str">
+        <v>Request received</v>
+      </c>
+      <c r="B787" t="str">
+        <v>Request received</v>
+      </c>
+      <c r="C787" t="str">
+        <v>Pedido recebido</v>
+      </c>
+      <c r="D787" t="str">
+        <v>Solicitud recibida</v>
+      </c>
+      <c r="E787" t="str">
+        <v>Demande reçue</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="str">
+        <v>Sent to a person when the team replies to their ticket</v>
+      </c>
+      <c r="B788" t="str">
+        <v>Sent to a person when the team replies to their ticket</v>
+      </c>
+      <c r="C788" t="str">
+        <v>Enviado a uma pessoa quando a equipa responde ao seu ticket</v>
+      </c>
+      <c r="D788" t="str">
+        <v>Se envía a una persona cuando el equipo responde a su ticket</v>
+      </c>
+      <c r="E788" t="str">
+        <v>Envoyé à une personne lorsque l’équipe répond à son ticket</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="str">
+        <v>Sent to a person when they complete a course</v>
+      </c>
+      <c r="B789" t="str">
+        <v>Sent to a person when they complete a course</v>
+      </c>
+      <c r="C789" t="str">
+        <v>Enviado a uma pessoa quando conclui um curso</v>
+      </c>
+      <c r="D789" t="str">
+        <v>Se envía a una persona cuando completa un curso</v>
+      </c>
+      <c r="E789" t="str">
+        <v>Envoyé à une personne lorsqu’elle termine un cours</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="str">
+        <v>Sent to a person when they open a ticket</v>
+      </c>
+      <c r="B790" t="str">
+        <v>Sent to a person when they open a ticket</v>
+      </c>
+      <c r="C790" t="str">
+        <v>Enviado a uma pessoa quando abre um ticket</v>
+      </c>
+      <c r="D790" t="str">
+        <v>Se envía a una persona cuando abre un ticket</v>
+      </c>
+      <c r="E790" t="str">
+        <v>Envoyé à une personne lorsqu’elle ouvre un ticket</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="str">
+        <v>Sent to confirm that the password of an account was changed</v>
+      </c>
+      <c r="B791" t="str">
+        <v>Sent to confirm that the password of an account was changed</v>
+      </c>
+      <c r="C791" t="str">
+        <v>Enviado para confirmar que a password de uma conta foi alterada</v>
+      </c>
+      <c r="D791" t="str">
+        <v>Se envía para confirmar que se cambió la contraseña de una cuenta</v>
+      </c>
+      <c r="E791" t="str">
+        <v>Envoyé pour confirmer que le mot de passe d’un compte a été modifié</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="str">
+        <v>Sent to people whose account was created or imported by an administrator, with the code to set their password</v>
+      </c>
+      <c r="B792" t="str">
+        <v>Sent to people whose account was created or imported by an administrator, with the code to set their password</v>
+      </c>
+      <c r="C792" t="str">
+        <v>Enviado a quem teve a conta criada ou importada por um administrador, com o código para definir a password</v>
+      </c>
+      <c r="D792" t="str">
+        <v>Se envía a quienes tienen la cuenta creada o importada por un administrador, con el código para definir su contraseña</v>
+      </c>
+      <c r="E792" t="str">
+        <v>Envoyé aux personnes dont le compte a été créé ou importé par un administrateur, avec le code pour définir leur mot de passe</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="str">
+        <v>Sent to the person who writes in the contact form</v>
+      </c>
+      <c r="B793" t="str">
+        <v>Sent to the person who writes in the contact form</v>
+      </c>
+      <c r="C793" t="str">
+        <v>Enviado a quem escreve no formulário de contacto</v>
+      </c>
+      <c r="D793" t="str">
+        <v>Se envía a quien escribe en el formulario de contacto</v>
+      </c>
+      <c r="E793" t="str">
+        <v>Envoyé à la personne qui écrit dans le formulaire de contact</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="str">
+        <v>Sent to the team when someone writes in the contact form</v>
+      </c>
+      <c r="B794" t="str">
+        <v>Sent to the team when someone writes in the contact form</v>
+      </c>
+      <c r="C794" t="str">
+        <v>Enviado à equipa quando alguém escreve no formulário de contacto</v>
+      </c>
+      <c r="D794" t="str">
+        <v>Se envía al equipo cuando alguien escribe en el formulario de contacto</v>
+      </c>
+      <c r="E794" t="str">
+        <v>Envoyé à l’équipe lorsque quelqu’un écrit dans le formulaire de contact</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="str">
+        <v>Sent when a person registers, while the account waits for approval</v>
+      </c>
+      <c r="B795" t="str">
+        <v>Sent when a person registers, while the account waits for approval</v>
+      </c>
+      <c r="C795" t="str">
+        <v>Enviado quando uma pessoa se regista, enquanto a conta aguarda aprovação</v>
+      </c>
+      <c r="D795" t="str">
+        <v>Se envía cuando una persona se registra, mientras la cuenta espera aprobación</v>
+      </c>
+      <c r="E795" t="str">
+        <v>Envoyé lorsqu’une personne s’inscrit, pendant que le compte attend l’approbation</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="str">
+        <v>Sent when an account is marked as not approved</v>
+      </c>
+      <c r="B796" t="str">
+        <v>Sent when an account is marked as not approved</v>
+      </c>
+      <c r="C796" t="str">
+        <v>Enviado quando uma conta é marcada como não aprovada</v>
+      </c>
+      <c r="D796" t="str">
+        <v>Se envía cuando una cuenta se marca como no aprobada</v>
+      </c>
+      <c r="E796" t="str">
+        <v>Envoyé lorsqu’un compte est marqué comme non approuvé</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="str">
+        <v>Sent when an administrator approves an account</v>
+      </c>
+      <c r="B797" t="str">
+        <v>Sent when an administrator approves an account</v>
+      </c>
+      <c r="C797" t="str">
+        <v>Enviado quando um administrador aprova uma conta</v>
+      </c>
+      <c r="D797" t="str">
+        <v>Se envía cuando un administrador aprueba una cuenta</v>
+      </c>
+      <c r="E797" t="str">
+        <v>Envoyé lorsqu’un administrateur approuve un compte</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="str">
+        <v>The address the button of the e-mail opens</v>
+      </c>
+      <c r="B798" t="str">
+        <v>The address the button of the e-mail opens</v>
+      </c>
+      <c r="C798" t="str">
+        <v>O endereço que o botão do e-mail abre</v>
+      </c>
+      <c r="D798" t="str">
+        <v>La dirección que abre el botón del correo</v>
+      </c>
+      <c r="E798" t="str">
+        <v>L’adresse ouverte par le bouton de l’e-mail</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="str">
+        <v>The e-mail address of the person receiving the e-mail</v>
+      </c>
+      <c r="B799" t="str">
+        <v>The e-mail address of the person receiving the e-mail</v>
+      </c>
+      <c r="C799" t="str">
+        <v>O endereço de e-mail de quem recebe o e-mail</v>
+      </c>
+      <c r="D799" t="str">
+        <v>La dirección de correo de quien recibe el correo</v>
+      </c>
+      <c r="E799" t="str">
+        <v>L’adresse e-mail de la personne qui reçoit l’e-mail</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="str">
+        <v>The subject of the ticket or of the contact message</v>
+      </c>
+      <c r="B800" t="str">
+        <v>The subject of the ticket or of the contact message</v>
+      </c>
+      <c r="C800" t="str">
+        <v>O assunto do ticket ou da mensagem de contacto</v>
+      </c>
+      <c r="D800" t="str">
+        <v>El asunto del ticket o del mensaje de contacto</v>
+      </c>
+      <c r="E800" t="str">
+        <v>L’objet du ticket ou du message de contact</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="str">
+        <v>The text of the message</v>
+      </c>
+      <c r="B801" t="str">
+        <v>The text of the message</v>
+      </c>
+      <c r="C801" t="str">
+        <v>O texto da mensagem</v>
+      </c>
+      <c r="D801" t="str">
+        <v>El texto del mensaje</v>
+      </c>
+      <c r="E801" t="str">
+        <v>Le texte du message</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="str">
+        <v>Answered</v>
+      </c>
+      <c r="B802" t="str">
+        <v>Answered</v>
+      </c>
+      <c r="C802" t="str">
+        <v>Respondida</v>
+      </c>
+      <c r="D802" t="str">
+        <v>Respondida</v>
+      </c>
+      <c r="E802" t="str">
+        <v>Répondue</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="str">
+        <v>Waiting for reply</v>
+      </c>
+      <c r="B803" t="str">
+        <v>Waiting for reply</v>
+      </c>
+      <c r="C803" t="str">
+        <v>Por responder</v>
+      </c>
+      <c r="D803" t="str">
+        <v>Pendiente de respuesta</v>
+      </c>
+      <c r="E803" t="str">
+        <v>En attente de réponse</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="str">
+        <v>Reply failed</v>
+      </c>
+      <c r="B804" t="str">
+        <v>Reply failed</v>
+      </c>
+      <c r="C804" t="str">
+        <v>Falhou o envio da resposta</v>
+      </c>
+      <c r="D804" t="str">
+        <v>Falló el envío de la respuesta</v>
+      </c>
+      <c r="E804" t="str">
+        <v>Échec de l’envoi de la réponse</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="str">
+        <v>Reply</v>
+      </c>
+      <c r="B805" t="str">
+        <v>Reply</v>
+      </c>
+      <c r="C805" t="str">
+        <v>Responder</v>
+      </c>
+      <c r="D805" t="str">
+        <v>Responder</v>
+      </c>
+      <c r="E805" t="str">
+        <v>Répondre</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="str">
+        <v>Replies</v>
+      </c>
+      <c r="B806" t="str">
+        <v>Replies</v>
+      </c>
+      <c r="C806" t="str">
+        <v>Respostas</v>
+      </c>
+      <c r="D806" t="str">
+        <v>Respuestas</v>
+      </c>
+      <c r="E806" t="str">
+        <v>Réponses</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="str">
+        <v>Send reply</v>
+      </c>
+      <c r="B807" t="str">
+        <v>Send reply</v>
+      </c>
+      <c r="C807" t="str">
+        <v>Enviar resposta</v>
+      </c>
+      <c r="D807" t="str">
+        <v>Enviar respuesta</v>
+      </c>
+      <c r="E807" t="str">
+        <v>Envoyer la réponse</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="str">
+        <v>Write your reply here</v>
+      </c>
+      <c r="B808" t="str">
+        <v>Write your reply here</v>
+      </c>
+      <c r="C808" t="str">
+        <v>Escreva aqui a sua resposta</v>
+      </c>
+      <c r="D808" t="str">
+        <v>Escriba aquí su respuesta</v>
+      </c>
+      <c r="E808" t="str">
+        <v>Écrivez votre réponse ici</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="str">
+        <v>The reply is sent from the platform to the e-mail of the person, and is recorded here</v>
+      </c>
+      <c r="B809" t="str">
+        <v>The reply is sent from the platform to the e-mail of the person, and is recorded here</v>
+      </c>
+      <c r="C809" t="str">
+        <v>A resposta sai da plataforma para o e-mail da pessoa e fica registada aqui</v>
+      </c>
+      <c r="D809" t="str">
+        <v>La respuesta sale de la plataforma al correo de la persona y queda registrada aquí</v>
+      </c>
+      <c r="E809" t="str">
+        <v>La réponse part de la plateforme vers l’e-mail de la personne et est enregistrée ici</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="str">
+        <v>This submission has no valid e-mail address to reply to</v>
+      </c>
+      <c r="B810" t="str">
+        <v>This submission has no valid e-mail address to reply to</v>
+      </c>
+      <c r="C810" t="str">
+        <v>Esta submissão não tem um endereço de e-mail válido para responder</v>
+      </c>
+      <c r="D810" t="str">
+        <v>Este envío no tiene una dirección de correo válida para responder</v>
+      </c>
+      <c r="E810" t="str">
+        <v>Cette soumission n’a pas d’adresse e-mail valide pour répondre</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="str">
+        <v>Reply sent to {{email}}</v>
+      </c>
+      <c r="B811" t="str">
+        <v>Reply sent to {{email}}</v>
+      </c>
+      <c r="C811" t="str">
+        <v>Resposta enviada para {{email}}</v>
+      </c>
+      <c r="D811" t="str">
+        <v>Respuesta enviada a {{email}}</v>
+      </c>
+      <c r="E811" t="str">
+        <v>Réponse envoyée à {{email}}</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="str">
+        <v>The reply could not be sent</v>
+      </c>
+      <c r="B812" t="str">
+        <v>The reply could not be sent</v>
+      </c>
+      <c r="C812" t="str">
+        <v>Não foi possível enviar a resposta</v>
+      </c>
+      <c r="D812" t="str">
+        <v>No se pudo enviar la respuesta</v>
+      </c>
+      <c r="E812" t="str">
+        <v>Impossible d’envoyer la réponse</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="str">
+        <v>What was answered, by whom and if the e-mail was delivered to the mail server</v>
+      </c>
+      <c r="B813" t="str">
+        <v>What was answered, by whom and if the e-mail was delivered to the mail server</v>
+      </c>
+      <c r="C813" t="str">
+        <v>O que foi respondido, por quem e se o e-mail foi entregue ao servidor de e-mail</v>
+      </c>
+      <c r="D813" t="str">
+        <v>Qué se respondió, quién lo hizo y si el correo se entregó al servidor de correo</v>
+      </c>
+      <c r="E813" t="str">
+        <v>Ce qui a été répondu, par qui et si l’e-mail a été remis au serveur de messagerie</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="str">
+        <v>Unknown user</v>
+      </c>
+      <c r="B814" t="str">
+        <v>Unknown user</v>
+      </c>
+      <c r="C814" t="str">
+        <v>Utilizador desconhecido</v>
+      </c>
+      <c r="D814" t="str">
+        <v>Usuario desconocido</v>
+      </c>
+      <c r="E814" t="str">
+        <v>Utilisateur inconnu</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="str">
+        <v>To</v>
+      </c>
+      <c r="B815" t="str">
+        <v>To</v>
+      </c>
+      <c r="C815" t="str">
+        <v>Para</v>
+      </c>
+      <c r="D815" t="str">
+        <v>Para</v>
+      </c>
+      <c r="E815" t="str">
+        <v>À</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="str">
+        <v>QR code</v>
+      </c>
+      <c r="B816" t="str">
+        <v>QR code</v>
+      </c>
+      <c r="C816" t="str">
+        <v>Código QR</v>
+      </c>
+      <c r="D816" t="str">
+        <v>Código QR</v>
+      </c>
+      <c r="E816" t="str">
+        <v>Code QR</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="str">
+        <v>Reply to the contact form</v>
+      </c>
+      <c r="B817" t="str">
+        <v>Reply to the contact form</v>
+      </c>
+      <c r="C817" t="str">
+        <v>Resposta ao formulário de contacto</v>
+      </c>
+      <c r="D817" t="str">
+        <v>Respuesta al formulario de contacto</v>
+      </c>
+      <c r="E817" t="str">
+        <v>Réponse au formulaire de contact</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="str">
+        <v>Sent to the person when the team replies to their message from the Submissions page</v>
+      </c>
+      <c r="B818" t="str">
+        <v>Sent to the person when the team replies to their message from the Submissions page</v>
+      </c>
+      <c r="C818" t="str">
+        <v>Enviado à pessoa quando a equipa responde à sua mensagem na página das Submissões</v>
+      </c>
+      <c r="D818" t="str">
+        <v>Se envía a la persona cuando el equipo responde a su mensaje desde la página de Envíos</v>
+      </c>
+      <c r="E818" t="str">
+        <v>Envoyé à la personne lorsque l’équipe répond à son message depuis la page des Soumissions</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="str">
+        <v>The reply written by the team</v>
+      </c>
+      <c r="B819" t="str">
+        <v>The reply written by the team</v>
+      </c>
+      <c r="C819" t="str">
+        <v>A resposta escrita pela equipa</v>
+      </c>
+      <c r="D819" t="str">
+        <v>La respuesta escrita por el equipo</v>
+      </c>
+      <c r="E819" t="str">
+        <v>La réponse rédigée par l’équipe</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="str">
+        <v>Original message</v>
+      </c>
+      <c r="B820" t="str">
+        <v>Original message</v>
+      </c>
+      <c r="C820" t="str">
+        <v>Mensagem original</v>
+      </c>
+      <c r="D820" t="str">
+        <v>Mensaje original</v>
+      </c>
+      <c r="E820" t="str">
+        <v>Message d’origine</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="str">
+        <v>The message the person sent in the contact form</v>
+      </c>
+      <c r="B821" t="str">
+        <v>The message the person sent in the contact form</v>
+      </c>
+      <c r="C821" t="str">
+        <v>A mensagem que a pessoa enviou no formulário de contacto</v>
+      </c>
+      <c r="D821" t="str">
+        <v>El mensaje que la persona envió en el formulario de contacto</v>
+      </c>
+      <c r="E821" t="str">
+        <v>Le message que la personne a envoyé dans le formulaire de contact</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="str">
+        <v>Current password</v>
+      </c>
+      <c r="B822" t="str">
+        <v>Current password</v>
+      </c>
+      <c r="C822" t="str">
+        <v>Password atual</v>
+      </c>
+      <c r="D822" t="str">
+        <v>Contraseña actual</v>
+      </c>
+      <c r="E822" t="str">
+        <v>Mot de passe actuel</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="str">
+        <v>Enter your current password</v>
+      </c>
+      <c r="B823" t="str">
+        <v>Enter your current password</v>
+      </c>
+      <c r="C823" t="str">
+        <v>Introduza a sua password atual</v>
+      </c>
+      <c r="D823" t="str">
+        <v>Introduzca su contraseña actual</v>
+      </c>
+      <c r="E823" t="str">
+        <v>Saisissez votre mot de passe actuel</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="str">
+        <v>Enter your current password to change it</v>
+      </c>
+      <c r="B824" t="str">
+        <v>Enter your current password to change it</v>
+      </c>
+      <c r="C824" t="str">
+        <v>Introduza a password atual para a alterar</v>
+      </c>
+      <c r="D824" t="str">
+        <v>Introduzca la contraseña actual para cambiarla</v>
+      </c>
+      <c r="E824" t="str">
+        <v>Saisissez le mot de passe actuel pour le modifier</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="str">
+        <v>The current password is incorrect</v>
+      </c>
+      <c r="B825" t="str">
+        <v>The current password is incorrect</v>
+      </c>
+      <c r="C825" t="str">
+        <v>A password atual está incorreta</v>
+      </c>
+      <c r="D825" t="str">
+        <v>La contraseña actual es incorrecta</v>
+      </c>
+      <c r="E825" t="str">
+        <v>Le mot de passe actuel est incorrect</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="str">
+        <v>Save or cancel the row you are editing first</v>
+      </c>
+      <c r="B826" t="str">
+        <v>Save or cancel the row you are editing first</v>
+      </c>
+      <c r="C826" t="str">
+        <v>Guarde ou cancele primeiro a linha que está a editar</v>
+      </c>
+      <c r="D826" t="str">
+        <v>Guarde o cancele primero la fila que está editando</v>
+      </c>
+      <c r="E826" t="str">
+        <v>Enregistrez ou annulez d’abord la ligne en cours de modification</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="str">
+        <v>No changes</v>
+      </c>
+      <c r="B827" t="str">
+        <v>No changes</v>
+      </c>
+      <c r="C827" t="str">
+        <v>Sem alterações</v>
+      </c>
+      <c r="D827" t="str">
+        <v>Sin cambios</v>
+      </c>
+      <c r="E827" t="str">
+        <v>Aucune modification</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="str">
+        <v>Search by key or translation...</v>
+      </c>
+      <c r="B828" t="str">
+        <v>Search by key or translation...</v>
+      </c>
+      <c r="C828" t="str">
+        <v>Pesquisar por chave ou tradução...</v>
+      </c>
+      <c r="D828" t="str">
+        <v>Buscar por clave o traducción...</v>
+      </c>
+      <c r="E828" t="str">
+        <v>Rechercher par clé ou traduction...</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="str">
+        <v>No translations match your search</v>
+      </c>
+      <c r="B829" t="str">
+        <v>No translations match your search</v>
+      </c>
+      <c r="C829" t="str">
+        <v>Nenhuma tradução corresponde à pesquisa</v>
+      </c>
+      <c r="D829" t="str">
+        <v>Ninguna traducción coincide con la búsqueda</v>
+      </c>
+      <c r="E829" t="str">
+        <v>Aucune traduction ne correspond à la recherche</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="str">
+        <v>No translations yet</v>
+      </c>
+      <c r="B830" t="str">
+        <v>No translations yet</v>
+      </c>
+      <c r="C830" t="str">
+        <v>Ainda não há traduções</v>
+      </c>
+      <c r="D830" t="str">
+        <v>Aún no hay traducciones</v>
+      </c>
+      <c r="E830" t="str">
+        <v>Aucune traduction pour l’instant</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="str">
+        <v>Close</v>
+      </c>
+      <c r="B831" t="str">
+        <v>Close</v>
+      </c>
+      <c r="C831" t="str">
+        <v>Fechar</v>
+      </c>
+      <c r="D831" t="str">
+        <v>Cerrar</v>
+      </c>
+      <c r="E831" t="str">
+        <v>Fermer</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="str">
+        <v>Total records</v>
+      </c>
+      <c r="B832" t="str">
+        <v>Total records</v>
+      </c>
+      <c r="C832" t="str">
+        <v>Total de registos</v>
+      </c>
+      <c r="D832" t="str">
+        <v>Total de registros</v>
+      </c>
+      <c r="E832" t="str">
+        <v>Total des enregistrements</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="str">
+        <v>Untitled objection</v>
+      </c>
+      <c r="B833" t="str">
+        <v>Untitled objection</v>
+      </c>
+      <c r="C833" t="str">
+        <v>Objeção sem título</v>
+      </c>
+      <c r="D833" t="str">
+        <v>Objeción sin título</v>
+      </c>
+      <c r="E833" t="str">
+        <v>Objection sans titre</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="str">
+        <v>Group the objections by theme. Each book appears as a tab in the course page</v>
+      </c>
+      <c r="B834" t="str">
+        <v>Group the objections by theme. Each book appears as a tab in the course page</v>
+      </c>
+      <c r="C834" t="str">
+        <v>Agrupe as objeções por tema. Cada livro aparece como um separador na página do curso</v>
+      </c>
+      <c r="D834" t="str">
+        <v>Agrupe las objeciones por tema. Cada libro aparece como una pestaña en la página del curso</v>
+      </c>
+      <c r="E834" t="str">
+        <v>Regroupez les objections par thème. Chaque livre apparaît comme un onglet dans la page du cours</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="str">
+        <v>Name of the book (shown as a tab)</v>
+      </c>
+      <c r="B835" t="str">
+        <v>Name of the book (shown as a tab)</v>
+      </c>
+      <c r="C835" t="str">
+        <v>Nome do livro (mostrado como separador)</v>
+      </c>
+      <c r="D835" t="str">
+        <v>Nombre del libro (se muestra como pestaña)</v>
+      </c>
+      <c r="E835" t="str">
+        <v>Nom du livre (affiché comme onglet)</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="str">
+        <v>Objections: {{count}}</v>
+      </c>
+      <c r="B836" t="str">
+        <v>Objections: {{count}}</v>
+      </c>
+      <c r="C836" t="str">
+        <v>Objeções: {{count}}</v>
+      </c>
+      <c r="D836" t="str">
+        <v>Objeciones: {{count}}</v>
+      </c>
+      <c r="E836" t="str">
+        <v>Objections : {{count}}</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="str">
+        <v>Move up</v>
+      </c>
+      <c r="B837" t="str">
+        <v>Move up</v>
+      </c>
+      <c r="C837" t="str">
+        <v>Mover para cima</v>
+      </c>
+      <c r="D837" t="str">
+        <v>Mover hacia arriba</v>
+      </c>
+      <c r="E837" t="str">
+        <v>Monter</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="str">
+        <v>Move down</v>
+      </c>
+      <c r="B838" t="str">
+        <v>Move down</v>
+      </c>
+      <c r="C838" t="str">
+        <v>Mover para baixo</v>
+      </c>
+      <c r="D838" t="str">
+        <v>Mover hacia abajo</v>
+      </c>
+      <c r="E838" t="str">
+        <v>Descendre</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="str">
+        <v>Delete this objection book?</v>
+      </c>
+      <c r="B839" t="str">
+        <v>Delete this objection book?</v>
+      </c>
+      <c r="C839" t="str">
+        <v>Apagar este livro de objeções?</v>
+      </c>
+      <c r="D839" t="str">
+        <v>¿Eliminar este libro de objeciones?</v>
+      </c>
+      <c r="E839" t="str">
+        <v>Supprimer ce livre d’objections ?</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="str">
+        <v>The book and all its objections are removed when you save the course settings</v>
+      </c>
+      <c r="B840" t="str">
+        <v>The book and all its objections are removed when you save the course settings</v>
+      </c>
+      <c r="C840" t="str">
+        <v>O livro e todas as suas objeções são removidos quando guardar as definições do curso</v>
+      </c>
+      <c r="D840" t="str">
+        <v>El libro y todas sus objeciones se eliminan al guardar la configuración del curso</v>
+      </c>
+      <c r="E840" t="str">
+        <v>Le livre et toutes ses objections sont supprimés lorsque vous enregistrez les paramètres du cours</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="str">
+        <v>Delete this objection?</v>
+      </c>
+      <c r="B841" t="str">
+        <v>Delete this objection?</v>
+      </c>
+      <c r="C841" t="str">
+        <v>Apagar esta objeção?</v>
+      </c>
+      <c r="D841" t="str">
+        <v>¿Eliminar esta objeción?</v>
+      </c>
+      <c r="E841" t="str">
+        <v>Supprimer cette objection ?</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="str">
+        <v>It is removed when you save the course settings</v>
+      </c>
+      <c r="B842" t="str">
+        <v>It is removed when you save the course settings</v>
+      </c>
+      <c r="C842" t="str">
+        <v>É removida quando guardar as definições do curso</v>
+      </c>
+      <c r="D842" t="str">
+        <v>Se elimina al guardar la configuración del curso</v>
+      </c>
+      <c r="E842" t="str">
+        <v>Elle est supprimée lorsque vous enregistrez les paramètres du cours</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="str">
+        <v>Base language</v>
+      </c>
+      <c r="B843" t="str">
+        <v>Base language</v>
+      </c>
+      <c r="C843" t="str">
+        <v>Idioma base</v>
+      </c>
+      <c r="D843" t="str">
+        <v>Idioma base</v>
+      </c>
+      <c r="E843" t="str">
+        <v>Langue de base</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="str">
+        <v>{{count}} missing</v>
+      </c>
+      <c r="B844" t="str">
+        <v>{{count}} missing</v>
+      </c>
+      <c r="C844" t="str">
+        <v>Faltam {{count}}</v>
+      </c>
+      <c r="D844" t="str">
+        <v>Faltan {{count}}</v>
+      </c>
+      <c r="E844" t="str">
+        <v>{{count}} manquantes</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="str">
+        <v>{{total}} languages</v>
+      </c>
+      <c r="B845" t="str">
+        <v>{{total}} languages</v>
+      </c>
+      <c r="C845" t="str">
+        <v>{{total}} idiomas</v>
+      </c>
+      <c r="D845" t="str">
+        <v>{{total}} idiomas</v>
+      </c>
+      <c r="E845" t="str">
+        <v>{{total}} langues</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="str">
+        <v>Search countries...</v>
+      </c>
+      <c r="B846" t="str">
+        <v>Search countries...</v>
+      </c>
+      <c r="C846" t="str">
+        <v>Pesquisar países...</v>
+      </c>
+      <c r="D846" t="str">
+        <v>Buscar países...</v>
+      </c>
+      <c r="E846" t="str">
+        <v>Rechercher des pays...</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="str">
+        <v>Only selected</v>
+      </c>
+      <c r="B847" t="str">
+        <v>Only selected</v>
+      </c>
+      <c r="C847" t="str">
+        <v>Só selecionados</v>
+      </c>
+      <c r="D847" t="str">
+        <v>Solo seleccionados</v>
+      </c>
+      <c r="E847" t="str">
+        <v>Sélectionnés uniquement</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="str">
+        <v>Select all</v>
+      </c>
+      <c r="B848" t="str">
+        <v>Select all</v>
+      </c>
+      <c r="C848" t="str">
+        <v>Selecionar todos</v>
+      </c>
+      <c r="D848" t="str">
+        <v>Seleccionar todos</v>
+      </c>
+      <c r="E848" t="str">
+        <v>Tout sélectionner</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="str">
+        <v>Select shown</v>
+      </c>
+      <c r="B849" t="str">
+        <v>Select shown</v>
+      </c>
+      <c r="C849" t="str">
+        <v>Selecionar os visíveis</v>
+      </c>
+      <c r="D849" t="str">
+        <v>Seleccionar los visibles</v>
+      </c>
+      <c r="E849" t="str">
+        <v>Sélectionner les pays affichés</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="str">
+        <v>Clear all</v>
+      </c>
+      <c r="B850" t="str">
+        <v>Clear all</v>
+      </c>
+      <c r="C850" t="str">
+        <v>Limpar tudo</v>
+      </c>
+      <c r="D850" t="str">
+        <v>Limpiar todo</v>
+      </c>
+      <c r="E850" t="str">
+        <v>Tout effacer</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="str">
+        <v>No countries found</v>
+      </c>
+      <c r="B851" t="str">
+        <v>No countries found</v>
+      </c>
+      <c r="C851" t="str">
+        <v>Nenhum país encontrado</v>
+      </c>
+      <c r="D851" t="str">
+        <v>Ningún país encontrado</v>
+      </c>
+      <c r="E851" t="str">
+        <v>Aucun pays trouvé</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="str">
+        <v>Notification</v>
+      </c>
+      <c r="B852" t="str">
+        <v>Notification</v>
+      </c>
+      <c r="C852" t="str">
+        <v>Notificação</v>
+      </c>
+      <c r="D852" t="str">
+        <v>Notificación</v>
+      </c>
+      <c r="E852" t="str">
+        <v>Notification</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="str">
+        <v>Read by</v>
+      </c>
+      <c r="B853" t="str">
+        <v>Read by</v>
+      </c>
+      <c r="C853" t="str">
+        <v>Lida por</v>
+      </c>
+      <c r="D853" t="str">
+        <v>Leída por</v>
+      </c>
+      <c r="E853" t="str">
+        <v>Lue par</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="str">
+        <v>Created</v>
+      </c>
+      <c r="B854" t="str">
+        <v>Created</v>
+      </c>
+      <c r="C854" t="str">
+        <v>Criada</v>
+      </c>
+      <c r="D854" t="str">
+        <v>Creada</v>
+      </c>
+      <c r="E854" t="str">
+        <v>Créée</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="str">
+        <v>Search by title or description...</v>
+      </c>
+      <c r="B855" t="str">
+        <v>Search by title or description...</v>
+      </c>
+      <c r="C855" t="str">
+        <v>Pesquisar por título ou descrição...</v>
+      </c>
+      <c r="D855" t="str">
+        <v>Buscar por título o descripción...</v>
+      </c>
+      <c r="E855" t="str">
+        <v>Rechercher par titre ou description...</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="str">
+        <v>All countries</v>
+      </c>
+      <c r="B856" t="str">
+        <v>All countries</v>
+      </c>
+      <c r="C856" t="str">
+        <v>Todos os países</v>
+      </c>
+      <c r="D856" t="str">
+        <v>Todos los países</v>
+      </c>
+      <c r="E856" t="str">
+        <v>Tous les pays</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="str">
+        <v>Send this notification now?</v>
+      </c>
+      <c r="B857" t="str">
+        <v>Send this notification now?</v>
+      </c>
+      <c r="C857" t="str">
+        <v>Enviar esta notificação agora?</v>
+      </c>
+      <c r="D857" t="str">
+        <v>¿Enviar esta notificación ahora?</v>
+      </c>
+      <c r="E857" t="str">
+        <v>Envoyer cette notification maintenant ?</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="str">
+        <v>It reaches everyone in the audience right away. This cannot be undone</v>
+      </c>
+      <c r="B858" t="str">
+        <v>It reaches everyone in the audience right away. This cannot be undone</v>
+      </c>
+      <c r="C858" t="str">
+        <v>Chega logo a todas as pessoas do público. Não se pode desfazer</v>
+      </c>
+      <c r="D858" t="str">
+        <v>Llega de inmediato a todas las personas del público. No se puede deshacer</v>
+      </c>
+      <c r="E858" t="str">
+        <v>Elle parvient immédiatement à toutes les personnes du public. Cette action est irréversible</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="str">
+        <v>It reaches {{count}} people right away. This cannot be undone</v>
+      </c>
+      <c r="B859" t="str">
+        <v>It reaches {{count}} people right away. This cannot be undone</v>
+      </c>
+      <c r="C859" t="str">
+        <v>Chega logo a {{count}} pessoas. Não se pode desfazer</v>
+      </c>
+      <c r="D859" t="str">
+        <v>Llega de inmediato a {{count}} personas. No se puede deshacer</v>
+      </c>
+      <c r="E859" t="str">
+        <v>Elle parvient immédiatement à {{count}} personnes. Cette action est irréversible</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="str">
+        <v>Delete this notification?</v>
+      </c>
+      <c r="B860" t="str">
+        <v>Delete this notification?</v>
+      </c>
+      <c r="C860" t="str">
+        <v>Apagar esta notificação?</v>
+      </c>
+      <c r="D860" t="str">
+        <v>¿Eliminar esta notificación?</v>
+      </c>
+      <c r="E860" t="str">
+        <v>Supprimer cette notification ?</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="str">
+        <v>It disappears from the notifications of everyone who received it</v>
+      </c>
+      <c r="B861" t="str">
+        <v>It disappears from the notifications of everyone who received it</v>
+      </c>
+      <c r="C861" t="str">
+        <v>Desaparece das notificações de todas as pessoas que a receberam</v>
+      </c>
+      <c r="D861" t="str">
+        <v>Desaparece de las notificaciones de todas las personas que la recibieron</v>
+      </c>
+      <c r="E861" t="str">
+        <v>Elle disparaît des notifications de toutes les personnes qui l’ont reçue</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="str">
+        <v>Notification deleted</v>
+      </c>
+      <c r="B862" t="str">
+        <v>Notification deleted</v>
+      </c>
+      <c r="C862" t="str">
+        <v>Notificação apagada</v>
+      </c>
+      <c r="D862" t="str">
+        <v>Notificación eliminada</v>
+      </c>
+      <c r="E862" t="str">
+        <v>Notification supprimée</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="str">
+        <v>Notification saved</v>
+      </c>
+      <c r="B863" t="str">
+        <v>Notification saved</v>
+      </c>
+      <c r="C863" t="str">
+        <v>Notificação guardada</v>
+      </c>
+      <c r="D863" t="str">
+        <v>Notificación guardada</v>
+      </c>
+      <c r="E863" t="str">
+        <v>Notification enregistrée</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="str">
+        <v>Notification scheduled for {{date}}</v>
+      </c>
+      <c r="B864" t="str">
+        <v>Notification scheduled for {{date}}</v>
+      </c>
+      <c r="C864" t="str">
+        <v>Notificação agendada para {{date}}</v>
+      </c>
+      <c r="D864" t="str">
+        <v>Notificación programada para {{date}}</v>
+      </c>
+      <c r="E864" t="str">
+        <v>Notification planifiée pour le {{date}}</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="str">
+        <v>What people see in their notifications</v>
+      </c>
+      <c r="B865" t="str">
+        <v>What people see in their notifications</v>
+      </c>
+      <c r="C865" t="str">
+        <v>O que as pessoas veem nas suas notificações</v>
+      </c>
+      <c r="D865" t="str">
+        <v>Lo que las personas ven en sus notificaciones</v>
+      </c>
+      <c r="E865" t="str">
+        <v>Ce que les personnes voient dans leurs notifications</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="str">
+        <v>Approved users of {{language}}</v>
+      </c>
+      <c r="B866" t="str">
+        <v>Approved users of {{language}}</v>
+      </c>
+      <c r="C866" t="str">
+        <v>Utilizadores aprovados de {{language}}</v>
+      </c>
+      <c r="D866" t="str">
+        <v>Usuarios aprobados de {{language}}</v>
+      </c>
+      <c r="E866" t="str">
+        <v>Utilisateurs approuvés de {{language}}</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="str">
+        <v>Leave empty to reach every country of this language</v>
+      </c>
+      <c r="B867" t="str">
+        <v>Leave empty to reach every country of this language</v>
+      </c>
+      <c r="C867" t="str">
+        <v>Deixe vazio para chegar a todos os países deste idioma</v>
+      </c>
+      <c r="D867" t="str">
+        <v>Déjelo vacío para llegar a todos los países de este idioma</v>
+      </c>
+      <c r="E867" t="str">
+        <v>Laissez vide pour atteindre tous les pays de cette langue</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="str">
+        <v>{{count}} people will receive it</v>
+      </c>
+      <c r="B868" t="str">
+        <v>{{count}} people will receive it</v>
+      </c>
+      <c r="C868" t="str">
+        <v>{{count}} pessoas vão recebê-la</v>
+      </c>
+      <c r="D868" t="str">
+        <v>{{count}} personas la recibirán</v>
+      </c>
+      <c r="E868" t="str">
+        <v>{{count}} personnes la recevront</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="str">
+        <v>Sent on {{date}} to {{count}} people</v>
+      </c>
+      <c r="B869" t="str">
+        <v>Sent on {{date}} to {{count}} people</v>
+      </c>
+      <c r="C869" t="str">
+        <v>Enviada a {{date}} para {{count}} pessoas</v>
+      </c>
+      <c r="D869" t="str">
+        <v>Enviada el {{date}} a {{count}} personas</v>
+      </c>
+      <c r="E869" t="str">
+        <v>Envoyée le {{date}} à {{count}} personnes</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="str">
+        <v>The audience and the language can no longer change; you can still correct the text</v>
+      </c>
+      <c r="B870" t="str">
+        <v>The audience and the language can no longer change; you can still correct the text</v>
+      </c>
+      <c r="C870" t="str">
+        <v>O público e o idioma já não se podem alterar; o texto ainda se pode corrigir</v>
+      </c>
+      <c r="D870" t="str">
+        <v>El público y el idioma ya no se pueden cambiar; el texto aún se puede corregir</v>
+      </c>
+      <c r="E870" t="str">
+        <v>Le public et la langue ne peuvent plus changer ; vous pouvez encore corriger le texte</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="str">
+        <v>Save as draft</v>
+      </c>
+      <c r="B871" t="str">
+        <v>Save as draft</v>
+      </c>
+      <c r="C871" t="str">
+        <v>Guardar como rascunho</v>
+      </c>
+      <c r="D871" t="str">
+        <v>Guardar como borrador</v>
+      </c>
+      <c r="E871" t="str">
+        <v>Enregistrer comme brouillon</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="str">
+        <v>Send on</v>
+      </c>
+      <c r="B872" t="str">
+        <v>Send on</v>
+      </c>
+      <c r="C872" t="str">
+        <v>Enviar a</v>
+      </c>
+      <c r="D872" t="str">
+        <v>Enviar el</v>
+      </c>
+      <c r="E872" t="str">
+        <v>Envoyer le</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="str">
+        <v>Choose when to send</v>
+      </c>
+      <c r="B873" t="str">
+        <v>Choose when to send</v>
+      </c>
+      <c r="C873" t="str">
+        <v>Escolha quando enviar</v>
+      </c>
+      <c r="D873" t="str">
+        <v>Elija cuándo enviar</v>
+      </c>
+      <c r="E873" t="str">
+        <v>Choisissez quand envoyer</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="str">
+        <v>Select date and time</v>
+      </c>
+      <c r="B874" t="str">
+        <v>Select date and time</v>
+      </c>
+      <c r="C874" t="str">
+        <v>Selecione a data e a hora</v>
+      </c>
+      <c r="D874" t="str">
+        <v>Seleccione la fecha y la hora</v>
+      </c>
+      <c r="E874" t="str">
+        <v>Sélectionnez la date et l’heure</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="str">
+        <v>Nobody receives it until you send it or schedule it</v>
+      </c>
+      <c r="B875" t="str">
+        <v>Nobody receives it until you send it or schedule it</v>
+      </c>
+      <c r="C875" t="str">
+        <v>Ninguém a recebe até a enviar ou agendar</v>
+      </c>
+      <c r="D875" t="str">
+        <v>Nadie la recibe hasta que la envíe o la programe</v>
+      </c>
+      <c r="E875" t="str">
+        <v>Personne ne la reçoit tant que vous ne l’envoyez pas ou ne la planifiez pas</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="str">
+        <v>It is delivered as soon as you click Send now</v>
+      </c>
+      <c r="B876" t="str">
+        <v>It is delivered as soon as you click Send now</v>
+      </c>
+      <c r="C876" t="str">
+        <v>É entregue assim que clicar em Enviar agora</v>
+      </c>
+      <c r="D876" t="str">
+        <v>Se entrega en cuanto haga clic en Enviar ahora</v>
+      </c>
+      <c r="E876" t="str">
+        <v>Elle est livrée dès que vous cliquez sur Envoyer maintenant</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="str">
+        <v>Desktop</v>
+      </c>
+      <c r="B877" t="str">
+        <v>Desktop</v>
+      </c>
+      <c r="C877" t="str">
+        <v>Computador</v>
+      </c>
+      <c r="D877" t="str">
+        <v>Ordenador</v>
+      </c>
+      <c r="E877" t="str">
+        <v>Ordinateur</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="str">
+        <v>The text you write appears here</v>
+      </c>
+      <c r="B878" t="str">
+        <v>The text you write appears here</v>
+      </c>
+      <c r="C878" t="str">
+        <v>O texto que escrever aparece aqui</v>
+      </c>
+      <c r="D878" t="str">
+        <v>El texto que escriba aparece aquí</v>
+      </c>
+      <c r="E878" t="str">
+        <v>Le texte que vous écrivez apparaît ici</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="str">
+        <v>Homepage text saved</v>
+      </c>
+      <c r="B879" t="str">
+        <v>Homepage text saved</v>
+      </c>
+      <c r="C879" t="str">
+        <v>Texto da página inicial guardado</v>
+      </c>
+      <c r="D879" t="str">
+        <v>Texto de la página de inicio guardado</v>
+      </c>
+      <c r="E879" t="str">
+        <v>Texte de la page d’accueil enregistré</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="str">
+        <v>Replace the current text?</v>
+      </c>
+      <c r="B880" t="str">
+        <v>Replace the current text?</v>
+      </c>
+      <c r="C880" t="str">
+        <v>Substituir o texto atual?</v>
+      </c>
+      <c r="D880" t="str">
+        <v>¿Reemplazar el texto actual?</v>
+      </c>
+      <c r="E880" t="str">
+        <v>Remplacer le texte actuel ?</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="str">
+        <v>The text below is replaced by the one from the other language. Nothing is saved until you click Save</v>
+      </c>
+      <c r="B881" t="str">
+        <v>The text below is replaced by the one from the other language. Nothing is saved until you click Save</v>
+      </c>
+      <c r="C881" t="str">
+        <v>O texto abaixo é substituído pelo do outro idioma. Nada é guardado até clicar em Guardar</v>
+      </c>
+      <c r="D881" t="str">
+        <v>El texto de abajo se reemplaza por el del otro idioma. No se guarda nada hasta que haga clic en Guardar</v>
+      </c>
+      <c r="E881" t="str">
+        <v>Le texte ci-dessous est remplacé par celui de l’autre langue. Rien n’est enregistré tant que vous ne cliquez pas sur Enregistrer</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="str">
+        <v>The content of the public pages, for each language</v>
+      </c>
+      <c r="B882" t="str">
+        <v>The content of the public pages, for each language</v>
+      </c>
+      <c r="C882" t="str">
+        <v>O conteúdo das páginas públicas, para cada idioma</v>
+      </c>
+      <c r="D882" t="str">
+        <v>El contenido de las páginas públicas, para cada idioma</v>
+      </c>
+      <c r="E882" t="str">
+        <v>Le contenu des pages publiques, pour chaque langue</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="str">
+        <v>Editing</v>
+      </c>
+      <c r="B883" t="str">
+        <v>Editing</v>
+      </c>
+      <c r="C883" t="str">
+        <v>A editar</v>
+      </c>
+      <c r="D883" t="str">
+        <v>Editando</v>
+      </c>
+      <c r="E883" t="str">
+        <v>Modification</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="str">
+        <v>You do not have permission to edit this content</v>
+      </c>
+      <c r="B884" t="str">
+        <v>You do not have permission to edit this content</v>
+      </c>
+      <c r="C884" t="str">
+        <v>Não tem permissão para editar este conteúdo</v>
+      </c>
+      <c r="D884" t="str">
+        <v>No tiene permiso para editar este contenido</v>
+      </c>
+      <c r="E884" t="str">
+        <v>Vous n’avez pas la permission de modifier ce contenu</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="str">
+        <v>Homepage text</v>
+      </c>
+      <c r="B885" t="str">
+        <v>Homepage text</v>
+      </c>
+      <c r="C885" t="str">
+        <v>Texto da página inicial</v>
+      </c>
+      <c r="D885" t="str">
+        <v>Texto de la página de inicio</v>
+      </c>
+      <c r="E885" t="str">
+        <v>Texte de la page d’accueil</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="str">
+        <v>The text shown on the homepage, next to the login buttons</v>
+      </c>
+      <c r="B886" t="str">
+        <v>The text shown on the homepage, next to the login buttons</v>
+      </c>
+      <c r="C886" t="str">
+        <v>O texto mostrado na página inicial, junto aos botões de entrada</v>
+      </c>
+      <c r="D886" t="str">
+        <v>El texto que se muestra en la página de inicio, junto a los botones de acceso</v>
+      </c>
+      <c r="E886" t="str">
+        <v>Le texte affiché sur la page d’accueil, à côté des boutons de connexion</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="str">
+        <v>Start from another language</v>
+      </c>
+      <c r="B887" t="str">
+        <v>Start from another language</v>
+      </c>
+      <c r="C887" t="str">
+        <v>Começar a partir de outro idioma</v>
+      </c>
+      <c r="D887" t="str">
+        <v>Empezar desde otro idioma</v>
+      </c>
+      <c r="E887" t="str">
+        <v>Partir d’une autre langue</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="str">
+        <v>Copy the text from...</v>
+      </c>
+      <c r="B888" t="str">
+        <v>Copy the text from...</v>
+      </c>
+      <c r="C888" t="str">
+        <v>Copiar o texto de...</v>
+      </c>
+      <c r="D888" t="str">
+        <v>Copiar el texto de...</v>
+      </c>
+      <c r="E888" t="str">
+        <v>Copier le texte de...</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="str">
+        <v>No text yet</v>
+      </c>
+      <c r="B889" t="str">
+        <v>No text yet</v>
+      </c>
+      <c r="C889" t="str">
+        <v>Sem texto</v>
+      </c>
+      <c r="D889" t="str">
+        <v>Sin texto</v>
+      </c>
+      <c r="E889" t="str">
+        <v>Pas de texte</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="str">
+        <v>With text</v>
+      </c>
+      <c r="B890" t="str">
+        <v>With text</v>
+      </c>
+      <c r="C890" t="str">
+        <v>Com texto</v>
+      </c>
+      <c r="D890" t="str">
+        <v>Con texto</v>
+      </c>
+      <c r="E890" t="str">
+        <v>Avec texte</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="str">
+        <v>Which languages already have a homepage text</v>
+      </c>
+      <c r="B891" t="str">
+        <v>Which languages already have a homepage text</v>
+      </c>
+      <c r="C891" t="str">
+        <v>Que idiomas já têm texto na página inicial</v>
+      </c>
+      <c r="D891" t="str">
+        <v>Qué idiomas ya tienen texto en la página de inicio</v>
+      </c>
+      <c r="E891" t="str">
+        <v>Quelles langues ont déjà un texte d’accueil</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="str">
+        <v>Without a text, the homepage shows the default welcome message</v>
+      </c>
+      <c r="B892" t="str">
+        <v>Without a text, the homepage shows the default welcome message</v>
+      </c>
+      <c r="C892" t="str">
+        <v>Sem texto, a página inicial mostra a mensagem de boas-vindas por omissão</v>
+      </c>
+      <c r="D892" t="str">
+        <v>Sin texto, la página de inicio muestra el mensaje de bienvenida por defecto</v>
+      </c>
+      <c r="E892" t="str">
+        <v>Sans texte, la page d’accueil affiche le message de bienvenue par défaut</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E651"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E892"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: deploy notes for JWT_SECRET, CORS, TRUST_PROXY and the security_block migration; new translation keys
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E892"/>
+  <dimension ref="A1:E915"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -15563,9 +15563,400 @@
         <v>Sans texte, la page d’accueil affiche le message de bienvenue par défaut</v>
       </c>
     </row>
+    <row r="893">
+      <c r="A893" t="str">
+        <v>The password must have at least {{count}} characters</v>
+      </c>
+      <c r="B893" t="str">
+        <v>The password must have at least {{count}} characters</v>
+      </c>
+      <c r="C893" t="str">
+        <v>A password deve ter pelo menos {{count}} caracteres</v>
+      </c>
+      <c r="D893" t="str">
+        <v>La contraseña debe tener al menos {{count}} caracteres</v>
+      </c>
+      <c r="E893" t="str">
+        <v>Le mot de passe doit contenir au moins {{count}} caractères</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="str">
+        <v>The password must have at least 8 characters</v>
+      </c>
+      <c r="B894" t="str">
+        <v>The password must have at least 8 characters</v>
+      </c>
+      <c r="C894" t="str">
+        <v>A password deve ter pelo menos 8 caracteres</v>
+      </c>
+      <c r="D894" t="str">
+        <v>La contraseña debe tener al menos 8 caracteres</v>
+      </c>
+      <c r="E894" t="str">
+        <v>Le mot de passe doit contenir au moins 8 caractères</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="str">
+        <v>Too many attempts, try again in a few minutes.</v>
+      </c>
+      <c r="B895" t="str">
+        <v>Too many attempts, try again in a few minutes.</v>
+      </c>
+      <c r="C895" t="str">
+        <v>Demasiadas tentativas, tente novamente dentro de alguns minutos.</v>
+      </c>
+      <c r="D895" t="str">
+        <v>Demasiados intentos, inténtelo de nuevo en unos minutos.</v>
+      </c>
+      <c r="E895" t="str">
+        <v>Trop de tentatives, réessayez dans quelques minutes.</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="str">
+        <v>Too many messages, try again later</v>
+      </c>
+      <c r="B896" t="str">
+        <v>Too many messages, try again later</v>
+      </c>
+      <c r="C896" t="str">
+        <v>Demasiadas mensagens, tente novamente mais tarde</v>
+      </c>
+      <c r="D896" t="str">
+        <v>Demasiados mensajes, inténtelo de nuevo más tarde</v>
+      </c>
+      <c r="E896" t="str">
+        <v>Trop de messages, réessayez plus tard</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="str">
+        <v>Blocks</v>
+      </c>
+      <c r="B897" t="str">
+        <v>Blocks</v>
+      </c>
+      <c r="C897" t="str">
+        <v>Bloqueios</v>
+      </c>
+      <c r="D897" t="str">
+        <v>Bloqueos</v>
+      </c>
+      <c r="E897" t="str">
+        <v>Blocages</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="str">
+        <v>Unblocked</v>
+      </c>
+      <c r="B898" t="str">
+        <v>Unblocked</v>
+      </c>
+      <c r="C898" t="str">
+        <v>Desbloqueado</v>
+      </c>
+      <c r="D898" t="str">
+        <v>Desbloqueado</v>
+      </c>
+      <c r="E898" t="str">
+        <v>Débloqué</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="str">
+        <v>All unblocked</v>
+      </c>
+      <c r="B899" t="str">
+        <v>All unblocked</v>
+      </c>
+      <c r="C899" t="str">
+        <v>Tudo desbloqueado</v>
+      </c>
+      <c r="D899" t="str">
+        <v>Todo desbloqueado</v>
+      </c>
+      <c r="E899" t="str">
+        <v>Tout débloqué</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="str">
+        <v>Unblock everyone?</v>
+      </c>
+      <c r="B900" t="str">
+        <v>Unblock everyone?</v>
+      </c>
+      <c r="C900" t="str">
+        <v>Desbloquear todos?</v>
+      </c>
+      <c r="D900" t="str">
+        <v>¿Desbloquear a todos?</v>
+      </c>
+      <c r="E900" t="str">
+        <v>Débloquer tout le monde ?</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="str">
+        <v>All blocks and failed-attempt counters are cleared</v>
+      </c>
+      <c r="B901" t="str">
+        <v>All blocks and failed-attempt counters are cleared</v>
+      </c>
+      <c r="C901" t="str">
+        <v>Todos os bloqueios e contadores de tentativas falhadas são limpos</v>
+      </c>
+      <c r="D901" t="str">
+        <v>Se borran todos los bloqueos y contadores de intentos fallidos</v>
+      </c>
+      <c r="E901" t="str">
+        <v>Tous les blocages et compteurs de tentatives échouées sont effacés</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="str">
+        <v>Unblock all</v>
+      </c>
+      <c r="B902" t="str">
+        <v>Unblock all</v>
+      </c>
+      <c r="C902" t="str">
+        <v>Desbloquear todos</v>
+      </c>
+      <c r="D902" t="str">
+        <v>Desbloquear todos</v>
+      </c>
+      <c r="E902" t="str">
+        <v>Tout débloquer</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="str">
+        <v>Unblock</v>
+      </c>
+      <c r="B903" t="str">
+        <v>Unblock</v>
+      </c>
+      <c r="C903" t="str">
+        <v>Desbloquear</v>
+      </c>
+      <c r="D903" t="str">
+        <v>Desbloquear</v>
+      </c>
+      <c r="E903" t="str">
+        <v>Débloquer</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="str">
+        <v>Blocked now</v>
+      </c>
+      <c r="B904" t="str">
+        <v>Blocked now</v>
+      </c>
+      <c r="C904" t="str">
+        <v>Bloqueados agora</v>
+      </c>
+      <c r="D904" t="str">
+        <v>Bloqueados ahora</v>
+      </c>
+      <c r="E904" t="str">
+        <v>Bloqués actuellement</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="str">
+        <v>With failed attempts</v>
+      </c>
+      <c r="B905" t="str">
+        <v>With failed attempts</v>
+      </c>
+      <c r="C905" t="str">
+        <v>Com tentativas falhadas</v>
+      </c>
+      <c r="D905" t="str">
+        <v>Con intentos fallidos</v>
+      </c>
+      <c r="E905" t="str">
+        <v>Avec tentatives échouées</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="str">
+        <v>Failed attempts</v>
+      </c>
+      <c r="B906" t="str">
+        <v>Failed attempts</v>
+      </c>
+      <c r="C906" t="str">
+        <v>Tentativas falhadas</v>
+      </c>
+      <c r="D906" t="str">
+        <v>Intentos fallidos</v>
+      </c>
+      <c r="E906" t="str">
+        <v>Tentatives échouées</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="str">
+        <v>Blocked until {{time}}</v>
+      </c>
+      <c r="B907" t="str">
+        <v>Blocked until {{time}}</v>
+      </c>
+      <c r="C907" t="str">
+        <v>Bloqueado até às {{time}}</v>
+      </c>
+      <c r="D907" t="str">
+        <v>Bloqueado hasta las {{time}}</v>
+      </c>
+      <c r="E907" t="str">
+        <v>Bloqué jusqu’à {{time}}</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="str">
+        <v>After too many failed attempts an e-mail or an IP is blocked for a few minutes. Unblock real users here</v>
+      </c>
+      <c r="B908" t="str">
+        <v>After too many failed attempts an e-mail or an IP is blocked for a few minutes. Unblock real users here</v>
+      </c>
+      <c r="C908" t="str">
+        <v>Depois de demasiadas tentativas falhadas, um e-mail ou um IP fica bloqueado alguns minutos. Desbloqueie aqui os utilizadores reais</v>
+      </c>
+      <c r="D908" t="str">
+        <v>Tras demasiados intentos fallidos, un correo o una IP queda bloqueado unos minutos. Desbloquee aquí a los usuarios reales</v>
+      </c>
+      <c r="E908" t="str">
+        <v>Après trop de tentatives échouées, un e-mail ou une IP est bloqué quelques minutes. Débloquez ici les vrais utilisateurs</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="str">
+        <v>Blocks are not available yet: the database migration is pending. Until then the limits work in memory and cannot be listed</v>
+      </c>
+      <c r="B909" t="str">
+        <v>Blocks are not available yet: the database migration is pending. Until then the limits work in memory and cannot be listed</v>
+      </c>
+      <c r="C909" t="str">
+        <v>Os bloqueios ainda não estão disponíveis: falta a migração da base de dados. Até lá os limites funcionam em memória e não se podem listar</v>
+      </c>
+      <c r="D909" t="str">
+        <v>Los bloqueos aún no están disponibles: falta la migración de la base de datos. Hasta entonces los límites funcionan en memoria y no se pueden listar</v>
+      </c>
+      <c r="E909" t="str">
+        <v>Les blocages ne sont pas encore disponibles : la migration de la base de données est en attente. D’ici là, les limites fonctionnent en mémoire et ne peuvent pas être listées</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="str">
+        <v>No blocks or failed attempts</v>
+      </c>
+      <c r="B910" t="str">
+        <v>No blocks or failed attempts</v>
+      </c>
+      <c r="C910" t="str">
+        <v>Sem bloqueios nem tentativas falhadas</v>
+      </c>
+      <c r="D910" t="str">
+        <v>Sin bloqueos ni intentos fallidos</v>
+      </c>
+      <c r="E910" t="str">
+        <v>Aucun blocage ni tentative échouée</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="str">
+        <v>E-mail / IP</v>
+      </c>
+      <c r="B911" t="str">
+        <v>E-mail / IP</v>
+      </c>
+      <c r="C911" t="str">
+        <v>E-mail / IP</v>
+      </c>
+      <c r="D911" t="str">
+        <v>Correo / IP</v>
+      </c>
+      <c r="E911" t="str">
+        <v>E-mail / IP</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="str">
+        <v>Attempts</v>
+      </c>
+      <c r="B912" t="str">
+        <v>Attempts</v>
+      </c>
+      <c r="C912" t="str">
+        <v>Tentativas</v>
+      </c>
+      <c r="D912" t="str">
+        <v>Intentos</v>
+      </c>
+      <c r="E912" t="str">
+        <v>Tentatives</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="str">
+        <v>Last attempt</v>
+      </c>
+      <c r="B913" t="str">
+        <v>Last attempt</v>
+      </c>
+      <c r="C913" t="str">
+        <v>Última tentativa</v>
+      </c>
+      <c r="D913" t="str">
+        <v>Último intento</v>
+      </c>
+      <c r="E913" t="str">
+        <v>Dernière tentative</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="str">
+        <v>Recovery code</v>
+      </c>
+      <c r="B914" t="str">
+        <v>Recovery code</v>
+      </c>
+      <c r="C914" t="str">
+        <v>Código de recuperação</v>
+      </c>
+      <c r="D914" t="str">
+        <v>Código de recuperación</v>
+      </c>
+      <c r="E914" t="str">
+        <v>Code de récupération</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="str">
+        <v>Recovery requests</v>
+      </c>
+      <c r="B915" t="str">
+        <v>Recovery requests</v>
+      </c>
+      <c r="C915" t="str">
+        <v>Pedidos de recuperação</v>
+      </c>
+      <c r="D915" t="str">
+        <v>Solicitudes de recuperación</v>
+      </c>
+      <c r="E915" t="str">
+        <v>Demandes de récupération</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E892"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E915"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: shared config (CORS, trust proxy, rate limit per IP, audit hook), indexes migration, endpoints, translations source and deploy notes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E915"/>
+  <dimension ref="A1:E960"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -15954,9 +15954,774 @@
         <v>Demandes de récupération</v>
       </c>
     </row>
+    <row r="916">
+      <c r="A916" t="str">
+        <v>Could not load the dashboard, try again</v>
+      </c>
+      <c r="B916" t="str">
+        <v>Could not load the dashboard, try again</v>
+      </c>
+      <c r="C916" t="str">
+        <v>Não foi possível carregar o painel, tente novamente</v>
+      </c>
+      <c r="D916" t="str">
+        <v>No se pudo cargar el panel, inténtelo de nuevo</v>
+      </c>
+      <c r="E916" t="str">
+        <v>Impossible de charger le tableau de bord, réessayez</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="str">
+        <v>Completed on {{date}}</v>
+      </c>
+      <c r="B917" t="str">
+        <v>Completed on {{date}}</v>
+      </c>
+      <c r="C917" t="str">
+        <v>Concluído a {{date}}</v>
+      </c>
+      <c r="D917" t="str">
+        <v>Completado el {{date}}</v>
+      </c>
+      <c r="E917" t="str">
+        <v>Terminé le {{date}}</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="str">
+        <v>Search course...</v>
+      </c>
+      <c r="B918" t="str">
+        <v>Search course...</v>
+      </c>
+      <c r="C918" t="str">
+        <v>Pesquisar curso...</v>
+      </c>
+      <c r="D918" t="str">
+        <v>Buscar curso...</v>
+      </c>
+      <c r="E918" t="str">
+        <v>Rechercher un cours...</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="str">
+        <v>No courses match your search</v>
+      </c>
+      <c r="B919" t="str">
+        <v>No courses match your search</v>
+      </c>
+      <c r="C919" t="str">
+        <v>Nenhum curso corresponde à pesquisa</v>
+      </c>
+      <c r="D919" t="str">
+        <v>Ningún curso coincide con la búsqueda</v>
+      </c>
+      <c r="E919" t="str">
+        <v>Aucun cours ne correspond à la recherche</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="str">
+        <v>No users found</v>
+      </c>
+      <c r="B920" t="str">
+        <v>No users found</v>
+      </c>
+      <c r="C920" t="str">
+        <v>Nenhum utilizador encontrado</v>
+      </c>
+      <c r="D920" t="str">
+        <v>Ningún usuario encontrado</v>
+      </c>
+      <c r="E920" t="str">
+        <v>Aucun utilisateur trouvé</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="str">
+        <v>Slow request</v>
+      </c>
+      <c r="B921" t="str">
+        <v>Slow request</v>
+      </c>
+      <c r="C921" t="str">
+        <v>Pedido lento</v>
+      </c>
+      <c r="D921" t="str">
+        <v>Solicitud lenta</v>
+      </c>
+      <c r="E921" t="str">
+        <v>Requête lente</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="str">
+        <v>Error loading translations</v>
+      </c>
+      <c r="B922" t="str">
+        <v>Error loading translations</v>
+      </c>
+      <c r="C922" t="str">
+        <v>Erro ao carregar as traduções</v>
+      </c>
+      <c r="D922" t="str">
+        <v>Error al cargar las traducciones</v>
+      </c>
+      <c r="E922" t="str">
+        <v>Erreur lors du chargement des traductions</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="str">
+        <v>Sent to</v>
+      </c>
+      <c r="B923" t="str">
+        <v>Sent to</v>
+      </c>
+      <c r="C923" t="str">
+        <v>Enviado para</v>
+      </c>
+      <c r="D923" t="str">
+        <v>Enviado a</v>
+      </c>
+      <c r="E923" t="str">
+        <v>Envoyé à</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="str">
+        <v>User</v>
+      </c>
+      <c r="B924" t="str">
+        <v>User</v>
+      </c>
+      <c r="C924" t="str">
+        <v>Utilizador</v>
+      </c>
+      <c r="D924" t="str">
+        <v>Usuario</v>
+      </c>
+      <c r="E924" t="str">
+        <v>Utilisateur</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="str">
+        <v>Team</v>
+      </c>
+      <c r="B925" t="str">
+        <v>Team</v>
+      </c>
+      <c r="C925" t="str">
+        <v>Equipa</v>
+      </c>
+      <c r="D925" t="str">
+        <v>Equipo</v>
+      </c>
+      <c r="E925" t="str">
+        <v>Équipe</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="str">
+        <v>Chosen when sending</v>
+      </c>
+      <c r="B926" t="str">
+        <v>Chosen when sending</v>
+      </c>
+      <c r="C926" t="str">
+        <v>Escolhido ao enviar</v>
+      </c>
+      <c r="D926" t="str">
+        <v>Se elige al enviar</v>
+      </c>
+      <c r="E926" t="str">
+        <v>Choisi à l’envoi</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="str">
+        <v>Sent to the person the e-mail is about</v>
+      </c>
+      <c r="B927" t="str">
+        <v>Sent to the person the e-mail is about</v>
+      </c>
+      <c r="C927" t="str">
+        <v>Enviado à pessoa a que o e-mail diz respeito</v>
+      </c>
+      <c r="D927" t="str">
+        <v>Se envía a la persona a la que se refiere el correo</v>
+      </c>
+      <c r="E927" t="str">
+        <v>Envoyé à la personne concernée par l’e-mail</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="str">
+        <v>Sent to the team (administrators), not to the user</v>
+      </c>
+      <c r="B928" t="str">
+        <v>Sent to the team (administrators), not to the user</v>
+      </c>
+      <c r="C928" t="str">
+        <v>Enviado à equipa (administradores), não ao utilizador</v>
+      </c>
+      <c r="D928" t="str">
+        <v>Se envía al equipo (administradores), no al usuario</v>
+      </c>
+      <c r="E928" t="str">
+        <v>Envoyé à l’équipe (administrateurs), pas à l’utilisateur</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="str">
+        <v>The audience is chosen in Communications when it is sent</v>
+      </c>
+      <c r="B929" t="str">
+        <v>The audience is chosen in Communications when it is sent</v>
+      </c>
+      <c r="C929" t="str">
+        <v>O público escolhe-se nas Comunicações quando é enviado</v>
+      </c>
+      <c r="D929" t="str">
+        <v>El público se elige en Comunicaciones al enviarlo</v>
+      </c>
+      <c r="E929" t="str">
+        <v>Le public est choisi dans Communications lors de l’envoi</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="str">
+        <v>New registration (team)</v>
+      </c>
+      <c r="B930" t="str">
+        <v>New registration (team)</v>
+      </c>
+      <c r="C930" t="str">
+        <v>Novo registo (equipa)</v>
+      </c>
+      <c r="D930" t="str">
+        <v>Nuevo registro (equipo)</v>
+      </c>
+      <c r="E930" t="str">
+        <v>Nouvelle inscription (équipe)</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="str">
+        <v>Sent to the team when someone registers and the account waits for approval</v>
+      </c>
+      <c r="B931" t="str">
+        <v>Sent to the team when someone registers and the account waits for approval</v>
+      </c>
+      <c r="C931" t="str">
+        <v>Enviado à equipa quando alguém se regista e a conta aguarda aprovação</v>
+      </c>
+      <c r="D931" t="str">
+        <v>Se envía al equipo cuando alguien se registra y la cuenta espera aprobación</v>
+      </c>
+      <c r="E931" t="str">
+        <v>Envoyé à l’équipe lorsque quelqu’un s’inscrit et que le compte attend l’approbation</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="str">
+        <v>New request (team)</v>
+      </c>
+      <c r="B932" t="str">
+        <v>New request (team)</v>
+      </c>
+      <c r="C932" t="str">
+        <v>Novo pedido (equipa)</v>
+      </c>
+      <c r="D932" t="str">
+        <v>Nueva solicitud (equipo)</v>
+      </c>
+      <c r="E932" t="str">
+        <v>Nouvelle demande (équipe)</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="str">
+        <v>Sent to the team when someone opens a ticket</v>
+      </c>
+      <c r="B933" t="str">
+        <v>Sent to the team when someone opens a ticket</v>
+      </c>
+      <c r="C933" t="str">
+        <v>Enviado à equipa quando alguém abre um pedido</v>
+      </c>
+      <c r="D933" t="str">
+        <v>Se envía al equipo cuando alguien abre una solicitud</v>
+      </c>
+      <c r="E933" t="str">
+        <v>Envoyé à l’équipe lorsque quelqu’un ouvre une demande</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="str">
+        <v>Reply to a request (team)</v>
+      </c>
+      <c r="B934" t="str">
+        <v>Reply to a request (team)</v>
+      </c>
+      <c r="C934" t="str">
+        <v>Resposta a um pedido (equipa)</v>
+      </c>
+      <c r="D934" t="str">
+        <v>Respuesta a una solicitud (equipo)</v>
+      </c>
+      <c r="E934" t="str">
+        <v>Réponse à une demande (équipe)</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="str">
+        <v>Sent to whoever has the ticket assigned (or to the team) when the person replies to their ticket</v>
+      </c>
+      <c r="B935" t="str">
+        <v>Sent to whoever has the ticket assigned (or to the team) when the person replies to their ticket</v>
+      </c>
+      <c r="C935" t="str">
+        <v>Enviado a quem tem o pedido atribuído (ou à equipa) quando a pessoa responde ao seu pedido</v>
+      </c>
+      <c r="D935" t="str">
+        <v>Se envía a quien tiene asignada la solicitud (o al equipo) cuando la persona responde a su solicitud</v>
+      </c>
+      <c r="E935" t="str">
+        <v>Envoyé à la personne à qui la demande est assignée (ou à l’équipe) lorsque la personne répond à sa demande</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="str">
+        <v>The country of the person who registered</v>
+      </c>
+      <c r="B936" t="str">
+        <v>The country of the person who registered</v>
+      </c>
+      <c r="C936" t="str">
+        <v>O país da pessoa que se registou</v>
+      </c>
+      <c r="D936" t="str">
+        <v>El país de la persona que se registró</v>
+      </c>
+      <c r="E936" t="str">
+        <v>Le pays de la personne qui s’est inscrite</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="str">
+        <v>The name of the person the e-mail is about (in the team e-mails, the person who registered or wrote)</v>
+      </c>
+      <c r="B937" t="str">
+        <v>The name of the person the e-mail is about (in the team e-mails, the person who registered or wrote)</v>
+      </c>
+      <c r="C937" t="str">
+        <v>O nome da pessoa a quem o e-mail diz respeito (nos e-mails da equipa, quem se registou ou escreveu)</v>
+      </c>
+      <c r="D937" t="str">
+        <v>El nombre de la persona a la que se refiere el correo (en los correos del equipo, quien se registró o escribió)</v>
+      </c>
+      <c r="E937" t="str">
+        <v>Le nom de la personne concernée par l’e-mail (dans les e-mails de l’équipe, la personne qui s’est inscrite ou a écrit)</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="str">
+        <v>The e-mail address of the person the e-mail is about (in the team e-mails, the person who registered or wrote)</v>
+      </c>
+      <c r="B938" t="str">
+        <v>The e-mail address of the person the e-mail is about (in the team e-mails, the person who registered or wrote)</v>
+      </c>
+      <c r="C938" t="str">
+        <v>O endereço de e-mail da pessoa a quem o e-mail diz respeito (nos e-mails da equipa, quem se registou ou escreveu)</v>
+      </c>
+      <c r="D938" t="str">
+        <v>La dirección de correo de la persona a la que se refiere el correo (en los correos del equipo, quien se registró o escribió)</v>
+      </c>
+      <c r="E938" t="str">
+        <v>L’adresse e-mail de la personne concernée par l’e-mail (dans les e-mails de l’équipe, la personne qui s’est inscrite ou a écrit)</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="str">
+        <v>Activity</v>
+      </c>
+      <c r="B939" t="str">
+        <v>Activity</v>
+      </c>
+      <c r="C939" t="str">
+        <v>Atividade</v>
+      </c>
+      <c r="D939" t="str">
+        <v>Actividad</v>
+      </c>
+      <c r="E939" t="str">
+        <v>Activité</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="str">
+        <v>Person</v>
+      </c>
+      <c r="B940" t="str">
+        <v>Person</v>
+      </c>
+      <c r="C940" t="str">
+        <v>Pessoa</v>
+      </c>
+      <c r="D940" t="str">
+        <v>Persona</v>
+      </c>
+      <c r="E940" t="str">
+        <v>Personne</v>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="str">
+        <v>Action</v>
+      </c>
+      <c r="B941" t="str">
+        <v>Action</v>
+      </c>
+      <c r="C941" t="str">
+        <v>Ação</v>
+      </c>
+      <c r="D941" t="str">
+        <v>Acción</v>
+      </c>
+      <c r="E941" t="str">
+        <v>Action</v>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="str">
+        <v>Section</v>
+      </c>
+      <c r="B942" t="str">
+        <v>Section</v>
+      </c>
+      <c r="C942" t="str">
+        <v>Secção</v>
+      </c>
+      <c r="D942" t="str">
+        <v>Sección</v>
+      </c>
+      <c r="E942" t="str">
+        <v>Section</v>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="str">
+        <v>Record</v>
+      </c>
+      <c r="B943" t="str">
+        <v>Record</v>
+      </c>
+      <c r="C943" t="str">
+        <v>Registo</v>
+      </c>
+      <c r="D943" t="str">
+        <v>Registro</v>
+      </c>
+      <c r="E943" t="str">
+        <v>Enregistrement</v>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="str">
+        <v>Updated</v>
+      </c>
+      <c r="B944" t="str">
+        <v>Updated</v>
+      </c>
+      <c r="C944" t="str">
+        <v>Atualizado</v>
+      </c>
+      <c r="D944" t="str">
+        <v>Actualizado</v>
+      </c>
+      <c r="E944" t="str">
+        <v>Modifié</v>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="str">
+        <v>Before</v>
+      </c>
+      <c r="B945" t="str">
+        <v>Before</v>
+      </c>
+      <c r="C945" t="str">
+        <v>Antes</v>
+      </c>
+      <c r="D945" t="str">
+        <v>Antes</v>
+      </c>
+      <c r="E945" t="str">
+        <v>Avant</v>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="str">
+        <v>After</v>
+      </c>
+      <c r="B946" t="str">
+        <v>After</v>
+      </c>
+      <c r="C946" t="str">
+        <v>Depois</v>
+      </c>
+      <c r="D946" t="str">
+        <v>Después</v>
+      </c>
+      <c r="E946" t="str">
+        <v>Après</v>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="str">
+        <v>No activity recorded</v>
+      </c>
+      <c r="B947" t="str">
+        <v>No activity recorded</v>
+      </c>
+      <c r="C947" t="str">
+        <v>Sem atividade registada</v>
+      </c>
+      <c r="D947" t="str">
+        <v>Sin actividad registrada</v>
+      </c>
+      <c r="E947" t="str">
+        <v>Aucune activité enregistrée</v>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="str">
+        <v>Search by record, id or address...</v>
+      </c>
+      <c r="B948" t="str">
+        <v>Search by record, id or address...</v>
+      </c>
+      <c r="C948" t="str">
+        <v>Pesquisar por registo, id ou endereço...</v>
+      </c>
+      <c r="D948" t="str">
+        <v>Buscar por registro, id o dirección...</v>
+      </c>
+      <c r="E948" t="str">
+        <v>Rechercher par enregistrement, id ou adresse...</v>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="str">
+        <v>The activity log is not available yet: the database migration is pending</v>
+      </c>
+      <c r="B949" t="str">
+        <v>The activity log is not available yet: the database migration is pending</v>
+      </c>
+      <c r="C949" t="str">
+        <v>O registo de atividade ainda não está disponível: falta a migração da base de dados</v>
+      </c>
+      <c r="D949" t="str">
+        <v>El registro de actividad aún no está disponible: falta la migración de la base de datos</v>
+      </c>
+      <c r="E949" t="str">
+        <v>Le journal d’activité n’est pas encore disponible : la migration de la base de données est en attente</v>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="str">
+        <v>Permissions</v>
+      </c>
+      <c r="B950" t="str">
+        <v>Permissions</v>
+      </c>
+      <c r="C950" t="str">
+        <v>Permissões</v>
+      </c>
+      <c r="D950" t="str">
+        <v>Permisos</v>
+      </c>
+      <c r="E950" t="str">
+        <v>Permissions</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="str">
+        <v>E-mail library</v>
+      </c>
+      <c r="B951" t="str">
+        <v>E-mail library</v>
+      </c>
+      <c r="C951" t="str">
+        <v>Biblioteca de e-mails</v>
+      </c>
+      <c r="D951" t="str">
+        <v>Biblioteca de correos</v>
+      </c>
+      <c r="E951" t="str">
+        <v>Bibliothèque d’e-mails</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="str">
+        <v>Settings</v>
+      </c>
+      <c r="B952" t="str">
+        <v>Settings</v>
+      </c>
+      <c r="C952" t="str">
+        <v>Definições</v>
+      </c>
+      <c r="D952" t="str">
+        <v>Configuración</v>
+      </c>
+      <c r="E952" t="str">
+        <v>Paramètres</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="str">
+        <v>Submissions</v>
+      </c>
+      <c r="B953" t="str">
+        <v>Submissions</v>
+      </c>
+      <c r="C953" t="str">
+        <v>Submissões</v>
+      </c>
+      <c r="D953" t="str">
+        <v>Envíos</v>
+      </c>
+      <c r="E953" t="str">
+        <v>Soumissions</v>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="str">
+        <v>Import</v>
+      </c>
+      <c r="B954" t="str">
+        <v>Import</v>
+      </c>
+      <c r="C954" t="str">
+        <v>Importar</v>
+      </c>
+      <c r="D954" t="str">
+        <v>Importar</v>
+      </c>
+      <c r="E954" t="str">
+        <v>Importer</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="str">
+        <v>Each template is sent by an action of the platform</v>
+      </c>
+      <c r="B955" t="str">
+        <v>Each template is sent by an action of the platform</v>
+      </c>
+      <c r="C955" t="str">
+        <v>Cada template é enviado por uma ação da plataforma</v>
+      </c>
+      <c r="D955" t="str">
+        <v>Cada plantilla se envía por una acción de la plataforma</v>
+      </c>
+      <c r="E955" t="str">
+        <v>Chaque modèle est envoyé par une action de la plateforme</v>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="str">
+        <v>Not sent automatically</v>
+      </c>
+      <c r="B956" t="str">
+        <v>Not sent automatically</v>
+      </c>
+      <c r="C956" t="str">
+        <v>Não é enviado automaticamente</v>
+      </c>
+      <c r="D956" t="str">
+        <v>No se envía automáticamente</v>
+      </c>
+      <c r="E956" t="str">
+        <v>Non envoyé automatiquement</v>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="str">
+        <v>This template is not linked to an action of the platform</v>
+      </c>
+      <c r="B957" t="str">
+        <v>This template is not linked to an action of the platform</v>
+      </c>
+      <c r="C957" t="str">
+        <v>Este template não está ligado a uma ação da plataforma</v>
+      </c>
+      <c r="D957" t="str">
+        <v>Esta plantilla no está vinculada a una acción de la plataforma</v>
+      </c>
+      <c r="E957" t="str">
+        <v>Ce modèle n’est lié à aucune action de la plateforme</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="str">
+        <v>Activity log</v>
+      </c>
+      <c r="B958" t="str">
+        <v>Activity log</v>
+      </c>
+      <c r="C958" t="str">
+        <v>Registo de atividade</v>
+      </c>
+      <c r="D958" t="str">
+        <v>Registro de actividad</v>
+      </c>
+      <c r="E958" t="str">
+        <v>Journal d’activité</v>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="str">
+        <v>Blocked access</v>
+      </c>
+      <c r="B959" t="str">
+        <v>Blocked access</v>
+      </c>
+      <c r="C959" t="str">
+        <v>Acessos bloqueados</v>
+      </c>
+      <c r="D959" t="str">
+        <v>Accesos bloqueados</v>
+      </c>
+      <c r="E959" t="str">
+        <v>Accès bloqués</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="str">
+        <v>Mark as unresolved</v>
+      </c>
+      <c r="B960" t="str">
+        <v>Mark as unresolved</v>
+      </c>
+      <c r="C960" t="str">
+        <v>Marcar como por resolver</v>
+      </c>
+      <c r="D960" t="str">
+        <v>Marcar como sin resolver</v>
+      </c>
+      <c r="E960" t="str">
+        <v>Marquer comme non résolu</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E915"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E960"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(tests): dates in Lisbon time with per-country dates, deadline warning, summary cards
- Test start/end are set in Lisbon time and stored as absolute instants, so each
  student sees them in their own local time; the server decides by the same
  instant and no longer by its own time zone
- Optional dates per country, written in that country's local time; the account
  country picks them (client and server share the same schedule code)
- The countdown uses the server clock; tests that have not opened yet are also
  refused by the API
- Students see a deadline banner (neutral, orange in the last 24 h, red in the
  last hour, then "deadline ended")
- The start screen shows mini-cards: questions, passing score, time limit, attempts
- Translations for the new texts added to the Excel

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E975"/>
+  <dimension ref="A1:E991"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26773,6 +26773,438 @@
         </is>
       </c>
     </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>Lisbon time</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Lisbon time</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>hora de Lisboa</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>hora de Lisboa</t>
+        </is>
+      </c>
+      <c r="E976" t="inlineStr">
+        <is>
+          <t>heure de Lisbonne</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>Students see these dates in their own time zone</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>Students see these dates in their own time zone</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>Os alunos veem estas datas na sua própria hora local</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>Los alumnos ven estas fechas en su propia hora local</t>
+        </is>
+      </c>
+      <c r="E977" t="inlineStr">
+        <is>
+          <t>Les étudiants voient ces dates dans leur propre fuseau horaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>Dates by country</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Dates by country</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Datas por país</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>Fechas por país</t>
+        </is>
+      </c>
+      <c r="E978" t="inlineStr">
+        <is>
+          <t>Dates par pays</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>A country can open and close at a different time, written in that country's local time. What is left empty follows the Lisbon date</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>A country can open and close at a different time, written in that country's local time. What is left empty follows the Lisbon date</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>Um país pode abrir e fechar a outra hora, escrita na hora local desse país. O que ficar vazio segue a data de Lisboa</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>Un país puede abrir y cerrar a otra hora, escrita en la hora local de ese país. Lo que quede vacío sigue la fecha de Lisboa</t>
+        </is>
+      </c>
+      <c r="E979" t="inlineStr">
+        <is>
+          <t>Un pays peut ouvrir et fermer à une autre heure, indiquée à l’heure locale de ce pays. Ce qui reste vide suit la date de Lisbonne</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>Add a country with its own dates</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Add a country with its own dates</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>Adicionar um país com datas próprias</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>Añadir un país con fechas propias</t>
+        </is>
+      </c>
+      <c r="E980" t="inlineStr">
+        <is>
+          <t>Ajouter un pays avec ses propres dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>The deadline for this test has ended</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>The deadline for this test has ended</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>O prazo deste teste terminou</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>El plazo de este test ha terminado</t>
+        </is>
+      </c>
+      <c r="E981" t="inlineStr">
+        <is>
+          <t>Le délai de ce test est terminé</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>The deadline for this test ends in</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>The deadline for this test ends in</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>O prazo deste teste termina em</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>El plazo de este test termina en</t>
+        </is>
+      </c>
+      <c r="E982" t="inlineStr">
+        <is>
+          <t>Le délai de ce test se termine dans</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>Available until</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Available until</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>Disponível até</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>Disponible hasta</t>
+        </is>
+      </c>
+      <c r="E983" t="inlineStr">
+        <is>
+          <t>Disponible jusqu’au</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>Complete it before the deadline to finish the course</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Complete it before the deadline to finish the course</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Faça-o antes do prazo para concluir o curso</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>Hágalo antes del plazo para completar el curso</t>
+        </is>
+      </c>
+      <c r="E984" t="inlineStr">
+        <is>
+          <t>Faites-le avant la date limite pour terminer le cours</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E985" t="inlineStr">
+        <is>
+          <t>j</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E986" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E987" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>Same as Lisbon</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Same as Lisbon</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Igual a Lisboa</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>Igual que Lisboa</t>
+        </is>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>Identique à Lisbonne</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>Local time</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>Local time</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>Hora local</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>Hora local</t>
+        </is>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>Heure locale</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>No limit</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>No limit</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>Sem limite</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>Sin límite</t>
+        </is>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>Sans limite</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(dashboard,notifications): period filter, translated labels, redesigned notifications
- Dashboard: date/time range picker (with presets) that limits activity, charts,
  best students, access logs and registrations on the API side; activity rows for
  course/module/enrol and user status tags are translated
- Notifications page: unread/all filter, mark all as read (new endpoint, own
  notifications only), grouping by day, cards in the platform style; the pop-up
  notice gets the brand bell and opens the page on click
- Translations for the new texts added to the Excel

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E991"/>
+  <dimension ref="A1:E999"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27205,6 +27205,222 @@
         </is>
       </c>
     </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>Enrolled in the course</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Enrolled in the course</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>Inscrito no curso</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>Inscrito en el curso</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>Inscrit au cours</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Módulo</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>Módulo</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Hoje</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>Hoy</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>Aujourd’hui</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>Yesterday</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>Yesterday</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Ontem</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>Ayer</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>Hier</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>This month</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>This month</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>Este mês</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>Este mes</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>Ce mois-ci</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>Showing activity, accesses and registrations in this period</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Showing activity, accesses and registrations in this period</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>A mostrar a atividade, os acessos e os registos deste período</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>Mostrando la actividad, los accesos y los registros de este período</t>
+        </is>
+      </c>
+      <c r="E997" t="inlineStr">
+        <is>
+          <t>Affichage de l’activité, des accès et des inscriptions de cette période</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>Mark all as read</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Mark all as read</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Marcar todas como lidas</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>Marcar todas como leídas</t>
+        </is>
+      </c>
+      <c r="E998" t="inlineStr">
+        <is>
+          <t>Tout marquer comme lu</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>You have no unread notifications</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>You have no unread notifications</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Não tem notificações por ler</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>No tiene notificaciones sin leer</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr">
+        <is>
+          <t>Vous n’avez aucune notification non lue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(email): Brevo API as an e-mail provider; fix(auth): check code expiry on the database clock
- Settings > E-mail integration: choose SMTP or Brevo API (nodemailer transport over the Brevo REST API, so logging, templates and communications work unchanged)
- Login and recovery codes: compare the expiry with NOW() in SQL instead of the Node clock, which broke when their time zones differ
- Translations for the new texts in the Excel

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1000"/>
+  <dimension ref="A1:E1012"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -17399,9 +17399,213 @@
         <v>Publication</v>
       </c>
     </row>
+    <row r="1001">
+      <c r="A1001" t="str">
+        <v>E-mail integration</v>
+      </c>
+      <c r="B1001" t="str">
+        <v>E-mail integration</v>
+      </c>
+      <c r="C1001" t="str">
+        <v>Integração de e-mail</v>
+      </c>
+      <c r="D1001" t="str">
+        <v>Integración de correo electrónico</v>
+      </c>
+      <c r="E1001" t="str">
+        <v>Intégration e-mail</v>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="str">
+        <v>How the platform sends e-mails: through an SMTP server or through the Brevo API</v>
+      </c>
+      <c r="B1002" t="str">
+        <v>How the platform sends e-mails: through an SMTP server or through the Brevo API</v>
+      </c>
+      <c r="C1002" t="str">
+        <v>Como a plataforma envia e-mails: por um servidor SMTP ou pela API da Brevo</v>
+      </c>
+      <c r="D1002" t="str">
+        <v>Cómo envía correos la plataforma: mediante un servidor SMTP o mediante la API de Brevo</v>
+      </c>
+      <c r="E1002" t="str">
+        <v>Comment la plateforme envoie les e-mails : via un serveur SMTP ou via l’API Brevo</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="str">
+        <v>Provider</v>
+      </c>
+      <c r="B1003" t="str">
+        <v>Provider</v>
+      </c>
+      <c r="C1003" t="str">
+        <v>Fornecedor</v>
+      </c>
+      <c r="D1003" t="str">
+        <v>Proveedor</v>
+      </c>
+      <c r="E1003" t="str">
+        <v>Fournisseur</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="str">
+        <v>Choose how the e-mails are sent</v>
+      </c>
+      <c r="B1004" t="str">
+        <v>Choose how the e-mails are sent</v>
+      </c>
+      <c r="C1004" t="str">
+        <v>Escolha como os e-mails são enviados</v>
+      </c>
+      <c r="D1004" t="str">
+        <v>Elija cómo se envían los correos</v>
+      </c>
+      <c r="E1004" t="str">
+        <v>Choisissez comment les e-mails sont envoyés</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="str">
+        <v>Brevo API</v>
+      </c>
+      <c r="B1005" t="str">
+        <v>Brevo API</v>
+      </c>
+      <c r="C1005" t="str">
+        <v>API da Brevo</v>
+      </c>
+      <c r="D1005" t="str">
+        <v>API de Brevo</v>
+      </c>
+      <c r="E1005" t="str">
+        <v>API Brevo</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="str">
+        <v>The API key of your Brevo account. Create it in Brevo under SMTP &amp; API &gt; API Keys</v>
+      </c>
+      <c r="B1006" t="str">
+        <v>The API key of your Brevo account. Create it in Brevo under SMTP &amp; API &gt; API Keys</v>
+      </c>
+      <c r="C1006" t="str">
+        <v>A chave de API da sua conta Brevo. Crie-a na Brevo em SMTP e API &gt; Chaves de API</v>
+      </c>
+      <c r="D1006" t="str">
+        <v>La clave de API de su cuenta de Brevo. Créela en Brevo en SMTP y API &gt; Claves de API</v>
+      </c>
+      <c r="E1006" t="str">
+        <v>La clé API de votre compte Brevo. Créez-la dans Brevo sous SMTP et API &gt; Clés API</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="str">
+        <v>API key</v>
+      </c>
+      <c r="B1007" t="str">
+        <v>API key</v>
+      </c>
+      <c r="C1007" t="str">
+        <v>Chave de API</v>
+      </c>
+      <c r="D1007" t="str">
+        <v>Clave de API</v>
+      </c>
+      <c r="E1007" t="str">
+        <v>Clé API</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="str">
+        <v>Kept on the server and only visible to people who can edit the settings</v>
+      </c>
+      <c r="B1008" t="str">
+        <v>Kept on the server and only visible to people who can edit the settings</v>
+      </c>
+      <c r="C1008" t="str">
+        <v>Fica guardada no servidor e só é visível para quem pode editar as definições</v>
+      </c>
+      <c r="D1008" t="str">
+        <v>Se guarda en el servidor y solo la ven quienes pueden editar la configuración</v>
+      </c>
+      <c r="E1008" t="str">
+        <v>Conservée sur le serveur et visible uniquement par les personnes pouvant modifier les paramètres</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="str">
+        <v>The address and the name the recipients see. The address must be a verified sender in Brevo</v>
+      </c>
+      <c r="B1009" t="str">
+        <v>The address and the name the recipients see. The address must be a verified sender in Brevo</v>
+      </c>
+      <c r="C1009" t="str">
+        <v>O endereço e o nome que os destinatários veem. O endereço tem de ser um remetente verificado na Brevo</v>
+      </c>
+      <c r="D1009" t="str">
+        <v>La dirección y el nombre que ven los destinatarios. La dirección debe ser un remitente verificado en Brevo</v>
+      </c>
+      <c r="E1009" t="str">
+        <v>L’adresse et le nom que voient les destinataires. L’adresse doit être un expéditeur vérifié dans Brevo</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="str">
+        <v>Must be a sender or domain verified in your Brevo account</v>
+      </c>
+      <c r="B1010" t="str">
+        <v>Must be a sender or domain verified in your Brevo account</v>
+      </c>
+      <c r="C1010" t="str">
+        <v>Tem de ser um remetente ou domínio verificado na sua conta Brevo</v>
+      </c>
+      <c r="D1010" t="str">
+        <v>Debe ser un remitente o dominio verificado en su cuenta de Brevo</v>
+      </c>
+      <c r="E1010" t="str">
+        <v>Doit être un expéditeur ou un domaine vérifié dans votre compte Brevo</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="str">
+        <v>Everything the platform sends goes through the Brevo API</v>
+      </c>
+      <c r="B1011" t="str">
+        <v>Everything the platform sends goes through the Brevo API</v>
+      </c>
+      <c r="C1011" t="str">
+        <v>Tudo o que a plataforma envia passa pela API da Brevo</v>
+      </c>
+      <c r="D1011" t="str">
+        <v>Todo lo que envía la plataforma pasa por la API de Brevo</v>
+      </c>
+      <c r="E1011" t="str">
+        <v>Tout ce que la plateforme envoie passe par l’API Brevo</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="str">
+        <v>Sending through the API does not depend on the hosting mail server or its hourly limits. Brevo's own plan limits apply</v>
+      </c>
+      <c r="B1012" t="str">
+        <v>Sending through the API does not depend on the hosting mail server or its hourly limits. Brevo's own plan limits apply</v>
+      </c>
+      <c r="C1012" t="str">
+        <v>O envio pela API não depende do servidor de e-mail do alojamento nem dos seus limites por hora. Aplicam-se os limites do plano da Brevo</v>
+      </c>
+      <c r="D1012" t="str">
+        <v>El envío mediante la API no depende del servidor de correo del alojamiento ni de sus límites por hora. Se aplican los límites del plan de Brevo</v>
+      </c>
+      <c r="E1012" t="str">
+        <v>L’envoi par l’API ne dépend pas du serveur de messagerie de l’hébergement ni de ses limites horaires. Les limites du forfait Brevo s’appliquent</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1000"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1012"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: deploy notes for the new migrations and the PDF viewer; translations for the new texts
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/translations/admin-redesign-translations.xlsx
+++ b/docs/translations/admin-redesign-translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1012"/>
+  <dimension ref="A1:E1043"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -17603,9 +17603,536 @@
         <v>L’envoi par l’API ne dépend pas du serveur de messagerie de l’hébergement ni de ses limites horaires. Les limites du forfait Brevo s’appliquent</v>
       </c>
     </row>
+    <row r="1013">
+      <c r="A1013" t="str">
+        <v>25 / 50 / 25</v>
+      </c>
+      <c r="B1013" t="str">
+        <v>25 / 50 / 25</v>
+      </c>
+      <c r="C1013" t="str">
+        <v>25 / 50 / 25</v>
+      </c>
+      <c r="D1013" t="str">
+        <v>25 / 50 / 25</v>
+      </c>
+      <c r="E1013" t="str">
+        <v>25 / 50 / 25</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="str">
+        <v>4 columns</v>
+      </c>
+      <c r="B1014" t="str">
+        <v>4 columns</v>
+      </c>
+      <c r="C1014" t="str">
+        <v>4 colunas</v>
+      </c>
+      <c r="D1014" t="str">
+        <v>4 columnas</v>
+      </c>
+      <c r="E1014" t="str">
+        <v>4 colonnes</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="str">
+        <v>Alignment</v>
+      </c>
+      <c r="B1015" t="str">
+        <v>Alignment</v>
+      </c>
+      <c r="C1015" t="str">
+        <v>Alinhamento</v>
+      </c>
+      <c r="D1015" t="str">
+        <v>Alineación</v>
+      </c>
+      <c r="E1015" t="str">
+        <v>Alignement</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="str">
+        <v>Background</v>
+      </c>
+      <c r="B1016" t="str">
+        <v>Background</v>
+      </c>
+      <c r="C1016" t="str">
+        <v>Fundo</v>
+      </c>
+      <c r="D1016" t="str">
+        <v>Fondo</v>
+      </c>
+      <c r="E1016" t="str">
+        <v>Arrière-plan</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="str">
+        <v>Bottom</v>
+      </c>
+      <c r="B1017" t="str">
+        <v>Bottom</v>
+      </c>
+      <c r="C1017" t="str">
+        <v>Baixo</v>
+      </c>
+      <c r="D1017" t="str">
+        <v>Abajo</v>
+      </c>
+      <c r="E1017" t="str">
+        <v>Bas</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="str">
+        <v>Top</v>
+      </c>
+      <c r="B1018" t="str">
+        <v>Top</v>
+      </c>
+      <c r="C1018" t="str">
+        <v>Cima</v>
+      </c>
+      <c r="D1018" t="str">
+        <v>Arriba</v>
+      </c>
+      <c r="E1018" t="str">
+        <v>Haut</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="str">
+        <v>Column layout</v>
+      </c>
+      <c r="B1019" t="str">
+        <v>Column layout</v>
+      </c>
+      <c r="C1019" t="str">
+        <v>Disposição das colunas</v>
+      </c>
+      <c r="D1019" t="str">
+        <v>Disposición de las columnas</v>
+      </c>
+      <c r="E1019" t="str">
+        <v>Disposition des colonnes</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="str">
+        <v>Column width</v>
+      </c>
+      <c r="B1020" t="str">
+        <v>Column width</v>
+      </c>
+      <c r="C1020" t="str">
+        <v>Largura da coluna</v>
+      </c>
+      <c r="D1020" t="str">
+        <v>Ancho de la columna</v>
+      </c>
+      <c r="E1020" t="str">
+        <v>Largeur de la colonne</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="str">
+        <v>Column width (%)</v>
+      </c>
+      <c r="B1021" t="str">
+        <v>Column width (%)</v>
+      </c>
+      <c r="C1021" t="str">
+        <v>Largura da coluna (%)</v>
+      </c>
+      <c r="D1021" t="str">
+        <v>Ancho de la columna (%)</v>
+      </c>
+      <c r="E1021" t="str">
+        <v>Largeur de la colonne (%)</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="str">
+        <v>Font size (px)</v>
+      </c>
+      <c r="B1022" t="str">
+        <v>Font size (px)</v>
+      </c>
+      <c r="C1022" t="str">
+        <v>Tamanho da letra (px)</v>
+      </c>
+      <c r="D1022" t="str">
+        <v>Tamaño de letra (px)</v>
+      </c>
+      <c r="E1022" t="str">
+        <v>Taille de police (px)</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="str">
+        <v>Full width</v>
+      </c>
+      <c r="B1023" t="str">
+        <v>Full width</v>
+      </c>
+      <c r="C1023" t="str">
+        <v>Largura total</v>
+      </c>
+      <c r="D1023" t="str">
+        <v>Ancho completo</v>
+      </c>
+      <c r="E1023" t="str">
+        <v>Pleine largeur</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="str">
+        <v>Has styles for this device</v>
+      </c>
+      <c r="B1024" t="str">
+        <v>Has styles for this device</v>
+      </c>
+      <c r="C1024" t="str">
+        <v>Tem estilos para este dispositivo</v>
+      </c>
+      <c r="D1024" t="str">
+        <v>Tiene estilos para este dispositivo</v>
+      </c>
+      <c r="E1024" t="str">
+        <v>A des styles pour cet appareil</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="str">
+        <v>Height (px)</v>
+      </c>
+      <c r="B1025" t="str">
+        <v>Height (px)</v>
+      </c>
+      <c r="C1025" t="str">
+        <v>Altura (px)</v>
+      </c>
+      <c r="D1025" t="str">
+        <v>Altura (px)</v>
+      </c>
+      <c r="E1025" t="str">
+        <v>Hauteur (px)</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="str">
+        <v>Hide on this device</v>
+      </c>
+      <c r="B1026" t="str">
+        <v>Hide on this device</v>
+      </c>
+      <c r="C1026" t="str">
+        <v>Esconder neste dispositivo</v>
+      </c>
+      <c r="D1026" t="str">
+        <v>Ocultar en este dispositivo</v>
+      </c>
+      <c r="E1026" t="str">
+        <v>Masquer sur cet appareil</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="str">
+        <v>Letter spacing (px)</v>
+      </c>
+      <c r="B1027" t="str">
+        <v>Letter spacing (px)</v>
+      </c>
+      <c r="C1027" t="str">
+        <v>Espaçamento entre letras (px)</v>
+      </c>
+      <c r="D1027" t="str">
+        <v>Espaciado entre letras (px)</v>
+      </c>
+      <c r="E1027" t="str">
+        <v>Espacement des lettres (px)</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="str">
+        <v>Line height</v>
+      </c>
+      <c r="B1028" t="str">
+        <v>Line height</v>
+      </c>
+      <c r="C1028" t="str">
+        <v>Altura da linha</v>
+      </c>
+      <c r="D1028" t="str">
+        <v>Altura de línea</v>
+      </c>
+      <c r="E1028" t="str">
+        <v>Hauteur de ligne</v>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="str">
+        <v>Padding (px)</v>
+      </c>
+      <c r="B1029" t="str">
+        <v>Padding (px)</v>
+      </c>
+      <c r="C1029" t="str">
+        <v>Espaçamento interno (px)</v>
+      </c>
+      <c r="D1029" t="str">
+        <v>Relleno interno (px)</v>
+      </c>
+      <c r="E1029" t="str">
+        <v>Marge intérieure (px)</v>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="str">
+        <v>Per device</v>
+      </c>
+      <c r="B1030" t="str">
+        <v>Per device</v>
+      </c>
+      <c r="C1030" t="str">
+        <v>Por dispositivo</v>
+      </c>
+      <c r="D1030" t="str">
+        <v>Por dispositivo</v>
+      </c>
+      <c r="E1030" t="str">
+        <v>Par appareil</v>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="str">
+        <v>Tablet</v>
+      </c>
+      <c r="B1031" t="str">
+        <v>Tablet</v>
+      </c>
+      <c r="C1031" t="str">
+        <v>Tablet</v>
+      </c>
+      <c r="D1031" t="str">
+        <v>Tableta</v>
+      </c>
+      <c r="E1031" t="str">
+        <v>Tablette</v>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="str">
+        <v>Text color</v>
+      </c>
+      <c r="B1032" t="str">
+        <v>Text color</v>
+      </c>
+      <c r="C1032" t="str">
+        <v>Cor do texto</v>
+      </c>
+      <c r="D1032" t="str">
+        <v>Color del texto</v>
+      </c>
+      <c r="E1032" t="str">
+        <v>Couleur du texte</v>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="str">
+        <v>up to 479px</v>
+      </c>
+      <c r="B1033" t="str">
+        <v>up to 479px</v>
+      </c>
+      <c r="C1033" t="str">
+        <v>até 479px</v>
+      </c>
+      <c r="D1033" t="str">
+        <v>hasta 479px</v>
+      </c>
+      <c r="E1033" t="str">
+        <v>jusqu’à 479px</v>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="str">
+        <v>wider than 820px</v>
+      </c>
+      <c r="B1034" t="str">
+        <v>wider than 820px</v>
+      </c>
+      <c r="C1034" t="str">
+        <v>acima de 820px</v>
+      </c>
+      <c r="D1034" t="str">
+        <v>más de 820px</v>
+      </c>
+      <c r="E1034" t="str">
+        <v>plus de 820px</v>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="str">
+        <v>Wide + narrow</v>
+      </c>
+      <c r="B1035" t="str">
+        <v>Wide + narrow</v>
+      </c>
+      <c r="C1035" t="str">
+        <v>Larga + estreita</v>
+      </c>
+      <c r="D1035" t="str">
+        <v>Ancha + estrecha</v>
+      </c>
+      <c r="E1035" t="str">
+        <v>Large + étroite</v>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="str">
+        <v>Download certificate</v>
+      </c>
+      <c r="B1036" t="str">
+        <v>Download certificate</v>
+      </c>
+      <c r="C1036" t="str">
+        <v>Descarregar certificado</v>
+      </c>
+      <c r="D1036" t="str">
+        <v>Descargar certificado</v>
+      </c>
+      <c r="E1036" t="str">
+        <v>Télécharger le certificat</v>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="str">
+        <v>Loading the document</v>
+      </c>
+      <c r="B1037" t="str">
+        <v>Loading the document</v>
+      </c>
+      <c r="C1037" t="str">
+        <v>A carregar o documento</v>
+      </c>
+      <c r="D1037" t="str">
+        <v>Cargando el documento</v>
+      </c>
+      <c r="E1037" t="str">
+        <v>Chargement du document</v>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="str">
+        <v>The document could not be loaded</v>
+      </c>
+      <c r="B1038" t="str">
+        <v>The document could not be loaded</v>
+      </c>
+      <c r="C1038" t="str">
+        <v>Não foi possível carregar o documento</v>
+      </c>
+      <c r="D1038" t="str">
+        <v>No se pudo cargar el documento</v>
+      </c>
+      <c r="E1038" t="str">
+        <v>Le document n’a pas pu être chargé</v>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="str">
+        <v>Check your connection and try again. Large documents can take a while to download.</v>
+      </c>
+      <c r="B1039" t="str">
+        <v>Check your connection and try again. Large documents can take a while to download.</v>
+      </c>
+      <c r="C1039" t="str">
+        <v>Verifique a ligação e tente novamente. Os documentos grandes podem demorar a descarregar.</v>
+      </c>
+      <c r="D1039" t="str">
+        <v>Compruebe la conexión e inténtelo de nuevo. Los documentos grandes pueden tardar en descargarse.</v>
+      </c>
+      <c r="E1039" t="str">
+        <v>Vérifiez votre connexion et réessayez. Les documents volumineux peuvent prendre un certain temps à se télécharger.</v>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="str">
+        <v>Minimum approval percentage</v>
+      </c>
+      <c r="B1040" t="str">
+        <v>Minimum approval percentage</v>
+      </c>
+      <c r="C1040" t="str">
+        <v>Percentagem mínima de aprovação</v>
+      </c>
+      <c r="D1040" t="str">
+        <v>Porcentaje mínimo de aprobación</v>
+      </c>
+      <c r="E1040" t="str">
+        <v>Pourcentage minimum de réussite</v>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="str">
+        <v>Correct answers</v>
+      </c>
+      <c r="B1041" t="str">
+        <v>Correct answers</v>
+      </c>
+      <c r="C1041" t="str">
+        <v>Respostas certas</v>
+      </c>
+      <c r="D1041" t="str">
+        <v>Respuestas correctas</v>
+      </c>
+      <c r="E1041" t="str">
+        <v>Bonnes réponses</v>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="str">
+        <v>You did not reach the minimum approval percentage. Review the content and try again.</v>
+      </c>
+      <c r="B1042" t="str">
+        <v>You did not reach the minimum approval percentage. Review the content and try again.</v>
+      </c>
+      <c r="C1042" t="str">
+        <v>Não atingiu a percentagem mínima de aprovação. Reveja os conteúdos e tente novamente.</v>
+      </c>
+      <c r="D1042" t="str">
+        <v>No alcanzó el porcentaje mínimo de aprobación. Repase los contenidos e inténtelo de nuevo.</v>
+      </c>
+      <c r="E1042" t="str">
+        <v>Vous n’avez pas atteint le pourcentage minimum de réussite. Revoyez le contenu et réessayez.</v>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="str">
+        <v>You can review the questions after you pass or use all your attempts</v>
+      </c>
+      <c r="B1043" t="str">
+        <v>You can review the questions after you pass or use all your attempts</v>
+      </c>
+      <c r="C1043" t="str">
+        <v>Pode rever as perguntas depois de ser aprovado ou de esgotar todas as tentativas</v>
+      </c>
+      <c r="D1043" t="str">
+        <v>Podrá repasar las preguntas cuando apruebe o agote todos los intentos</v>
+      </c>
+      <c r="E1043" t="str">
+        <v>Vous pourrez revoir les questions après avoir réussi ou épuisé toutes vos tentatives</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1012"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1043"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>